<commit_message>
Update course plans and related documents for IHV and ISLL
- Updated the number of rows in the Excel download links for "Vilande kursplaner" in IHV and ISLL.
- Added new course plans AVÅ27L and AVÅ28H to the IHV section.
- Adjusted course counts in the "Omvårdnad" and "Svenska" sections to reflect the latest changes.
- Updated tags and scrape hashes for various course plans across IHV and ISLL.
- Modified the course plan for GSV3KH to remove the "vilande" tag and updated its associated metadata.
- Updated multiple Excel files across IKS and ISLL for consistency and accuracy.
</commit_message>
<xml_diff>
--- a/vault-dalarna-university/02 IHV/Analys/Vilande kursplaner.xlsx
+++ b/vault-dalarna-university/02 IHV/Analys/Vilande kursplaner.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Vilande kursplaner" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Vilande kursplaner'!$A$1:$I$237</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Vilande kursplaner'!$A$1:$I$239</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I237"/>
+  <dimension ref="A1:I239"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7632,12 +7632,12 @@
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
         <is>
-          <t>GIH2UR</t>
+          <t>AVÅ27L</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>IDA</t>
+          <t>OMV</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
@@ -7647,18 +7647,18 @@
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>2022-02-24</t>
+          <t>2021-12-08</t>
         </is>
       </c>
       <c r="E162" t="inlineStr"/>
       <c r="F162" t="inlineStr">
         <is>
-          <t>Idrotts- och hälsovetenskap</t>
+          <t>Omvårdnad</t>
         </is>
       </c>
       <c r="G162" t="inlineStr">
         <is>
-          <t>Grundläggande vetenskaplig metod</t>
+          <t>Vård och omsorg för personer med demens (fristående kurs)</t>
         </is>
       </c>
       <c r="H162" t="inlineStr">
@@ -7668,19 +7668,19 @@
       </c>
       <c r="I162" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2UR</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AVÅ27L</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
         <is>
-          <t>AVÅ27S</t>
+          <t>GIH2UR</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>OMV</t>
+          <t>IDA</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
@@ -7696,12 +7696,12 @@
       <c r="E163" t="inlineStr"/>
       <c r="F163" t="inlineStr">
         <is>
-          <t>Omvårdnad</t>
+          <t>Idrotts- och hälsovetenskap</t>
         </is>
       </c>
       <c r="G163" t="inlineStr">
         <is>
-          <t>Bedömning och rådgivning vid distanskontakter inom hälso- och sjukvården</t>
+          <t>Grundläggande vetenskaplig metod</t>
         </is>
       </c>
       <c r="H163" t="inlineStr">
@@ -7711,19 +7711,19 @@
       </c>
       <c r="I163" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AVÅ27S</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2UR</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
         <is>
-          <t>GIH2UY</t>
+          <t>AVÅ27S</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>IDA</t>
+          <t>OMV</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
@@ -7733,18 +7733,18 @@
       </c>
       <c r="D164" t="inlineStr">
         <is>
-          <t>2022-02-28</t>
+          <t>2022-02-24</t>
         </is>
       </c>
       <c r="E164" t="inlineStr"/>
       <c r="F164" t="inlineStr">
         <is>
-          <t>Idrotts- och hälsovetenskap</t>
+          <t>Omvårdnad</t>
         </is>
       </c>
       <c r="G164" t="inlineStr">
         <is>
-          <t>Näringslära med inriktning mot idrott och fysisk aktivitet</t>
+          <t>Bedömning och rådgivning vid distanskontakter inom hälso- och sjukvården</t>
         </is>
       </c>
       <c r="H164" t="inlineStr">
@@ -7754,14 +7754,14 @@
       </c>
       <c r="I164" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2UY</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AVÅ27S</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
         <is>
-          <t>GIH2VJ</t>
+          <t>GIH2UY</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
@@ -7776,7 +7776,7 @@
       </c>
       <c r="D165" t="inlineStr">
         <is>
-          <t>2022-03-03</t>
+          <t>2022-02-28</t>
         </is>
       </c>
       <c r="E165" t="inlineStr"/>
@@ -7787,7 +7787,7 @@
       </c>
       <c r="G165" t="inlineStr">
         <is>
-          <t>Idrottsmedicin</t>
+          <t>Näringslära med inriktning mot idrott och fysisk aktivitet</t>
         </is>
       </c>
       <c r="H165" t="inlineStr">
@@ -7797,14 +7797,14 @@
       </c>
       <c r="I165" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2VJ</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2UY</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" s="2" t="inlineStr">
         <is>
-          <t>GIH2VK</t>
+          <t>GIH2VJ</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
@@ -7830,7 +7830,7 @@
       </c>
       <c r="G166" t="inlineStr">
         <is>
-          <t>Grundläggande upplevelseproduktion</t>
+          <t>Idrottsmedicin</t>
         </is>
       </c>
       <c r="H166" t="inlineStr">
@@ -7840,19 +7840,19 @@
       </c>
       <c r="I166" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2VK</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2VJ</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" s="2" t="inlineStr">
         <is>
-          <t>GVÅ2VZ</t>
+          <t>GIH2VK</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>OMV</t>
+          <t>IDA</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
@@ -7862,18 +7862,18 @@
       </c>
       <c r="D167" t="inlineStr">
         <is>
-          <t>2022-04-13</t>
+          <t>2022-03-03</t>
         </is>
       </c>
       <c r="E167" t="inlineStr"/>
       <c r="F167" t="inlineStr">
         <is>
-          <t>Omvårdnad</t>
+          <t>Idrotts- och hälsovetenskap</t>
         </is>
       </c>
       <c r="G167" t="inlineStr">
         <is>
-          <t>Palliativ och evidensbaserad omvårdnad för personer med demens</t>
+          <t>Grundläggande upplevelseproduktion</t>
         </is>
       </c>
       <c r="H167" t="inlineStr">
@@ -7883,19 +7883,19 @@
       </c>
       <c r="I167" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GVÅ2VZ</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2VK</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" s="2" t="inlineStr">
         <is>
-          <t>GIH2WT</t>
+          <t>GVÅ2VZ</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>IDA</t>
+          <t>OMV</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
@@ -7905,18 +7905,18 @@
       </c>
       <c r="D168" t="inlineStr">
         <is>
-          <t>2022-06-16</t>
+          <t>2022-04-13</t>
         </is>
       </c>
       <c r="E168" t="inlineStr"/>
       <c r="F168" t="inlineStr">
         <is>
-          <t>Idrotts- och hälsovetenskap</t>
+          <t>Omvårdnad</t>
         </is>
       </c>
       <c r="G168" t="inlineStr">
         <is>
-          <t>Fotbollstränare - inriktning barn och ungdom (6-15 år)</t>
+          <t>Palliativ och evidensbaserad omvårdnad för personer med demens</t>
         </is>
       </c>
       <c r="H168" t="inlineStr">
@@ -7926,14 +7926,14 @@
       </c>
       <c r="I168" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2WT</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GVÅ2VZ</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" s="2" t="inlineStr">
         <is>
-          <t>GIH2WX</t>
+          <t>GIH2WT</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
@@ -7959,7 +7959,7 @@
       </c>
       <c r="G169" t="inlineStr">
         <is>
-          <t>Idrotten i samhället (VAL)</t>
+          <t>Fotbollstränare - inriktning barn och ungdom (6-15 år)</t>
         </is>
       </c>
       <c r="H169" t="inlineStr">
@@ -7969,14 +7969,14 @@
       </c>
       <c r="I169" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2WX</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2WT</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" s="2" t="inlineStr">
         <is>
-          <t>GIH2WY</t>
+          <t>GIH2WX</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
@@ -8002,7 +8002,7 @@
       </c>
       <c r="G170" t="inlineStr">
         <is>
-          <t>Friluftsliv i närmiljön: orientering, vandring, paddling (VAL)</t>
+          <t>Idrotten i samhället (VAL)</t>
         </is>
       </c>
       <c r="H170" t="inlineStr">
@@ -8012,19 +8012,19 @@
       </c>
       <c r="I170" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2WY</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2WX</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" s="2" t="inlineStr">
         <is>
-          <t>ASR284</t>
+          <t>GIH2WY</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>SRP</t>
+          <t>IDA</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
@@ -8040,12 +8040,12 @@
       <c r="E171" t="inlineStr"/>
       <c r="F171" t="inlineStr">
         <is>
-          <t>Sexuell, reproduktiv och perinatal hälsa</t>
+          <t>Idrotts- och hälsovetenskap</t>
         </is>
       </c>
       <c r="G171" t="inlineStr">
         <is>
-          <t>Förlossningsvård I, verksamhetsförlagd utbildning</t>
+          <t>Friluftsliv i närmiljön: orientering, vandring, paddling (VAL)</t>
         </is>
       </c>
       <c r="H171" t="inlineStr">
@@ -8055,14 +8055,14 @@
       </c>
       <c r="I171" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR284</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2WY</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" s="2" t="inlineStr">
         <is>
-          <t>ASR285</t>
+          <t>ASR284</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
@@ -8088,7 +8088,7 @@
       </c>
       <c r="G172" t="inlineStr">
         <is>
-          <t>Gynekologisk vård och postpartumvård, verksamhetsförlagd utbildning</t>
+          <t>Förlossningsvård I, verksamhetsförlagd utbildning</t>
         </is>
       </c>
       <c r="H172" t="inlineStr">
@@ -8098,14 +8098,14 @@
       </c>
       <c r="I172" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR285</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR284</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" s="2" t="inlineStr">
         <is>
-          <t>ASR286</t>
+          <t>ASR285</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
@@ -8131,7 +8131,7 @@
       </c>
       <c r="G173" t="inlineStr">
         <is>
-          <t>Examensarbete i sexuell, reproduktiv och perinatal hälsa</t>
+          <t>Gynekologisk vård och postpartumvård, verksamhetsförlagd utbildning</t>
         </is>
       </c>
       <c r="H173" t="inlineStr">
@@ -8141,19 +8141,19 @@
       </c>
       <c r="I173" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR286</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR285</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" s="2" t="inlineStr">
         <is>
-          <t>GIH2X3</t>
+          <t>ASR286</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>IDA</t>
+          <t>SRP</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
@@ -8166,19 +8166,15 @@
           <t>2022-06-16</t>
         </is>
       </c>
-      <c r="E174" t="inlineStr">
-        <is>
-          <t>2022-08-22</t>
-        </is>
-      </c>
+      <c r="E174" t="inlineStr"/>
       <c r="F174" t="inlineStr">
         <is>
-          <t>Idrotts- och hälsovetenskap</t>
+          <t>Sexuell, reproduktiv och perinatal hälsa</t>
         </is>
       </c>
       <c r="G174" t="inlineStr">
         <is>
-          <t>Träningslära för tävlingsinriktad idrott</t>
+          <t>Examensarbete i sexuell, reproduktiv och perinatal hälsa</t>
         </is>
       </c>
       <c r="H174" t="inlineStr">
@@ -8188,19 +8184,19 @@
       </c>
       <c r="I174" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2X3</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR286</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" s="2" t="inlineStr">
         <is>
-          <t>AMC288</t>
+          <t>GIH2X3</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>MCA</t>
+          <t>IDA</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
@@ -8210,18 +8206,22 @@
       </c>
       <c r="D175" t="inlineStr">
         <is>
-          <t>2022-09-08</t>
-        </is>
-      </c>
-      <c r="E175" t="inlineStr"/>
+          <t>2022-06-16</t>
+        </is>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>2022-08-22</t>
+        </is>
+      </c>
       <c r="F175" t="inlineStr">
         <is>
-          <t>Medicinsk vetenskap</t>
+          <t>Idrotts- och hälsovetenskap</t>
         </is>
       </c>
       <c r="G175" t="inlineStr">
         <is>
-          <t>Fysisk aktivitet och träning som prevention och behandling</t>
+          <t>Träningslära för tävlingsinriktad idrott</t>
         </is>
       </c>
       <c r="H175" t="inlineStr">
@@ -8231,19 +8231,19 @@
       </c>
       <c r="I175" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMC288</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2X3</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" s="2" t="inlineStr">
         <is>
-          <t>GSA2XN</t>
+          <t>AMC288</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>SAA</t>
+          <t>MCA</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
@@ -8259,12 +8259,12 @@
       <c r="E176" t="inlineStr"/>
       <c r="F176" t="inlineStr">
         <is>
-          <t>Socialt arbete</t>
+          <t>Medicinsk vetenskap</t>
         </is>
       </c>
       <c r="G176" t="inlineStr">
         <is>
-          <t>Missbruk och beroende</t>
+          <t>Fysisk aktivitet och träning som prevention och behandling</t>
         </is>
       </c>
       <c r="H176" t="inlineStr">
@@ -8274,19 +8274,19 @@
       </c>
       <c r="I176" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA2XN</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMC288</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" s="2" t="inlineStr">
         <is>
-          <t>GIH2XY</t>
+          <t>GSA2XN</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>IDA</t>
+          <t>SAA</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
@@ -8296,22 +8296,18 @@
       </c>
       <c r="D177" t="inlineStr">
         <is>
-          <t>2022-09-26</t>
-        </is>
-      </c>
-      <c r="E177" t="inlineStr">
-        <is>
-          <t>2022-09-30</t>
-        </is>
-      </c>
+          <t>2022-09-08</t>
+        </is>
+      </c>
+      <c r="E177" t="inlineStr"/>
       <c r="F177" t="inlineStr">
         <is>
-          <t>Idrotts- och hälsovetenskap</t>
+          <t>Socialt arbete</t>
         </is>
       </c>
       <c r="G177" t="inlineStr">
         <is>
-          <t>Idrottsvetenskaplig uppsats</t>
+          <t>Missbruk och beroende</t>
         </is>
       </c>
       <c r="H177" t="inlineStr">
@@ -8321,19 +8317,19 @@
       </c>
       <c r="I177" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2XY</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA2XN</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" s="2" t="inlineStr">
         <is>
-          <t>AVÅ28C</t>
+          <t>GIH2XY</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>OMV</t>
+          <t>IDA</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
@@ -8343,18 +8339,22 @@
       </c>
       <c r="D178" t="inlineStr">
         <is>
-          <t>2022-11-14</t>
-        </is>
-      </c>
-      <c r="E178" t="inlineStr"/>
+          <t>2022-09-26</t>
+        </is>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>2022-09-30</t>
+        </is>
+      </c>
       <c r="F178" t="inlineStr">
         <is>
-          <t>Omvårdnad</t>
+          <t>Idrotts- och hälsovetenskap</t>
         </is>
       </c>
       <c r="G178" t="inlineStr">
         <is>
-          <t>Telefonrådgivning vid distanskontakter inom hälso- och sjukvården</t>
+          <t>Idrottsvetenskaplig uppsats</t>
         </is>
       </c>
       <c r="H178" t="inlineStr">
@@ -8364,19 +8364,19 @@
       </c>
       <c r="I178" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AVÅ28C</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2XY</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" s="2" t="inlineStr">
         <is>
-          <t>GIH2ZA</t>
+          <t>AVÅ28C</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>IDA</t>
+          <t>OMV</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
@@ -8386,18 +8386,18 @@
       </c>
       <c r="D179" t="inlineStr">
         <is>
-          <t>2022-12-12</t>
+          <t>2022-11-14</t>
         </is>
       </c>
       <c r="E179" t="inlineStr"/>
       <c r="F179" t="inlineStr">
         <is>
-          <t>Idrotts- och hälsovetenskap</t>
+          <t>Omvårdnad</t>
         </is>
       </c>
       <c r="G179" t="inlineStr">
         <is>
-          <t>Vinterfriluftsliv genom skidor och skridskor (VAL)</t>
+          <t>Telefonrådgivning vid distanskontakter inom hälso- och sjukvården</t>
         </is>
       </c>
       <c r="H179" t="inlineStr">
@@ -8407,19 +8407,19 @@
       </c>
       <c r="I179" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2ZA</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AVÅ28C</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" s="2" t="inlineStr">
         <is>
-          <t>GIH2ZB</t>
+          <t>AVÅ28H</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>IDA</t>
+          <t>OMV</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
@@ -8429,18 +8429,18 @@
       </c>
       <c r="D180" t="inlineStr">
         <is>
-          <t>2022-12-12</t>
+          <t>2022-11-14</t>
         </is>
       </c>
       <c r="E180" t="inlineStr"/>
       <c r="F180" t="inlineStr">
         <is>
-          <t>Idrotts- och hälsovetenskap</t>
+          <t>Omvårdnad</t>
         </is>
       </c>
       <c r="G180" t="inlineStr">
         <is>
-          <t>Hälsopedagogik (VAL)</t>
+          <t>Nutrition och ätande (fristående kurs)</t>
         </is>
       </c>
       <c r="H180" t="inlineStr">
@@ -8450,14 +8450,14 @@
       </c>
       <c r="I180" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2ZB</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AVÅ28H</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" s="2" t="inlineStr">
         <is>
-          <t>GIH2ZC</t>
+          <t>GIH2ZA</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
@@ -8483,7 +8483,7 @@
       </c>
       <c r="G181" t="inlineStr">
         <is>
-          <t>Humanbiologi 1 (VAL)</t>
+          <t>Vinterfriluftsliv genom skidor och skridskor (VAL)</t>
         </is>
       </c>
       <c r="H181" t="inlineStr">
@@ -8493,14 +8493,14 @@
       </c>
       <c r="I181" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2ZC</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2ZA</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" s="2" t="inlineStr">
         <is>
-          <t>GIH2ZD</t>
+          <t>GIH2ZB</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
@@ -8526,7 +8526,7 @@
       </c>
       <c r="G182" t="inlineStr">
         <is>
-          <t>Simning (VAL)</t>
+          <t>Hälsopedagogik (VAL)</t>
         </is>
       </c>
       <c r="H182" t="inlineStr">
@@ -8536,14 +8536,14 @@
       </c>
       <c r="I182" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2ZD</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2ZB</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" s="2" t="inlineStr">
         <is>
-          <t>GIH2ZE</t>
+          <t>GIH2ZC</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
@@ -8569,7 +8569,7 @@
       </c>
       <c r="G183" t="inlineStr">
         <is>
-          <t>Bedömning och betygssättning i idrott och hälsa (VAL)</t>
+          <t>Humanbiologi 1 (VAL)</t>
         </is>
       </c>
       <c r="H183" t="inlineStr">
@@ -8579,19 +8579,19 @@
       </c>
       <c r="I183" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2ZE</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2ZC</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" s="2" t="inlineStr">
         <is>
-          <t>GVÅ2ZG</t>
+          <t>GIH2ZD</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>OMV</t>
+          <t>IDA</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
@@ -8607,12 +8607,12 @@
       <c r="E184" t="inlineStr"/>
       <c r="F184" t="inlineStr">
         <is>
-          <t>Omvårdnad</t>
+          <t>Idrotts- och hälsovetenskap</t>
         </is>
       </c>
       <c r="G184" t="inlineStr">
         <is>
-          <t>Personcentrerad vård med fördjupning inom omvårdnad</t>
+          <t>Simning (VAL)</t>
         </is>
       </c>
       <c r="H184" t="inlineStr">
@@ -8622,19 +8622,19 @@
       </c>
       <c r="I184" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GVÅ2ZG</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2ZD</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" s="2" t="inlineStr">
         <is>
-          <t>GVÅ2ZY</t>
+          <t>GIH2ZE</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>OMV</t>
+          <t>IDA</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
@@ -8650,12 +8650,12 @@
       <c r="E185" t="inlineStr"/>
       <c r="F185" t="inlineStr">
         <is>
-          <t>Omvårdnad</t>
+          <t>Idrotts- och hälsovetenskap</t>
         </is>
       </c>
       <c r="G185" t="inlineStr">
         <is>
-          <t>Metoder för evidensbaserad vård II</t>
+          <t>Bedömning och betygssättning i idrott och hälsa (VAL)</t>
         </is>
       </c>
       <c r="H185" t="inlineStr">
@@ -8665,19 +8665,19 @@
       </c>
       <c r="I185" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GVÅ2ZY</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2ZE</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" s="2" t="inlineStr">
         <is>
-          <t>GIH334</t>
+          <t>GVÅ2ZG</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>IDA</t>
+          <t>OMV</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
@@ -8687,18 +8687,18 @@
       </c>
       <c r="D186" t="inlineStr">
         <is>
-          <t>2023-02-07</t>
+          <t>2022-12-12</t>
         </is>
       </c>
       <c r="E186" t="inlineStr"/>
       <c r="F186" t="inlineStr">
         <is>
-          <t>Idrotts- och hälsovetenskap</t>
+          <t>Omvårdnad</t>
         </is>
       </c>
       <c r="G186" t="inlineStr">
         <is>
-          <t>Sportjournalistik</t>
+          <t>Personcentrerad vård med fördjupning inom omvårdnad</t>
         </is>
       </c>
       <c r="H186" t="inlineStr">
@@ -8708,19 +8708,19 @@
       </c>
       <c r="I186" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH334</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GVÅ2ZG</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" s="2" t="inlineStr">
         <is>
-          <t>GSA32Y</t>
+          <t>GVÅ2ZY</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>SAA</t>
+          <t>OMV</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
@@ -8730,18 +8730,18 @@
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>2023-02-07</t>
+          <t>2022-12-12</t>
         </is>
       </c>
       <c r="E187" t="inlineStr"/>
       <c r="F187" t="inlineStr">
         <is>
-          <t>Socialt arbete</t>
+          <t>Omvårdnad</t>
         </is>
       </c>
       <c r="G187" t="inlineStr">
         <is>
-          <t>Organisation, grupp och samverkan</t>
+          <t>Metoder för evidensbaserad vård II</t>
         </is>
       </c>
       <c r="H187" t="inlineStr">
@@ -8751,14 +8751,14 @@
       </c>
       <c r="I187" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA32Y</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GVÅ2ZY</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" s="2" t="inlineStr">
         <is>
-          <t>GIH33J</t>
+          <t>GIH334</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
@@ -8773,7 +8773,7 @@
       </c>
       <c r="D188" t="inlineStr">
         <is>
-          <t>2023-02-23</t>
+          <t>2023-02-07</t>
         </is>
       </c>
       <c r="E188" t="inlineStr"/>
@@ -8784,7 +8784,7 @@
       </c>
       <c r="G188" t="inlineStr">
         <is>
-          <t>Grundläggande fysiologi och tillämpad idrottsfysiologi (Klättring)</t>
+          <t>Sportjournalistik</t>
         </is>
       </c>
       <c r="H188" t="inlineStr">
@@ -8794,19 +8794,19 @@
       </c>
       <c r="I188" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH33J</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH334</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" s="2" t="inlineStr">
         <is>
-          <t>GIH33K</t>
+          <t>GSA32Y</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>IDA</t>
+          <t>SAA</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
@@ -8816,18 +8816,18 @@
       </c>
       <c r="D189" t="inlineStr">
         <is>
-          <t>2023-02-23</t>
+          <t>2023-02-07</t>
         </is>
       </c>
       <c r="E189" t="inlineStr"/>
       <c r="F189" t="inlineStr">
         <is>
-          <t>Idrotts- och hälsovetenskap</t>
+          <t>Socialt arbete</t>
         </is>
       </c>
       <c r="G189" t="inlineStr">
         <is>
-          <t>Funktionell anatomi (Klättring)</t>
+          <t>Organisation, grupp och samverkan</t>
         </is>
       </c>
       <c r="H189" t="inlineStr">
@@ -8837,14 +8837,14 @@
       </c>
       <c r="I189" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH33K</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA32Y</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" s="2" t="inlineStr">
         <is>
-          <t>GIH33P</t>
+          <t>GIH33J</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
@@ -8870,7 +8870,7 @@
       </c>
       <c r="G190" t="inlineStr">
         <is>
-          <t>Biomekanik (Klättring)</t>
+          <t>Grundläggande fysiologi och tillämpad idrottsfysiologi (Klättring)</t>
         </is>
       </c>
       <c r="H190" t="inlineStr">
@@ -8880,14 +8880,14 @@
       </c>
       <c r="I190" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH33P</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH33J</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" s="2" t="inlineStr">
         <is>
-          <t>GIH34D</t>
+          <t>GIH33K</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
@@ -8902,7 +8902,7 @@
       </c>
       <c r="D191" t="inlineStr">
         <is>
-          <t>2023-04-05</t>
+          <t>2023-02-23</t>
         </is>
       </c>
       <c r="E191" t="inlineStr"/>
@@ -8913,7 +8913,7 @@
       </c>
       <c r="G191" t="inlineStr">
         <is>
-          <t>Kvalitativ och kvantitativ vetenskaplig metod</t>
+          <t>Funktionell anatomi (Klättring)</t>
         </is>
       </c>
       <c r="H191" t="inlineStr">
@@ -8923,14 +8923,14 @@
       </c>
       <c r="I191" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH34D</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH33K</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" s="2" t="inlineStr">
         <is>
-          <t>GIH34S</t>
+          <t>GIH33P</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
@@ -8945,7 +8945,7 @@
       </c>
       <c r="D192" t="inlineStr">
         <is>
-          <t>2023-05-09</t>
+          <t>2023-02-23</t>
         </is>
       </c>
       <c r="E192" t="inlineStr"/>
@@ -8956,7 +8956,7 @@
       </c>
       <c r="G192" t="inlineStr">
         <is>
-          <t>Lek, dans samt mål- och nätspel (VAL)</t>
+          <t>Biomekanik (Klättring)</t>
         </is>
       </c>
       <c r="H192" t="inlineStr">
@@ -8966,14 +8966,14 @@
       </c>
       <c r="I192" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH34S</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH33P</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" s="2" t="inlineStr">
         <is>
-          <t>GIH34T</t>
+          <t>GIH34D</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
@@ -8988,7 +8988,7 @@
       </c>
       <c r="D193" t="inlineStr">
         <is>
-          <t>2023-05-09</t>
+          <t>2023-04-05</t>
         </is>
       </c>
       <c r="E193" t="inlineStr"/>
@@ -8999,7 +8999,7 @@
       </c>
       <c r="G193" t="inlineStr">
         <is>
-          <t>Humanbiologi 2 (VAL)</t>
+          <t>Kvalitativ och kvantitativ vetenskaplig metod</t>
         </is>
       </c>
       <c r="H193" t="inlineStr">
@@ -9009,14 +9009,14 @@
       </c>
       <c r="I193" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH34T</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH34D</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" s="2" t="inlineStr">
         <is>
-          <t>GIH34U</t>
+          <t>GIH34S</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
@@ -9042,7 +9042,7 @@
       </c>
       <c r="G194" t="inlineStr">
         <is>
-          <t>Dans, gymnastik och friidrott (VAL)</t>
+          <t>Lek, dans samt mål- och nätspel (VAL)</t>
         </is>
       </c>
       <c r="H194" t="inlineStr">
@@ -9052,14 +9052,14 @@
       </c>
       <c r="I194" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH34U</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH34S</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" s="2" t="inlineStr">
         <is>
-          <t>GIH34V</t>
+          <t>GIH34T</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
@@ -9085,7 +9085,7 @@
       </c>
       <c r="G195" t="inlineStr">
         <is>
-          <t>Arbetsmiljö, ergonomi och näringslära (VAL)</t>
+          <t>Humanbiologi 2 (VAL)</t>
         </is>
       </c>
       <c r="H195" t="inlineStr">
@@ -9095,14 +9095,14 @@
       </c>
       <c r="I195" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH34V</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH34T</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" s="2" t="inlineStr">
         <is>
-          <t>GIH35B</t>
+          <t>GIH34U</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
@@ -9117,7 +9117,7 @@
       </c>
       <c r="D196" t="inlineStr">
         <is>
-          <t>2023-06-19</t>
+          <t>2023-05-09</t>
         </is>
       </c>
       <c r="E196" t="inlineStr"/>
@@ -9128,7 +9128,7 @@
       </c>
       <c r="G196" t="inlineStr">
         <is>
-          <t>Examensarbete för kandidatexamen i idrotts- och hälsovetenskap</t>
+          <t>Dans, gymnastik och friidrott (VAL)</t>
         </is>
       </c>
       <c r="H196" t="inlineStr">
@@ -9138,14 +9138,14 @@
       </c>
       <c r="I196" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH35B</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH34U</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" s="2" t="inlineStr">
         <is>
-          <t>GIH35P</t>
+          <t>GIH34V</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
@@ -9160,7 +9160,7 @@
       </c>
       <c r="D197" t="inlineStr">
         <is>
-          <t>2023-08-30</t>
+          <t>2023-05-09</t>
         </is>
       </c>
       <c r="E197" t="inlineStr"/>
@@ -9171,7 +9171,7 @@
       </c>
       <c r="G197" t="inlineStr">
         <is>
-          <t>Träningslära: styrkelyft för öppen klass och veteraner</t>
+          <t>Arbetsmiljö, ergonomi och näringslära (VAL)</t>
         </is>
       </c>
       <c r="H197" t="inlineStr">
@@ -9181,14 +9181,14 @@
       </c>
       <c r="I197" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH35P</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH34V</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" s="2" t="inlineStr">
         <is>
-          <t>GIH35V</t>
+          <t>GIH35B</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
@@ -9203,7 +9203,7 @@
       </c>
       <c r="D198" t="inlineStr">
         <is>
-          <t>2023-08-30</t>
+          <t>2023-06-19</t>
         </is>
       </c>
       <c r="E198" t="inlineStr"/>
@@ -9214,7 +9214,7 @@
       </c>
       <c r="G198" t="inlineStr">
         <is>
-          <t>Idrottens träningslära</t>
+          <t>Examensarbete för kandidatexamen i idrotts- och hälsovetenskap</t>
         </is>
       </c>
       <c r="H198" t="inlineStr">
@@ -9224,14 +9224,14 @@
       </c>
       <c r="I198" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH35V</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH35B</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" s="2" t="inlineStr">
         <is>
-          <t>GIH35Z</t>
+          <t>GIH35P</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
@@ -9257,7 +9257,7 @@
       </c>
       <c r="G199" t="inlineStr">
         <is>
-          <t>Medier och kommunikation inom hälsa och idrott</t>
+          <t>Träningslära: styrkelyft för öppen klass och veteraner</t>
         </is>
       </c>
       <c r="H199" t="inlineStr">
@@ -9267,19 +9267,19 @@
       </c>
       <c r="I199" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH35Z</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH35P</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" s="2" t="inlineStr">
         <is>
-          <t>AMC29F</t>
+          <t>GIH35V</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>MCA</t>
+          <t>IDA</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
@@ -9295,12 +9295,12 @@
       <c r="E200" t="inlineStr"/>
       <c r="F200" t="inlineStr">
         <is>
-          <t>Medicinsk vetenskap</t>
+          <t>Idrotts- och hälsovetenskap</t>
         </is>
       </c>
       <c r="G200" t="inlineStr">
         <is>
-          <t>Examensarbete för magisterexamen i fysioterapi</t>
+          <t>Idrottens träningslära</t>
         </is>
       </c>
       <c r="H200" t="inlineStr">
@@ -9310,19 +9310,19 @@
       </c>
       <c r="I200" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMC29F</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH35V</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" s="2" t="inlineStr">
         <is>
-          <t>ASR29U</t>
+          <t>GIH35Z</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>SRP</t>
+          <t>IDA</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
@@ -9332,18 +9332,18 @@
       </c>
       <c r="D201" t="inlineStr">
         <is>
-          <t>2023-10-03</t>
+          <t>2023-08-30</t>
         </is>
       </c>
       <c r="E201" t="inlineStr"/>
       <c r="F201" t="inlineStr">
         <is>
-          <t>Sexuell, reproduktiv och perinatal hälsa</t>
+          <t>Idrotts- och hälsovetenskap</t>
         </is>
       </c>
       <c r="G201" t="inlineStr">
         <is>
-          <t>Graviditet, förlossning och postpartumvård II</t>
+          <t>Medier och kommunikation inom hälsa och idrott</t>
         </is>
       </c>
       <c r="H201" t="inlineStr">
@@ -9353,19 +9353,19 @@
       </c>
       <c r="I201" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29U</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH35Z</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" s="2" t="inlineStr">
         <is>
-          <t>GIH37B</t>
+          <t>AMC29F</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>IDA</t>
+          <t>MCA</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
@@ -9375,18 +9375,18 @@
       </c>
       <c r="D202" t="inlineStr">
         <is>
-          <t>2023-11-07</t>
+          <t>2023-08-30</t>
         </is>
       </c>
       <c r="E202" t="inlineStr"/>
       <c r="F202" t="inlineStr">
         <is>
-          <t>Idrotts- och hälsovetenskap</t>
+          <t>Medicinsk vetenskap</t>
         </is>
       </c>
       <c r="G202" t="inlineStr">
         <is>
-          <t>Mål- och nätspel (VAL)</t>
+          <t>Examensarbete för magisterexamen i fysioterapi</t>
         </is>
       </c>
       <c r="H202" t="inlineStr">
@@ -9396,19 +9396,19 @@
       </c>
       <c r="I202" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH37B</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMC29F</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" s="2" t="inlineStr">
         <is>
-          <t>GIH37C</t>
+          <t>ASR29U</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>IDA</t>
+          <t>SRP</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
@@ -9418,18 +9418,18 @@
       </c>
       <c r="D203" t="inlineStr">
         <is>
-          <t>2023-11-07</t>
+          <t>2023-10-03</t>
         </is>
       </c>
       <c r="E203" t="inlineStr"/>
       <c r="F203" t="inlineStr">
         <is>
-          <t>Idrotts- och hälsovetenskap</t>
+          <t>Sexuell, reproduktiv och perinatal hälsa</t>
         </is>
       </c>
       <c r="G203" t="inlineStr">
         <is>
-          <t>Rörelse, rytm och dans (VAL)</t>
+          <t>Graviditet, förlossning och postpartumvård II</t>
         </is>
       </c>
       <c r="H203" t="inlineStr">
@@ -9439,19 +9439,19 @@
       </c>
       <c r="I203" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH37C</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29U</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" s="2" t="inlineStr">
         <is>
-          <t>GVÅ37H</t>
+          <t>GIH37B</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>OMV</t>
+          <t>IDA</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
@@ -9467,12 +9467,12 @@
       <c r="E204" t="inlineStr"/>
       <c r="F204" t="inlineStr">
         <is>
-          <t>Omvårdnad</t>
+          <t>Idrotts- och hälsovetenskap</t>
         </is>
       </c>
       <c r="G204" t="inlineStr">
         <is>
-          <t>Personcentrerad vård inom psykiatrisk vård</t>
+          <t>Mål- och nätspel (VAL)</t>
         </is>
       </c>
       <c r="H204" t="inlineStr">
@@ -9482,19 +9482,19 @@
       </c>
       <c r="I204" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GVÅ37H</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH37B</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" s="2" t="inlineStr">
         <is>
-          <t>GVÅ382</t>
+          <t>GIH37C</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>OMV</t>
+          <t>IDA</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
@@ -9510,12 +9510,12 @@
       <c r="E205" t="inlineStr"/>
       <c r="F205" t="inlineStr">
         <is>
-          <t>Omvårdnad</t>
+          <t>Idrotts- och hälsovetenskap</t>
         </is>
       </c>
       <c r="G205" t="inlineStr">
         <is>
-          <t>Personcentrerad vård inom olika vårdsammanhang</t>
+          <t>Rörelse, rytm och dans (VAL)</t>
         </is>
       </c>
       <c r="H205" t="inlineStr">
@@ -9525,19 +9525,19 @@
       </c>
       <c r="I205" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GVÅ382</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH37C</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" s="2" t="inlineStr">
         <is>
-          <t>GSA2DW</t>
+          <t>GVÅ37H</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>SAA</t>
+          <t>OMV</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
@@ -9547,22 +9547,18 @@
       </c>
       <c r="D206" t="inlineStr">
         <is>
-          <t>2020-02-20</t>
-        </is>
-      </c>
-      <c r="E206" t="inlineStr">
-        <is>
-          <t>2023-11-30</t>
-        </is>
-      </c>
+          <t>2023-11-07</t>
+        </is>
+      </c>
+      <c r="E206" t="inlineStr"/>
       <c r="F206" t="inlineStr">
         <is>
-          <t>Socialt arbete</t>
+          <t>Omvårdnad</t>
         </is>
       </c>
       <c r="G206" t="inlineStr">
         <is>
-          <t>Försörjning, rehabilitering och aktivering i socialt arbete</t>
+          <t>Personcentrerad vård inom psykiatrisk vård</t>
         </is>
       </c>
       <c r="H206" t="inlineStr">
@@ -9572,19 +9568,19 @@
       </c>
       <c r="I206" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA2DW</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GVÅ37H</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" s="2" t="inlineStr">
         <is>
-          <t>GIH37N</t>
+          <t>GVÅ382</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>IDA</t>
+          <t>OMV</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
@@ -9594,18 +9590,18 @@
       </c>
       <c r="D207" t="inlineStr">
         <is>
-          <t>2023-12-05</t>
+          <t>2023-11-07</t>
         </is>
       </c>
       <c r="E207" t="inlineStr"/>
       <c r="F207" t="inlineStr">
         <is>
-          <t>Idrotts- och hälsovetenskap</t>
+          <t>Omvårdnad</t>
         </is>
       </c>
       <c r="G207" t="inlineStr">
         <is>
-          <t>Friluftsliv och bedömning i ämnet idrott och hälsa</t>
+          <t>Personcentrerad vård inom olika vårdsammanhang</t>
         </is>
       </c>
       <c r="H207" t="inlineStr">
@@ -9615,19 +9611,19 @@
       </c>
       <c r="I207" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH37N</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GVÅ382</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" s="2" t="inlineStr">
         <is>
-          <t>GIH37P</t>
+          <t>GSA2DW</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>IDA</t>
+          <t>SAA</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
@@ -9637,18 +9633,22 @@
       </c>
       <c r="D208" t="inlineStr">
         <is>
-          <t>2023-12-05</t>
-        </is>
-      </c>
-      <c r="E208" t="inlineStr"/>
+          <t>2020-02-20</t>
+        </is>
+      </c>
+      <c r="E208" t="inlineStr">
+        <is>
+          <t>2023-11-30</t>
+        </is>
+      </c>
       <c r="F208" t="inlineStr">
         <is>
-          <t>Idrotts- och hälsovetenskap</t>
+          <t>Socialt arbete</t>
         </is>
       </c>
       <c r="G208" t="inlineStr">
         <is>
-          <t>Idrott och hälsa I med didaktisk inriktning åk 4-6</t>
+          <t>Försörjning, rehabilitering och aktivering i socialt arbete</t>
         </is>
       </c>
       <c r="H208" t="inlineStr">
@@ -9658,14 +9658,14 @@
       </c>
       <c r="I208" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH37P</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA2DW</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" s="2" t="inlineStr">
         <is>
-          <t>GIH37Q</t>
+          <t>GIH37N</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
@@ -9691,7 +9691,7 @@
       </c>
       <c r="G209" t="inlineStr">
         <is>
-          <t>Idrott och hälsa I med didaktisk inriktning</t>
+          <t>Friluftsliv och bedömning i ämnet idrott och hälsa</t>
         </is>
       </c>
       <c r="H209" t="inlineStr">
@@ -9701,19 +9701,19 @@
       </c>
       <c r="I209" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH37Q</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH37N</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" s="2" t="inlineStr">
         <is>
-          <t>AMC29Y</t>
+          <t>GIH37P</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>MCA</t>
+          <t>IDA</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
@@ -9729,12 +9729,12 @@
       <c r="E210" t="inlineStr"/>
       <c r="F210" t="inlineStr">
         <is>
-          <t>Medicinsk vetenskap</t>
+          <t>Idrotts- och hälsovetenskap</t>
         </is>
       </c>
       <c r="G210" t="inlineStr">
         <is>
-          <t>Förskrivningsrätt för vissa läkemedel och förbrukningsartiklar</t>
+          <t>Idrott och hälsa I med didaktisk inriktning åk 4-6</t>
         </is>
       </c>
       <c r="H210" t="inlineStr">
@@ -9744,19 +9744,19 @@
       </c>
       <c r="I210" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMC29Y</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH37P</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" s="2" t="inlineStr">
         <is>
-          <t>AMC2A7</t>
+          <t>GIH37Q</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>MCA</t>
+          <t>IDA</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
@@ -9772,12 +9772,12 @@
       <c r="E211" t="inlineStr"/>
       <c r="F211" t="inlineStr">
         <is>
-          <t>Medicinsk vetenskap</t>
+          <t>Idrotts- och hälsovetenskap</t>
         </is>
       </c>
       <c r="G211" t="inlineStr">
         <is>
-          <t>Kardiologi: Arytmi</t>
+          <t>Idrott och hälsa I med didaktisk inriktning</t>
         </is>
       </c>
       <c r="H211" t="inlineStr">
@@ -9787,19 +9787,19 @@
       </c>
       <c r="I211" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMC2A7</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH37Q</t>
         </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" s="2" t="inlineStr">
         <is>
-          <t>GVÅ384</t>
+          <t>AMC29Y</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>OMV</t>
+          <t>MCA</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
@@ -9815,12 +9815,12 @@
       <c r="E212" t="inlineStr"/>
       <c r="F212" t="inlineStr">
         <is>
-          <t>Omvårdnad</t>
+          <t>Medicinsk vetenskap</t>
         </is>
       </c>
       <c r="G212" t="inlineStr">
         <is>
-          <t>Personcentrerad vård inom somatisk vård</t>
+          <t>Förskrivningsrätt för vissa läkemedel och förbrukningsartiklar</t>
         </is>
       </c>
       <c r="H212" t="inlineStr">
@@ -9830,19 +9830,19 @@
       </c>
       <c r="I212" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GVÅ384</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMC29Y</t>
         </is>
       </c>
     </row>
     <row r="213">
       <c r="A213" s="2" t="inlineStr">
         <is>
-          <t>GSR38B</t>
+          <t>AMC2A7</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>SRP</t>
+          <t>MCA</t>
         </is>
       </c>
       <c r="C213" t="inlineStr">
@@ -9858,12 +9858,12 @@
       <c r="E213" t="inlineStr"/>
       <c r="F213" t="inlineStr">
         <is>
-          <t>Sexuell, reproduktiv och perinatal hälsa</t>
+          <t>Medicinsk vetenskap</t>
         </is>
       </c>
       <c r="G213" t="inlineStr">
         <is>
-          <t>Sexuell och reproduktiv hälsa samt rättigheter för ungdomar och unga vuxna i Ukraina</t>
+          <t>Kardiologi: Arytmi</t>
         </is>
       </c>
       <c r="H213" t="inlineStr">
@@ -9873,19 +9873,19 @@
       </c>
       <c r="I213" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSR38B</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMC2A7</t>
         </is>
       </c>
     </row>
     <row r="214">
       <c r="A214" s="2" t="inlineStr">
         <is>
-          <t>GNV396</t>
+          <t>GVÅ384</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>NAV</t>
+          <t>OMV</t>
         </is>
       </c>
       <c r="C214" t="inlineStr">
@@ -9895,18 +9895,18 @@
       </c>
       <c r="D214" t="inlineStr">
         <is>
-          <t>2023-12-20</t>
+          <t>2023-12-05</t>
         </is>
       </c>
       <c r="E214" t="inlineStr"/>
       <c r="F214" t="inlineStr">
         <is>
-          <t>Naturvetenskap</t>
+          <t>Omvårdnad</t>
         </is>
       </c>
       <c r="G214" t="inlineStr">
         <is>
-          <t>Teknik för grundlärare i förskoleklass och årskurs 1-6</t>
+          <t>Personcentrerad vård inom somatisk vård</t>
         </is>
       </c>
       <c r="H214" t="inlineStr">
@@ -9916,19 +9916,19 @@
       </c>
       <c r="I214" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GNV396</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GVÅ384</t>
         </is>
       </c>
     </row>
     <row r="215">
       <c r="A215" s="2" t="inlineStr">
         <is>
-          <t>GIH3AM</t>
+          <t>GSR38B</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>IDA</t>
+          <t>SRP</t>
         </is>
       </c>
       <c r="C215" t="inlineStr">
@@ -9938,18 +9938,18 @@
       </c>
       <c r="D215" t="inlineStr">
         <is>
-          <t>2024-02-27</t>
+          <t>2023-12-05</t>
         </is>
       </c>
       <c r="E215" t="inlineStr"/>
       <c r="F215" t="inlineStr">
         <is>
-          <t>Idrotts- och hälsovetenskap</t>
+          <t>Sexuell, reproduktiv och perinatal hälsa</t>
         </is>
       </c>
       <c r="G215" t="inlineStr">
         <is>
-          <t>Klättringens tränarskap</t>
+          <t>Sexuell och reproduktiv hälsa samt rättigheter för ungdomar och unga vuxna i Ukraina</t>
         </is>
       </c>
       <c r="H215" t="inlineStr">
@@ -9959,19 +9959,19 @@
       </c>
       <c r="I215" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3AM</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSR38B</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" s="2" t="inlineStr">
         <is>
-          <t>GIH3AQ</t>
+          <t>GNV396</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>IDA</t>
+          <t>NAV</t>
         </is>
       </c>
       <c r="C216" t="inlineStr">
@@ -9981,18 +9981,18 @@
       </c>
       <c r="D216" t="inlineStr">
         <is>
-          <t>2024-02-27</t>
+          <t>2023-12-20</t>
         </is>
       </c>
       <c r="E216" t="inlineStr"/>
       <c r="F216" t="inlineStr">
         <is>
-          <t>Idrotts- och hälsovetenskap</t>
+          <t>Naturvetenskap</t>
         </is>
       </c>
       <c r="G216" t="inlineStr">
         <is>
-          <t>Styrketräningens teori och praktiska tillämpning</t>
+          <t>Teknik för grundlärare i förskoleklass och årskurs 1-6</t>
         </is>
       </c>
       <c r="H216" t="inlineStr">
@@ -10002,19 +10002,19 @@
       </c>
       <c r="I216" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3AQ</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GNV396</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" s="2" t="inlineStr">
         <is>
-          <t>AMC2AE</t>
+          <t>GIH3AM</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>MCA</t>
+          <t>IDA</t>
         </is>
       </c>
       <c r="C217" t="inlineStr">
@@ -10030,12 +10030,12 @@
       <c r="E217" t="inlineStr"/>
       <c r="F217" t="inlineStr">
         <is>
-          <t>Medicinsk vetenskap</t>
+          <t>Idrotts- och hälsovetenskap</t>
         </is>
       </c>
       <c r="G217" t="inlineStr">
         <is>
-          <t>Fysioterapi med fokus på smärta och hållbar utveckling</t>
+          <t>Klättringens tränarskap</t>
         </is>
       </c>
       <c r="H217" t="inlineStr">
@@ -10045,19 +10045,19 @@
       </c>
       <c r="I217" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMC2AE</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3AM</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" s="2" t="inlineStr">
         <is>
-          <t>GSA3AS</t>
+          <t>GIH3AQ</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>SAA</t>
+          <t>IDA</t>
         </is>
       </c>
       <c r="C218" t="inlineStr">
@@ -10067,18 +10067,18 @@
       </c>
       <c r="D218" t="inlineStr">
         <is>
-          <t>2024-03-04</t>
+          <t>2024-02-27</t>
         </is>
       </c>
       <c r="E218" t="inlineStr"/>
       <c r="F218" t="inlineStr">
         <is>
-          <t>Socialt arbete</t>
+          <t>Idrotts- och hälsovetenskap</t>
         </is>
       </c>
       <c r="G218" t="inlineStr">
         <is>
-          <t>Samsjuklighet - skadligt bruk eller beroende och samtidig psykisk ohälsa</t>
+          <t>Styrketräningens teori och praktiska tillämpning</t>
         </is>
       </c>
       <c r="H218" t="inlineStr">
@@ -10088,19 +10088,19 @@
       </c>
       <c r="I218" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA3AS</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3AQ</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" s="2" t="inlineStr">
         <is>
-          <t>GIH3CS</t>
+          <t>AMC2AE</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>IDA</t>
+          <t>MCA</t>
         </is>
       </c>
       <c r="C219" t="inlineStr">
@@ -10110,18 +10110,18 @@
       </c>
       <c r="D219" t="inlineStr">
         <is>
-          <t>2024-11-12</t>
+          <t>2024-02-27</t>
         </is>
       </c>
       <c r="E219" t="inlineStr"/>
       <c r="F219" t="inlineStr">
         <is>
-          <t>Idrotts- och hälsovetenskap</t>
+          <t>Medicinsk vetenskap</t>
         </is>
       </c>
       <c r="G219" t="inlineStr">
         <is>
-          <t>Grundläggande idrottsfysiologi</t>
+          <t>Fysioterapi med fokus på smärta och hållbar utveckling</t>
         </is>
       </c>
       <c r="H219" t="inlineStr">
@@ -10131,19 +10131,19 @@
       </c>
       <c r="I219" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3CS</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMC2AE</t>
         </is>
       </c>
     </row>
     <row r="220">
       <c r="A220" s="2" t="inlineStr">
         <is>
-          <t>GIH3D4</t>
+          <t>GSA3AS</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>IDA</t>
+          <t>SAA</t>
         </is>
       </c>
       <c r="C220" t="inlineStr">
@@ -10153,18 +10153,18 @@
       </c>
       <c r="D220" t="inlineStr">
         <is>
-          <t>2024-11-12</t>
+          <t>2024-03-04</t>
         </is>
       </c>
       <c r="E220" t="inlineStr"/>
       <c r="F220" t="inlineStr">
         <is>
-          <t>Idrotts- och hälsovetenskap</t>
+          <t>Socialt arbete</t>
         </is>
       </c>
       <c r="G220" t="inlineStr">
         <is>
-          <t>Träningslära för tävlingsinriktad idrott</t>
+          <t>Samsjuklighet - skadligt bruk eller beroende och samtidig psykisk ohälsa</t>
         </is>
       </c>
       <c r="H220" t="inlineStr">
@@ -10174,14 +10174,14 @@
       </c>
       <c r="I220" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3D4</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA3AS</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" s="2" t="inlineStr">
         <is>
-          <t>GIH3D5</t>
+          <t>GIH3CS</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
@@ -10207,7 +10207,7 @@
       </c>
       <c r="G221" t="inlineStr">
         <is>
-          <t>Träningslära för hälsoinriktad fysisk aktivitet</t>
+          <t>Grundläggande idrottsfysiologi</t>
         </is>
       </c>
       <c r="H221" t="inlineStr">
@@ -10217,14 +10217,14 @@
       </c>
       <c r="I221" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3D5</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3CS</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" s="2" t="inlineStr">
         <is>
-          <t>GIH3D6</t>
+          <t>GIH3D4</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
@@ -10250,7 +10250,7 @@
       </c>
       <c r="G222" t="inlineStr">
         <is>
-          <t>Näringslära med inriktning mot idrott och fysisk aktivitet</t>
+          <t>Träningslära för tävlingsinriktad idrott</t>
         </is>
       </c>
       <c r="H222" t="inlineStr">
@@ -10260,19 +10260,19 @@
       </c>
       <c r="I222" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3D6</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3D4</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" s="2" t="inlineStr">
         <is>
-          <t>GSA3DN</t>
+          <t>GIH3D5</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>SAA</t>
+          <t>IDA</t>
         </is>
       </c>
       <c r="C223" t="inlineStr">
@@ -10282,18 +10282,18 @@
       </c>
       <c r="D223" t="inlineStr">
         <is>
-          <t>2024-12-10</t>
+          <t>2024-11-12</t>
         </is>
       </c>
       <c r="E223" t="inlineStr"/>
       <c r="F223" t="inlineStr">
         <is>
-          <t>Socialt arbete</t>
+          <t>Idrotts- och hälsovetenskap</t>
         </is>
       </c>
       <c r="G223" t="inlineStr">
         <is>
-          <t>Försörjning, rehabilitering och aktivering i socialt arbete</t>
+          <t>Träningslära för hälsoinriktad fysisk aktivitet</t>
         </is>
       </c>
       <c r="H223" t="inlineStr">
@@ -10303,19 +10303,19 @@
       </c>
       <c r="I223" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA3DN</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3D5</t>
         </is>
       </c>
     </row>
     <row r="224">
       <c r="A224" s="2" t="inlineStr">
         <is>
-          <t>GSA3DS</t>
+          <t>GIH3D6</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>SAA</t>
+          <t>IDA</t>
         </is>
       </c>
       <c r="C224" t="inlineStr">
@@ -10325,18 +10325,18 @@
       </c>
       <c r="D224" t="inlineStr">
         <is>
-          <t>2024-12-10</t>
+          <t>2024-11-12</t>
         </is>
       </c>
       <c r="E224" t="inlineStr"/>
       <c r="F224" t="inlineStr">
         <is>
-          <t>Socialt arbete</t>
+          <t>Idrotts- och hälsovetenskap</t>
         </is>
       </c>
       <c r="G224" t="inlineStr">
         <is>
-          <t>Organisation, grupp och samverkan</t>
+          <t>Näringslära med inriktning mot idrott och fysisk aktivitet</t>
         </is>
       </c>
       <c r="H224" t="inlineStr">
@@ -10346,19 +10346,19 @@
       </c>
       <c r="I224" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA3DS</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3D6</t>
         </is>
       </c>
     </row>
     <row r="225">
       <c r="A225" s="2" t="inlineStr">
         <is>
-          <t>GVÅ35Q</t>
+          <t>GSA3DN</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>OMV</t>
+          <t>SAA</t>
         </is>
       </c>
       <c r="C225" t="inlineStr">
@@ -10368,22 +10368,18 @@
       </c>
       <c r="D225" t="inlineStr">
         <is>
-          <t>2023-08-30</t>
-        </is>
-      </c>
-      <c r="E225" t="inlineStr">
-        <is>
-          <t>2025-01-13</t>
-        </is>
-      </c>
+          <t>2024-12-10</t>
+        </is>
+      </c>
+      <c r="E225" t="inlineStr"/>
       <c r="F225" t="inlineStr">
         <is>
-          <t>Omvårdnad</t>
+          <t>Socialt arbete</t>
         </is>
       </c>
       <c r="G225" t="inlineStr">
         <is>
-          <t>Personcentrerad vård inom olika vårdsammanhang</t>
+          <t>Försörjning, rehabilitering och aktivering i socialt arbete</t>
         </is>
       </c>
       <c r="H225" t="inlineStr">
@@ -10393,19 +10389,19 @@
       </c>
       <c r="I225" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GVÅ35Q</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA3DN</t>
         </is>
       </c>
     </row>
     <row r="226">
       <c r="A226" s="2" t="inlineStr">
         <is>
-          <t>GIH3F4</t>
+          <t>GSA3DS</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>IDA</t>
+          <t>SAA</t>
         </is>
       </c>
       <c r="C226" t="inlineStr">
@@ -10415,18 +10411,18 @@
       </c>
       <c r="D226" t="inlineStr">
         <is>
-          <t>2025-02-24</t>
+          <t>2024-12-10</t>
         </is>
       </c>
       <c r="E226" t="inlineStr"/>
       <c r="F226" t="inlineStr">
         <is>
-          <t>Idrotts- och hälsovetenskap</t>
+          <t>Socialt arbete</t>
         </is>
       </c>
       <c r="G226" t="inlineStr">
         <is>
-          <t>Idrottspsykologi med praktisk tillämpning</t>
+          <t>Organisation, grupp och samverkan</t>
         </is>
       </c>
       <c r="H226" t="inlineStr">
@@ -10436,19 +10432,19 @@
       </c>
       <c r="I226" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3F4</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA3DS</t>
         </is>
       </c>
     </row>
     <row r="227">
       <c r="A227" s="2" t="inlineStr">
         <is>
-          <t>GIH3F5</t>
+          <t>GVÅ35Q</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>IDA</t>
+          <t>OMV</t>
         </is>
       </c>
       <c r="C227" t="inlineStr">
@@ -10458,18 +10454,22 @@
       </c>
       <c r="D227" t="inlineStr">
         <is>
-          <t>2025-02-24</t>
-        </is>
-      </c>
-      <c r="E227" t="inlineStr"/>
+          <t>2023-08-30</t>
+        </is>
+      </c>
+      <c r="E227" t="inlineStr">
+        <is>
+          <t>2025-01-13</t>
+        </is>
+      </c>
       <c r="F227" t="inlineStr">
         <is>
-          <t>Idrotts- och hälsovetenskap</t>
+          <t>Omvårdnad</t>
         </is>
       </c>
       <c r="G227" t="inlineStr">
         <is>
-          <t>Idrottens organisation i samhället</t>
+          <t>Personcentrerad vård inom olika vårdsammanhang</t>
         </is>
       </c>
       <c r="H227" t="inlineStr">
@@ -10479,14 +10479,14 @@
       </c>
       <c r="I227" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3F5</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GVÅ35Q</t>
         </is>
       </c>
     </row>
     <row r="228">
       <c r="A228" s="2" t="inlineStr">
         <is>
-          <t>GIH3F8</t>
+          <t>GIH3F4</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
@@ -10512,7 +10512,7 @@
       </c>
       <c r="G228" t="inlineStr">
         <is>
-          <t>Idrottens funktionella anatomi och biomekanik</t>
+          <t>Idrottspsykologi med praktisk tillämpning</t>
         </is>
       </c>
       <c r="H228" t="inlineStr">
@@ -10522,14 +10522,14 @@
       </c>
       <c r="I228" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3F8</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3F4</t>
         </is>
       </c>
     </row>
     <row r="229">
       <c r="A229" s="2" t="inlineStr">
         <is>
-          <t>GIH3G5</t>
+          <t>GIH3F5</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
@@ -10544,7 +10544,7 @@
       </c>
       <c r="D229" t="inlineStr">
         <is>
-          <t>2025-06-09</t>
+          <t>2025-02-24</t>
         </is>
       </c>
       <c r="E229" t="inlineStr"/>
@@ -10555,7 +10555,7 @@
       </c>
       <c r="G229" t="inlineStr">
         <is>
-          <t>Idrottsvetenskaplig metod</t>
+          <t>Idrottens organisation i samhället</t>
         </is>
       </c>
       <c r="H229" t="inlineStr">
@@ -10565,14 +10565,14 @@
       </c>
       <c r="I229" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3G5</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3F5</t>
         </is>
       </c>
     </row>
     <row r="230">
       <c r="A230" s="2" t="inlineStr">
         <is>
-          <t>GIH3G6</t>
+          <t>GIH3F8</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
@@ -10587,7 +10587,7 @@
       </c>
       <c r="D230" t="inlineStr">
         <is>
-          <t>2025-06-09</t>
+          <t>2025-02-24</t>
         </is>
       </c>
       <c r="E230" t="inlineStr"/>
@@ -10598,7 +10598,7 @@
       </c>
       <c r="G230" t="inlineStr">
         <is>
-          <t>Idrottsvetenskaplig fördjupning</t>
+          <t>Idrottens funktionella anatomi och biomekanik</t>
         </is>
       </c>
       <c r="H230" t="inlineStr">
@@ -10608,14 +10608,14 @@
       </c>
       <c r="I230" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3G6</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3F8</t>
         </is>
       </c>
     </row>
     <row r="231">
       <c r="A231" s="2" t="inlineStr">
         <is>
-          <t>GIH3G8</t>
+          <t>GIH3G5</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
@@ -10641,7 +10641,7 @@
       </c>
       <c r="G231" t="inlineStr">
         <is>
-          <t>Coachning och träningsprocesser i praktiken</t>
+          <t>Idrottsvetenskaplig metod</t>
         </is>
       </c>
       <c r="H231" t="inlineStr">
@@ -10651,14 +10651,14 @@
       </c>
       <c r="I231" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3G8</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3G5</t>
         </is>
       </c>
     </row>
     <row r="232">
       <c r="A232" s="2" t="inlineStr">
         <is>
-          <t>GIH3G9</t>
+          <t>GIH3G6</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
@@ -10684,7 +10684,7 @@
       </c>
       <c r="G232" t="inlineStr">
         <is>
-          <t>Entreprenörskap inom idrott och hälsa</t>
+          <t>Idrottsvetenskaplig fördjupning</t>
         </is>
       </c>
       <c r="H232" t="inlineStr">
@@ -10694,14 +10694,14 @@
       </c>
       <c r="I232" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3G9</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3G6</t>
         </is>
       </c>
     </row>
     <row r="233">
       <c r="A233" s="2" t="inlineStr">
         <is>
-          <t>GIH3GA</t>
+          <t>GIH3G8</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
@@ -10727,7 +10727,7 @@
       </c>
       <c r="G233" t="inlineStr">
         <is>
-          <t>Examensarbete för kandidatexamen i idrotts- och hälsovetenskap</t>
+          <t>Coachning och träningsprocesser i praktiken</t>
         </is>
       </c>
       <c r="H233" t="inlineStr">
@@ -10737,14 +10737,14 @@
       </c>
       <c r="I233" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3GA</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3G8</t>
         </is>
       </c>
     </row>
     <row r="234">
       <c r="A234" s="2" t="inlineStr">
         <is>
-          <t>GIH3GC</t>
+          <t>GIH3G9</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
@@ -10770,7 +10770,7 @@
       </c>
       <c r="G234" t="inlineStr">
         <is>
-          <t>Idrottsnutrition</t>
+          <t>Entreprenörskap inom idrott och hälsa</t>
         </is>
       </c>
       <c r="H234" t="inlineStr">
@@ -10780,19 +10780,19 @@
       </c>
       <c r="I234" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3GC</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3G9</t>
         </is>
       </c>
     </row>
     <row r="235">
       <c r="A235" s="2" t="inlineStr">
         <is>
-          <t>GNV3GV</t>
+          <t>GIH3GA</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>NAV</t>
+          <t>IDA</t>
         </is>
       </c>
       <c r="C235" t="inlineStr">
@@ -10802,18 +10802,18 @@
       </c>
       <c r="D235" t="inlineStr">
         <is>
-          <t>2025-09-10</t>
+          <t>2025-06-09</t>
         </is>
       </c>
       <c r="E235" t="inlineStr"/>
       <c r="F235" t="inlineStr">
         <is>
-          <t>Naturvetenskap</t>
+          <t>Idrotts- och hälsovetenskap</t>
         </is>
       </c>
       <c r="G235" t="inlineStr">
         <is>
-          <t>Naturorienterande ämnen och teknik för lärare i årskurs 1-3. Ingår i lärarlyftet.</t>
+          <t>Examensarbete för kandidatexamen i idrotts- och hälsovetenskap</t>
         </is>
       </c>
       <c r="H235" t="inlineStr">
@@ -10823,19 +10823,19 @@
       </c>
       <c r="I235" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GNV3GV</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3GA</t>
         </is>
       </c>
     </row>
     <row r="236">
       <c r="A236" s="2" t="inlineStr">
         <is>
-          <t>AFT2C8</t>
+          <t>GIH3GC</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>FYS</t>
+          <t>IDA</t>
         </is>
       </c>
       <c r="C236" t="inlineStr">
@@ -10845,18 +10845,18 @@
       </c>
       <c r="D236" t="inlineStr">
         <is>
-          <t>2025-12-04</t>
+          <t>2025-06-09</t>
         </is>
       </c>
       <c r="E236" t="inlineStr"/>
       <c r="F236" t="inlineStr">
         <is>
-          <t>Fysioterapi</t>
+          <t>Idrotts- och hälsovetenskap</t>
         </is>
       </c>
       <c r="G236" t="inlineStr">
         <is>
-          <t>Forskningsmetodik och projektplan inför examensarbete för magisterexamen i fysioterapi</t>
+          <t>Idrottsnutrition</t>
         </is>
       </c>
       <c r="H236" t="inlineStr">
@@ -10866,19 +10866,19 @@
       </c>
       <c r="I236" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AFT2C8</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3GC</t>
         </is>
       </c>
     </row>
     <row r="237">
       <c r="A237" s="2" t="inlineStr">
         <is>
-          <t>GIH3JL</t>
+          <t>GNV3GV</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>IDA</t>
+          <t>NAV</t>
         </is>
       </c>
       <c r="C237" t="inlineStr">
@@ -10888,33 +10888,119 @@
       </c>
       <c r="D237" t="inlineStr">
         <is>
-          <t>2026-03-03</t>
+          <t>2025-09-10</t>
         </is>
       </c>
       <c r="E237" t="inlineStr"/>
       <c r="F237" t="inlineStr">
         <is>
+          <t>Naturvetenskap</t>
+        </is>
+      </c>
+      <c r="G237" t="inlineStr">
+        <is>
+          <t>Naturorienterande ämnen och teknik för lärare i årskurs 1-3. Ingår i lärarlyftet.</t>
+        </is>
+      </c>
+      <c r="H237" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I237" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GNV3GV</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" s="2" t="inlineStr">
+        <is>
+          <t>AFT2C8</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>FYS</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>IHV</t>
+        </is>
+      </c>
+      <c r="D238" t="inlineStr">
+        <is>
+          <t>2025-12-04</t>
+        </is>
+      </c>
+      <c r="E238" t="inlineStr"/>
+      <c r="F238" t="inlineStr">
+        <is>
+          <t>Fysioterapi</t>
+        </is>
+      </c>
+      <c r="G238" t="inlineStr">
+        <is>
+          <t>Forskningsmetodik och projektplan inför examensarbete för magisterexamen i fysioterapi</t>
+        </is>
+      </c>
+      <c r="H238" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I238" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AFT2C8</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" s="2" t="inlineStr">
+        <is>
+          <t>GIH3JL</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>IDA</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>IHV</t>
+        </is>
+      </c>
+      <c r="D239" t="inlineStr">
+        <is>
+          <t>2026-03-03</t>
+        </is>
+      </c>
+      <c r="E239" t="inlineStr"/>
+      <c r="F239" t="inlineStr">
+        <is>
           <t>Idrotts- och hälsovetenskap</t>
         </is>
       </c>
-      <c r="G237" t="inlineStr">
+      <c r="G239" t="inlineStr">
         <is>
           <t>Tillämpad idrottsfysiologi</t>
         </is>
       </c>
-      <c r="H237" t="inlineStr">
-        <is>
-          <t>Ingen aktiv kursomgång</t>
-        </is>
-      </c>
-      <c r="I237" s="2" t="inlineStr">
+      <c r="H239" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I239" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3JL</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I237"/>
+  <autoFilter ref="A1:I239"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I2" r:id="rId2"/>
@@ -11388,6 +11474,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I236" r:id="rId470"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A237" r:id="rId471"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I237" r:id="rId472"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A238" r:id="rId473"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I238" r:id="rId474"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A239" r:id="rId475"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I239" r:id="rId476"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update course plans and analysis files for Dalarna University
- Updated the scrape date in the Dalarna Dashboard to reflect the latest data retrieval on 2026-08-25.
- Modified the Vilande kursplaner.md to update the number of entries from 238 to 239 and added a new course reference.
- Adjusted the number of courses listed in the Omvårdnad course plan from 35 to 34, reflecting the removal of GVÅ2WS.
- Updated various Excel analysis files across IIT, IHV, IKS, and ISLL directories to reflect the latest data changes.
- Added new entries and corrected inconsistencies in multiple analysis files, ensuring data accuracy and completeness.
</commit_message>
<xml_diff>
--- a/vault-dalarna-university/02 IHV/Analys/Vilande kursplaner.xlsx
+++ b/vault-dalarna-university/02 IHV/Analys/Vilande kursplaner.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Vilande kursplaner" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Vilande kursplaner'!$A$1:$I$239</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Vilande kursplaner'!$A$1:$I$240</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I239"/>
+  <dimension ref="A1:I240"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8062,12 +8062,12 @@
     <row r="172">
       <c r="A172" s="2" t="inlineStr">
         <is>
-          <t>ASR284</t>
+          <t>GVÅ2WS</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>SRP</t>
+          <t>OMV</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
@@ -8083,12 +8083,12 @@
       <c r="E172" t="inlineStr"/>
       <c r="F172" t="inlineStr">
         <is>
-          <t>Sexuell, reproduktiv och perinatal hälsa</t>
+          <t>Omvårdnad</t>
         </is>
       </c>
       <c r="G172" t="inlineStr">
         <is>
-          <t>Förlossningsvård I, verksamhetsförlagd utbildning</t>
+          <t>Global hälsa</t>
         </is>
       </c>
       <c r="H172" t="inlineStr">
@@ -8098,14 +8098,14 @@
       </c>
       <c r="I172" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR284</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GVÅ2WS</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" s="2" t="inlineStr">
         <is>
-          <t>ASR285</t>
+          <t>ASR284</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
@@ -8131,7 +8131,7 @@
       </c>
       <c r="G173" t="inlineStr">
         <is>
-          <t>Gynekologisk vård och postpartumvård, verksamhetsförlagd utbildning</t>
+          <t>Förlossningsvård I, verksamhetsförlagd utbildning</t>
         </is>
       </c>
       <c r="H173" t="inlineStr">
@@ -8141,14 +8141,14 @@
       </c>
       <c r="I173" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR285</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR284</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" s="2" t="inlineStr">
         <is>
-          <t>ASR286</t>
+          <t>ASR285</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
@@ -8174,7 +8174,7 @@
       </c>
       <c r="G174" t="inlineStr">
         <is>
-          <t>Examensarbete i sexuell, reproduktiv och perinatal hälsa</t>
+          <t>Gynekologisk vård och postpartumvård, verksamhetsförlagd utbildning</t>
         </is>
       </c>
       <c r="H174" t="inlineStr">
@@ -8184,19 +8184,19 @@
       </c>
       <c r="I174" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR286</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR285</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" s="2" t="inlineStr">
         <is>
-          <t>GIH2X3</t>
+          <t>ASR286</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>IDA</t>
+          <t>SRP</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
@@ -8209,19 +8209,15 @@
           <t>2022-06-16</t>
         </is>
       </c>
-      <c r="E175" t="inlineStr">
-        <is>
-          <t>2022-08-22</t>
-        </is>
-      </c>
+      <c r="E175" t="inlineStr"/>
       <c r="F175" t="inlineStr">
         <is>
-          <t>Idrotts- och hälsovetenskap</t>
+          <t>Sexuell, reproduktiv och perinatal hälsa</t>
         </is>
       </c>
       <c r="G175" t="inlineStr">
         <is>
-          <t>Träningslära för tävlingsinriktad idrott</t>
+          <t>Examensarbete i sexuell, reproduktiv och perinatal hälsa</t>
         </is>
       </c>
       <c r="H175" t="inlineStr">
@@ -8231,19 +8227,19 @@
       </c>
       <c r="I175" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2X3</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR286</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" s="2" t="inlineStr">
         <is>
-          <t>AMC288</t>
+          <t>GIH2X3</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>MCA</t>
+          <t>IDA</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
@@ -8253,18 +8249,22 @@
       </c>
       <c r="D176" t="inlineStr">
         <is>
-          <t>2022-09-08</t>
-        </is>
-      </c>
-      <c r="E176" t="inlineStr"/>
+          <t>2022-06-16</t>
+        </is>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>2022-08-22</t>
+        </is>
+      </c>
       <c r="F176" t="inlineStr">
         <is>
-          <t>Medicinsk vetenskap</t>
+          <t>Idrotts- och hälsovetenskap</t>
         </is>
       </c>
       <c r="G176" t="inlineStr">
         <is>
-          <t>Fysisk aktivitet och träning som prevention och behandling</t>
+          <t>Träningslära för tävlingsinriktad idrott</t>
         </is>
       </c>
       <c r="H176" t="inlineStr">
@@ -8274,19 +8274,19 @@
       </c>
       <c r="I176" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMC288</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2X3</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" s="2" t="inlineStr">
         <is>
-          <t>GSA2XN</t>
+          <t>AMC288</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>SAA</t>
+          <t>MCA</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
@@ -8302,12 +8302,12 @@
       <c r="E177" t="inlineStr"/>
       <c r="F177" t="inlineStr">
         <is>
-          <t>Socialt arbete</t>
+          <t>Medicinsk vetenskap</t>
         </is>
       </c>
       <c r="G177" t="inlineStr">
         <is>
-          <t>Missbruk och beroende</t>
+          <t>Fysisk aktivitet och träning som prevention och behandling</t>
         </is>
       </c>
       <c r="H177" t="inlineStr">
@@ -8317,19 +8317,19 @@
       </c>
       <c r="I177" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA2XN</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMC288</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" s="2" t="inlineStr">
         <is>
-          <t>GIH2XY</t>
+          <t>GSA2XN</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>IDA</t>
+          <t>SAA</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
@@ -8339,22 +8339,18 @@
       </c>
       <c r="D178" t="inlineStr">
         <is>
-          <t>2022-09-26</t>
-        </is>
-      </c>
-      <c r="E178" t="inlineStr">
-        <is>
-          <t>2022-09-30</t>
-        </is>
-      </c>
+          <t>2022-09-08</t>
+        </is>
+      </c>
+      <c r="E178" t="inlineStr"/>
       <c r="F178" t="inlineStr">
         <is>
-          <t>Idrotts- och hälsovetenskap</t>
+          <t>Socialt arbete</t>
         </is>
       </c>
       <c r="G178" t="inlineStr">
         <is>
-          <t>Idrottsvetenskaplig uppsats</t>
+          <t>Missbruk och beroende</t>
         </is>
       </c>
       <c r="H178" t="inlineStr">
@@ -8364,19 +8360,19 @@
       </c>
       <c r="I178" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2XY</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA2XN</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" s="2" t="inlineStr">
         <is>
-          <t>AVÅ28C</t>
+          <t>GIH2XY</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>OMV</t>
+          <t>IDA</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
@@ -8386,18 +8382,22 @@
       </c>
       <c r="D179" t="inlineStr">
         <is>
-          <t>2022-11-14</t>
-        </is>
-      </c>
-      <c r="E179" t="inlineStr"/>
+          <t>2022-09-26</t>
+        </is>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>2022-09-30</t>
+        </is>
+      </c>
       <c r="F179" t="inlineStr">
         <is>
-          <t>Omvårdnad</t>
+          <t>Idrotts- och hälsovetenskap</t>
         </is>
       </c>
       <c r="G179" t="inlineStr">
         <is>
-          <t>Telefonrådgivning vid distanskontakter inom hälso- och sjukvården</t>
+          <t>Idrottsvetenskaplig uppsats</t>
         </is>
       </c>
       <c r="H179" t="inlineStr">
@@ -8407,14 +8407,14 @@
       </c>
       <c r="I179" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AVÅ28C</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2XY</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" s="2" t="inlineStr">
         <is>
-          <t>AVÅ28H</t>
+          <t>AVÅ28C</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
@@ -8440,7 +8440,7 @@
       </c>
       <c r="G180" t="inlineStr">
         <is>
-          <t>Nutrition och ätande (fristående kurs)</t>
+          <t>Telefonrådgivning vid distanskontakter inom hälso- och sjukvården</t>
         </is>
       </c>
       <c r="H180" t="inlineStr">
@@ -8450,19 +8450,19 @@
       </c>
       <c r="I180" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AVÅ28H</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AVÅ28C</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" s="2" t="inlineStr">
         <is>
-          <t>GIH2ZA</t>
+          <t>AVÅ28H</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>IDA</t>
+          <t>OMV</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
@@ -8472,18 +8472,18 @@
       </c>
       <c r="D181" t="inlineStr">
         <is>
-          <t>2022-12-12</t>
+          <t>2022-11-14</t>
         </is>
       </c>
       <c r="E181" t="inlineStr"/>
       <c r="F181" t="inlineStr">
         <is>
-          <t>Idrotts- och hälsovetenskap</t>
+          <t>Omvårdnad</t>
         </is>
       </c>
       <c r="G181" t="inlineStr">
         <is>
-          <t>Vinterfriluftsliv genom skidor och skridskor (VAL)</t>
+          <t>Nutrition och ätande (fristående kurs)</t>
         </is>
       </c>
       <c r="H181" t="inlineStr">
@@ -8493,14 +8493,14 @@
       </c>
       <c r="I181" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2ZA</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AVÅ28H</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" s="2" t="inlineStr">
         <is>
-          <t>GIH2ZB</t>
+          <t>GIH2ZA</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
@@ -8526,7 +8526,7 @@
       </c>
       <c r="G182" t="inlineStr">
         <is>
-          <t>Hälsopedagogik (VAL)</t>
+          <t>Vinterfriluftsliv genom skidor och skridskor (VAL)</t>
         </is>
       </c>
       <c r="H182" t="inlineStr">
@@ -8536,14 +8536,14 @@
       </c>
       <c r="I182" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2ZB</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2ZA</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" s="2" t="inlineStr">
         <is>
-          <t>GIH2ZC</t>
+          <t>GIH2ZB</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
@@ -8569,7 +8569,7 @@
       </c>
       <c r="G183" t="inlineStr">
         <is>
-          <t>Humanbiologi 1 (VAL)</t>
+          <t>Hälsopedagogik (VAL)</t>
         </is>
       </c>
       <c r="H183" t="inlineStr">
@@ -8579,14 +8579,14 @@
       </c>
       <c r="I183" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2ZC</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2ZB</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" s="2" t="inlineStr">
         <is>
-          <t>GIH2ZD</t>
+          <t>GIH2ZC</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
@@ -8612,7 +8612,7 @@
       </c>
       <c r="G184" t="inlineStr">
         <is>
-          <t>Simning (VAL)</t>
+          <t>Humanbiologi 1 (VAL)</t>
         </is>
       </c>
       <c r="H184" t="inlineStr">
@@ -8622,14 +8622,14 @@
       </c>
       <c r="I184" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2ZD</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2ZC</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" s="2" t="inlineStr">
         <is>
-          <t>GIH2ZE</t>
+          <t>GIH2ZD</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
@@ -8655,7 +8655,7 @@
       </c>
       <c r="G185" t="inlineStr">
         <is>
-          <t>Bedömning och betygssättning i idrott och hälsa (VAL)</t>
+          <t>Simning (VAL)</t>
         </is>
       </c>
       <c r="H185" t="inlineStr">
@@ -8665,19 +8665,19 @@
       </c>
       <c r="I185" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2ZE</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2ZD</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" s="2" t="inlineStr">
         <is>
-          <t>GVÅ2ZG</t>
+          <t>GIH2ZE</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>OMV</t>
+          <t>IDA</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
@@ -8693,12 +8693,12 @@
       <c r="E186" t="inlineStr"/>
       <c r="F186" t="inlineStr">
         <is>
-          <t>Omvårdnad</t>
+          <t>Idrotts- och hälsovetenskap</t>
         </is>
       </c>
       <c r="G186" t="inlineStr">
         <is>
-          <t>Personcentrerad vård med fördjupning inom omvårdnad</t>
+          <t>Bedömning och betygssättning i idrott och hälsa (VAL)</t>
         </is>
       </c>
       <c r="H186" t="inlineStr">
@@ -8708,14 +8708,14 @@
       </c>
       <c r="I186" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GVÅ2ZG</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2ZE</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" s="2" t="inlineStr">
         <is>
-          <t>GVÅ2ZY</t>
+          <t>GVÅ2ZG</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
@@ -8741,7 +8741,7 @@
       </c>
       <c r="G187" t="inlineStr">
         <is>
-          <t>Metoder för evidensbaserad vård II</t>
+          <t>Personcentrerad vård med fördjupning inom omvårdnad</t>
         </is>
       </c>
       <c r="H187" t="inlineStr">
@@ -8751,19 +8751,19 @@
       </c>
       <c r="I187" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GVÅ2ZY</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GVÅ2ZG</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" s="2" t="inlineStr">
         <is>
-          <t>GIH334</t>
+          <t>GVÅ2ZY</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>IDA</t>
+          <t>OMV</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
@@ -8773,18 +8773,18 @@
       </c>
       <c r="D188" t="inlineStr">
         <is>
-          <t>2023-02-07</t>
+          <t>2022-12-12</t>
         </is>
       </c>
       <c r="E188" t="inlineStr"/>
       <c r="F188" t="inlineStr">
         <is>
-          <t>Idrotts- och hälsovetenskap</t>
+          <t>Omvårdnad</t>
         </is>
       </c>
       <c r="G188" t="inlineStr">
         <is>
-          <t>Sportjournalistik</t>
+          <t>Metoder för evidensbaserad vård II</t>
         </is>
       </c>
       <c r="H188" t="inlineStr">
@@ -8794,19 +8794,19 @@
       </c>
       <c r="I188" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH334</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GVÅ2ZY</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" s="2" t="inlineStr">
         <is>
-          <t>GSA32Y</t>
+          <t>GIH334</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>SAA</t>
+          <t>IDA</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
@@ -8822,12 +8822,12 @@
       <c r="E189" t="inlineStr"/>
       <c r="F189" t="inlineStr">
         <is>
-          <t>Socialt arbete</t>
+          <t>Idrotts- och hälsovetenskap</t>
         </is>
       </c>
       <c r="G189" t="inlineStr">
         <is>
-          <t>Organisation, grupp och samverkan</t>
+          <t>Sportjournalistik</t>
         </is>
       </c>
       <c r="H189" t="inlineStr">
@@ -8837,19 +8837,19 @@
       </c>
       <c r="I189" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA32Y</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH334</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" s="2" t="inlineStr">
         <is>
-          <t>GIH33J</t>
+          <t>GSA32Y</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>IDA</t>
+          <t>SAA</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
@@ -8859,18 +8859,18 @@
       </c>
       <c r="D190" t="inlineStr">
         <is>
-          <t>2023-02-23</t>
+          <t>2023-02-07</t>
         </is>
       </c>
       <c r="E190" t="inlineStr"/>
       <c r="F190" t="inlineStr">
         <is>
-          <t>Idrotts- och hälsovetenskap</t>
+          <t>Socialt arbete</t>
         </is>
       </c>
       <c r="G190" t="inlineStr">
         <is>
-          <t>Grundläggande fysiologi och tillämpad idrottsfysiologi (Klättring)</t>
+          <t>Organisation, grupp och samverkan</t>
         </is>
       </c>
       <c r="H190" t="inlineStr">
@@ -8880,14 +8880,14 @@
       </c>
       <c r="I190" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH33J</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA32Y</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" s="2" t="inlineStr">
         <is>
-          <t>GIH33K</t>
+          <t>GIH33J</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
@@ -8913,7 +8913,7 @@
       </c>
       <c r="G191" t="inlineStr">
         <is>
-          <t>Funktionell anatomi (Klättring)</t>
+          <t>Grundläggande fysiologi och tillämpad idrottsfysiologi (Klättring)</t>
         </is>
       </c>
       <c r="H191" t="inlineStr">
@@ -8923,14 +8923,14 @@
       </c>
       <c r="I191" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH33K</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH33J</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" s="2" t="inlineStr">
         <is>
-          <t>GIH33P</t>
+          <t>GIH33K</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
@@ -8956,7 +8956,7 @@
       </c>
       <c r="G192" t="inlineStr">
         <is>
-          <t>Biomekanik (Klättring)</t>
+          <t>Funktionell anatomi (Klättring)</t>
         </is>
       </c>
       <c r="H192" t="inlineStr">
@@ -8966,14 +8966,14 @@
       </c>
       <c r="I192" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH33P</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH33K</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" s="2" t="inlineStr">
         <is>
-          <t>GIH34D</t>
+          <t>GIH33P</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
@@ -8988,7 +8988,7 @@
       </c>
       <c r="D193" t="inlineStr">
         <is>
-          <t>2023-04-05</t>
+          <t>2023-02-23</t>
         </is>
       </c>
       <c r="E193" t="inlineStr"/>
@@ -8999,7 +8999,7 @@
       </c>
       <c r="G193" t="inlineStr">
         <is>
-          <t>Kvalitativ och kvantitativ vetenskaplig metod</t>
+          <t>Biomekanik (Klättring)</t>
         </is>
       </c>
       <c r="H193" t="inlineStr">
@@ -9009,14 +9009,14 @@
       </c>
       <c r="I193" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH34D</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH33P</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" s="2" t="inlineStr">
         <is>
-          <t>GIH34S</t>
+          <t>GIH34D</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
@@ -9031,7 +9031,7 @@
       </c>
       <c r="D194" t="inlineStr">
         <is>
-          <t>2023-05-09</t>
+          <t>2023-04-05</t>
         </is>
       </c>
       <c r="E194" t="inlineStr"/>
@@ -9042,7 +9042,7 @@
       </c>
       <c r="G194" t="inlineStr">
         <is>
-          <t>Lek, dans samt mål- och nätspel (VAL)</t>
+          <t>Kvalitativ och kvantitativ vetenskaplig metod</t>
         </is>
       </c>
       <c r="H194" t="inlineStr">
@@ -9052,14 +9052,14 @@
       </c>
       <c r="I194" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH34S</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH34D</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" s="2" t="inlineStr">
         <is>
-          <t>GIH34T</t>
+          <t>GIH34S</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
@@ -9085,7 +9085,7 @@
       </c>
       <c r="G195" t="inlineStr">
         <is>
-          <t>Humanbiologi 2 (VAL)</t>
+          <t>Lek, dans samt mål- och nätspel (VAL)</t>
         </is>
       </c>
       <c r="H195" t="inlineStr">
@@ -9095,14 +9095,14 @@
       </c>
       <c r="I195" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH34T</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH34S</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" s="2" t="inlineStr">
         <is>
-          <t>GIH34U</t>
+          <t>GIH34T</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
@@ -9128,7 +9128,7 @@
       </c>
       <c r="G196" t="inlineStr">
         <is>
-          <t>Dans, gymnastik och friidrott (VAL)</t>
+          <t>Humanbiologi 2 (VAL)</t>
         </is>
       </c>
       <c r="H196" t="inlineStr">
@@ -9138,14 +9138,14 @@
       </c>
       <c r="I196" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH34U</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH34T</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" s="2" t="inlineStr">
         <is>
-          <t>GIH34V</t>
+          <t>GIH34U</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
@@ -9171,7 +9171,7 @@
       </c>
       <c r="G197" t="inlineStr">
         <is>
-          <t>Arbetsmiljö, ergonomi och näringslära (VAL)</t>
+          <t>Dans, gymnastik och friidrott (VAL)</t>
         </is>
       </c>
       <c r="H197" t="inlineStr">
@@ -9181,14 +9181,14 @@
       </c>
       <c r="I197" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH34V</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH34U</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" s="2" t="inlineStr">
         <is>
-          <t>GIH35B</t>
+          <t>GIH34V</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
@@ -9203,7 +9203,7 @@
       </c>
       <c r="D198" t="inlineStr">
         <is>
-          <t>2023-06-19</t>
+          <t>2023-05-09</t>
         </is>
       </c>
       <c r="E198" t="inlineStr"/>
@@ -9214,7 +9214,7 @@
       </c>
       <c r="G198" t="inlineStr">
         <is>
-          <t>Examensarbete för kandidatexamen i idrotts- och hälsovetenskap</t>
+          <t>Arbetsmiljö, ergonomi och näringslära (VAL)</t>
         </is>
       </c>
       <c r="H198" t="inlineStr">
@@ -9224,14 +9224,14 @@
       </c>
       <c r="I198" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH35B</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH34V</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" s="2" t="inlineStr">
         <is>
-          <t>GIH35P</t>
+          <t>GIH35B</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
@@ -9246,7 +9246,7 @@
       </c>
       <c r="D199" t="inlineStr">
         <is>
-          <t>2023-08-30</t>
+          <t>2023-06-19</t>
         </is>
       </c>
       <c r="E199" t="inlineStr"/>
@@ -9257,7 +9257,7 @@
       </c>
       <c r="G199" t="inlineStr">
         <is>
-          <t>Träningslära: styrkelyft för öppen klass och veteraner</t>
+          <t>Examensarbete för kandidatexamen i idrotts- och hälsovetenskap</t>
         </is>
       </c>
       <c r="H199" t="inlineStr">
@@ -9267,14 +9267,14 @@
       </c>
       <c r="I199" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH35P</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH35B</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" s="2" t="inlineStr">
         <is>
-          <t>GIH35V</t>
+          <t>GIH35P</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
@@ -9300,7 +9300,7 @@
       </c>
       <c r="G200" t="inlineStr">
         <is>
-          <t>Idrottens träningslära</t>
+          <t>Träningslära: styrkelyft för öppen klass och veteraner</t>
         </is>
       </c>
       <c r="H200" t="inlineStr">
@@ -9310,14 +9310,14 @@
       </c>
       <c r="I200" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH35V</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH35P</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" s="2" t="inlineStr">
         <is>
-          <t>GIH35Z</t>
+          <t>GIH35V</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
@@ -9343,7 +9343,7 @@
       </c>
       <c r="G201" t="inlineStr">
         <is>
-          <t>Medier och kommunikation inom hälsa och idrott</t>
+          <t>Idrottens träningslära</t>
         </is>
       </c>
       <c r="H201" t="inlineStr">
@@ -9353,19 +9353,19 @@
       </c>
       <c r="I201" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH35Z</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH35V</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" s="2" t="inlineStr">
         <is>
-          <t>AMC29F</t>
+          <t>GIH35Z</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>MCA</t>
+          <t>IDA</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
@@ -9381,12 +9381,12 @@
       <c r="E202" t="inlineStr"/>
       <c r="F202" t="inlineStr">
         <is>
-          <t>Medicinsk vetenskap</t>
+          <t>Idrotts- och hälsovetenskap</t>
         </is>
       </c>
       <c r="G202" t="inlineStr">
         <is>
-          <t>Examensarbete för magisterexamen i fysioterapi</t>
+          <t>Medier och kommunikation inom hälsa och idrott</t>
         </is>
       </c>
       <c r="H202" t="inlineStr">
@@ -9396,19 +9396,19 @@
       </c>
       <c r="I202" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMC29F</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH35Z</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" s="2" t="inlineStr">
         <is>
-          <t>ASR29U</t>
+          <t>AMC29F</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>SRP</t>
+          <t>MCA</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
@@ -9418,18 +9418,18 @@
       </c>
       <c r="D203" t="inlineStr">
         <is>
-          <t>2023-10-03</t>
+          <t>2023-08-30</t>
         </is>
       </c>
       <c r="E203" t="inlineStr"/>
       <c r="F203" t="inlineStr">
         <is>
-          <t>Sexuell, reproduktiv och perinatal hälsa</t>
+          <t>Medicinsk vetenskap</t>
         </is>
       </c>
       <c r="G203" t="inlineStr">
         <is>
-          <t>Graviditet, förlossning och postpartumvård II</t>
+          <t>Examensarbete för magisterexamen i fysioterapi</t>
         </is>
       </c>
       <c r="H203" t="inlineStr">
@@ -9439,19 +9439,19 @@
       </c>
       <c r="I203" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29U</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMC29F</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" s="2" t="inlineStr">
         <is>
-          <t>GIH37B</t>
+          <t>ASR29U</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>IDA</t>
+          <t>SRP</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
@@ -9461,18 +9461,18 @@
       </c>
       <c r="D204" t="inlineStr">
         <is>
-          <t>2023-11-07</t>
+          <t>2023-10-03</t>
         </is>
       </c>
       <c r="E204" t="inlineStr"/>
       <c r="F204" t="inlineStr">
         <is>
-          <t>Idrotts- och hälsovetenskap</t>
+          <t>Sexuell, reproduktiv och perinatal hälsa</t>
         </is>
       </c>
       <c r="G204" t="inlineStr">
         <is>
-          <t>Mål- och nätspel (VAL)</t>
+          <t>Graviditet, förlossning och postpartumvård II</t>
         </is>
       </c>
       <c r="H204" t="inlineStr">
@@ -9482,14 +9482,14 @@
       </c>
       <c r="I204" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH37B</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29U</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" s="2" t="inlineStr">
         <is>
-          <t>GIH37C</t>
+          <t>GIH37B</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
@@ -9515,7 +9515,7 @@
       </c>
       <c r="G205" t="inlineStr">
         <is>
-          <t>Rörelse, rytm och dans (VAL)</t>
+          <t>Mål- och nätspel (VAL)</t>
         </is>
       </c>
       <c r="H205" t="inlineStr">
@@ -9525,19 +9525,19 @@
       </c>
       <c r="I205" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH37C</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH37B</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" s="2" t="inlineStr">
         <is>
-          <t>GVÅ37H</t>
+          <t>GIH37C</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>OMV</t>
+          <t>IDA</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
@@ -9553,12 +9553,12 @@
       <c r="E206" t="inlineStr"/>
       <c r="F206" t="inlineStr">
         <is>
-          <t>Omvårdnad</t>
+          <t>Idrotts- och hälsovetenskap</t>
         </is>
       </c>
       <c r="G206" t="inlineStr">
         <is>
-          <t>Personcentrerad vård inom psykiatrisk vård</t>
+          <t>Rörelse, rytm och dans (VAL)</t>
         </is>
       </c>
       <c r="H206" t="inlineStr">
@@ -9568,14 +9568,14 @@
       </c>
       <c r="I206" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GVÅ37H</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH37C</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" s="2" t="inlineStr">
         <is>
-          <t>GVÅ382</t>
+          <t>GVÅ37H</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
@@ -9601,7 +9601,7 @@
       </c>
       <c r="G207" t="inlineStr">
         <is>
-          <t>Personcentrerad vård inom olika vårdsammanhang</t>
+          <t>Personcentrerad vård inom psykiatrisk vård</t>
         </is>
       </c>
       <c r="H207" t="inlineStr">
@@ -9611,19 +9611,19 @@
       </c>
       <c r="I207" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GVÅ382</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GVÅ37H</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" s="2" t="inlineStr">
         <is>
-          <t>GSA2DW</t>
+          <t>GVÅ382</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>SAA</t>
+          <t>OMV</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
@@ -9633,22 +9633,18 @@
       </c>
       <c r="D208" t="inlineStr">
         <is>
-          <t>2020-02-20</t>
-        </is>
-      </c>
-      <c r="E208" t="inlineStr">
-        <is>
-          <t>2023-11-30</t>
-        </is>
-      </c>
+          <t>2023-11-07</t>
+        </is>
+      </c>
+      <c r="E208" t="inlineStr"/>
       <c r="F208" t="inlineStr">
         <is>
-          <t>Socialt arbete</t>
+          <t>Omvårdnad</t>
         </is>
       </c>
       <c r="G208" t="inlineStr">
         <is>
-          <t>Försörjning, rehabilitering och aktivering i socialt arbete</t>
+          <t>Personcentrerad vård inom olika vårdsammanhang</t>
         </is>
       </c>
       <c r="H208" t="inlineStr">
@@ -9658,19 +9654,19 @@
       </c>
       <c r="I208" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA2DW</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GVÅ382</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" s="2" t="inlineStr">
         <is>
-          <t>GIH37N</t>
+          <t>GSA2DW</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>IDA</t>
+          <t>SAA</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
@@ -9680,18 +9676,22 @@
       </c>
       <c r="D209" t="inlineStr">
         <is>
-          <t>2023-12-05</t>
-        </is>
-      </c>
-      <c r="E209" t="inlineStr"/>
+          <t>2020-02-20</t>
+        </is>
+      </c>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t>2023-11-30</t>
+        </is>
+      </c>
       <c r="F209" t="inlineStr">
         <is>
-          <t>Idrotts- och hälsovetenskap</t>
+          <t>Socialt arbete</t>
         </is>
       </c>
       <c r="G209" t="inlineStr">
         <is>
-          <t>Friluftsliv och bedömning i ämnet idrott och hälsa</t>
+          <t>Försörjning, rehabilitering och aktivering i socialt arbete</t>
         </is>
       </c>
       <c r="H209" t="inlineStr">
@@ -9701,14 +9701,14 @@
       </c>
       <c r="I209" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH37N</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA2DW</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" s="2" t="inlineStr">
         <is>
-          <t>GIH37P</t>
+          <t>GIH37N</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
@@ -9734,7 +9734,7 @@
       </c>
       <c r="G210" t="inlineStr">
         <is>
-          <t>Idrott och hälsa I med didaktisk inriktning åk 4-6</t>
+          <t>Friluftsliv och bedömning i ämnet idrott och hälsa</t>
         </is>
       </c>
       <c r="H210" t="inlineStr">
@@ -9744,14 +9744,14 @@
       </c>
       <c r="I210" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH37P</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH37N</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" s="2" t="inlineStr">
         <is>
-          <t>GIH37Q</t>
+          <t>GIH37P</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
@@ -9777,7 +9777,7 @@
       </c>
       <c r="G211" t="inlineStr">
         <is>
-          <t>Idrott och hälsa I med didaktisk inriktning</t>
+          <t>Idrott och hälsa I med didaktisk inriktning åk 4-6</t>
         </is>
       </c>
       <c r="H211" t="inlineStr">
@@ -9787,19 +9787,19 @@
       </c>
       <c r="I211" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH37Q</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH37P</t>
         </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" s="2" t="inlineStr">
         <is>
-          <t>AMC29Y</t>
+          <t>GIH37Q</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>MCA</t>
+          <t>IDA</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
@@ -9815,12 +9815,12 @@
       <c r="E212" t="inlineStr"/>
       <c r="F212" t="inlineStr">
         <is>
-          <t>Medicinsk vetenskap</t>
+          <t>Idrotts- och hälsovetenskap</t>
         </is>
       </c>
       <c r="G212" t="inlineStr">
         <is>
-          <t>Förskrivningsrätt för vissa läkemedel och förbrukningsartiklar</t>
+          <t>Idrott och hälsa I med didaktisk inriktning</t>
         </is>
       </c>
       <c r="H212" t="inlineStr">
@@ -9830,14 +9830,14 @@
       </c>
       <c r="I212" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMC29Y</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH37Q</t>
         </is>
       </c>
     </row>
     <row r="213">
       <c r="A213" s="2" t="inlineStr">
         <is>
-          <t>AMC2A7</t>
+          <t>AMC29Y</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
@@ -9863,7 +9863,7 @@
       </c>
       <c r="G213" t="inlineStr">
         <is>
-          <t>Kardiologi: Arytmi</t>
+          <t>Förskrivningsrätt för vissa läkemedel och förbrukningsartiklar</t>
         </is>
       </c>
       <c r="H213" t="inlineStr">
@@ -9873,19 +9873,19 @@
       </c>
       <c r="I213" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMC2A7</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMC29Y</t>
         </is>
       </c>
     </row>
     <row r="214">
       <c r="A214" s="2" t="inlineStr">
         <is>
-          <t>GVÅ384</t>
+          <t>AMC2A7</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>OMV</t>
+          <t>MCA</t>
         </is>
       </c>
       <c r="C214" t="inlineStr">
@@ -9901,12 +9901,12 @@
       <c r="E214" t="inlineStr"/>
       <c r="F214" t="inlineStr">
         <is>
-          <t>Omvårdnad</t>
+          <t>Medicinsk vetenskap</t>
         </is>
       </c>
       <c r="G214" t="inlineStr">
         <is>
-          <t>Personcentrerad vård inom somatisk vård</t>
+          <t>Kardiologi: Arytmi</t>
         </is>
       </c>
       <c r="H214" t="inlineStr">
@@ -9916,19 +9916,19 @@
       </c>
       <c r="I214" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GVÅ384</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMC2A7</t>
         </is>
       </c>
     </row>
     <row r="215">
       <c r="A215" s="2" t="inlineStr">
         <is>
-          <t>GSR38B</t>
+          <t>GVÅ384</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>SRP</t>
+          <t>OMV</t>
         </is>
       </c>
       <c r="C215" t="inlineStr">
@@ -9944,12 +9944,12 @@
       <c r="E215" t="inlineStr"/>
       <c r="F215" t="inlineStr">
         <is>
-          <t>Sexuell, reproduktiv och perinatal hälsa</t>
+          <t>Omvårdnad</t>
         </is>
       </c>
       <c r="G215" t="inlineStr">
         <is>
-          <t>Sexuell och reproduktiv hälsa samt rättigheter för ungdomar och unga vuxna i Ukraina</t>
+          <t>Personcentrerad vård inom somatisk vård</t>
         </is>
       </c>
       <c r="H215" t="inlineStr">
@@ -9959,19 +9959,19 @@
       </c>
       <c r="I215" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSR38B</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GVÅ384</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" s="2" t="inlineStr">
         <is>
-          <t>GNV396</t>
+          <t>GSR38B</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>NAV</t>
+          <t>SRP</t>
         </is>
       </c>
       <c r="C216" t="inlineStr">
@@ -9981,18 +9981,18 @@
       </c>
       <c r="D216" t="inlineStr">
         <is>
-          <t>2023-12-20</t>
+          <t>2023-12-05</t>
         </is>
       </c>
       <c r="E216" t="inlineStr"/>
       <c r="F216" t="inlineStr">
         <is>
-          <t>Naturvetenskap</t>
+          <t>Sexuell, reproduktiv och perinatal hälsa</t>
         </is>
       </c>
       <c r="G216" t="inlineStr">
         <is>
-          <t>Teknik för grundlärare i förskoleklass och årskurs 1-6</t>
+          <t>Sexuell och reproduktiv hälsa samt rättigheter för ungdomar och unga vuxna i Ukraina</t>
         </is>
       </c>
       <c r="H216" t="inlineStr">
@@ -10002,19 +10002,19 @@
       </c>
       <c r="I216" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GNV396</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSR38B</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" s="2" t="inlineStr">
         <is>
-          <t>GIH3AM</t>
+          <t>GNV396</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>IDA</t>
+          <t>NAV</t>
         </is>
       </c>
       <c r="C217" t="inlineStr">
@@ -10024,18 +10024,18 @@
       </c>
       <c r="D217" t="inlineStr">
         <is>
-          <t>2024-02-27</t>
+          <t>2023-12-20</t>
         </is>
       </c>
       <c r="E217" t="inlineStr"/>
       <c r="F217" t="inlineStr">
         <is>
-          <t>Idrotts- och hälsovetenskap</t>
+          <t>Naturvetenskap</t>
         </is>
       </c>
       <c r="G217" t="inlineStr">
         <is>
-          <t>Klättringens tränarskap</t>
+          <t>Teknik för grundlärare i förskoleklass och årskurs 1-6</t>
         </is>
       </c>
       <c r="H217" t="inlineStr">
@@ -10045,14 +10045,14 @@
       </c>
       <c r="I217" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3AM</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GNV396</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" s="2" t="inlineStr">
         <is>
-          <t>GIH3AQ</t>
+          <t>GIH3AM</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
@@ -10078,7 +10078,7 @@
       </c>
       <c r="G218" t="inlineStr">
         <is>
-          <t>Styrketräningens teori och praktiska tillämpning</t>
+          <t>Klättringens tränarskap</t>
         </is>
       </c>
       <c r="H218" t="inlineStr">
@@ -10088,19 +10088,19 @@
       </c>
       <c r="I218" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3AQ</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3AM</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" s="2" t="inlineStr">
         <is>
-          <t>AMC2AE</t>
+          <t>GIH3AQ</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>MCA</t>
+          <t>IDA</t>
         </is>
       </c>
       <c r="C219" t="inlineStr">
@@ -10116,12 +10116,12 @@
       <c r="E219" t="inlineStr"/>
       <c r="F219" t="inlineStr">
         <is>
-          <t>Medicinsk vetenskap</t>
+          <t>Idrotts- och hälsovetenskap</t>
         </is>
       </c>
       <c r="G219" t="inlineStr">
         <is>
-          <t>Fysioterapi med fokus på smärta och hållbar utveckling</t>
+          <t>Styrketräningens teori och praktiska tillämpning</t>
         </is>
       </c>
       <c r="H219" t="inlineStr">
@@ -10131,19 +10131,19 @@
       </c>
       <c r="I219" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMC2AE</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3AQ</t>
         </is>
       </c>
     </row>
     <row r="220">
       <c r="A220" s="2" t="inlineStr">
         <is>
-          <t>GSA3AS</t>
+          <t>AMC2AE</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>SAA</t>
+          <t>MCA</t>
         </is>
       </c>
       <c r="C220" t="inlineStr">
@@ -10153,18 +10153,18 @@
       </c>
       <c r="D220" t="inlineStr">
         <is>
-          <t>2024-03-04</t>
+          <t>2024-02-27</t>
         </is>
       </c>
       <c r="E220" t="inlineStr"/>
       <c r="F220" t="inlineStr">
         <is>
-          <t>Socialt arbete</t>
+          <t>Medicinsk vetenskap</t>
         </is>
       </c>
       <c r="G220" t="inlineStr">
         <is>
-          <t>Samsjuklighet - skadligt bruk eller beroende och samtidig psykisk ohälsa</t>
+          <t>Fysioterapi med fokus på smärta och hållbar utveckling</t>
         </is>
       </c>
       <c r="H220" t="inlineStr">
@@ -10174,19 +10174,19 @@
       </c>
       <c r="I220" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA3AS</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMC2AE</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" s="2" t="inlineStr">
         <is>
-          <t>GIH3CS</t>
+          <t>GSA3AS</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>IDA</t>
+          <t>SAA</t>
         </is>
       </c>
       <c r="C221" t="inlineStr">
@@ -10196,18 +10196,18 @@
       </c>
       <c r="D221" t="inlineStr">
         <is>
-          <t>2024-11-12</t>
+          <t>2024-03-04</t>
         </is>
       </c>
       <c r="E221" t="inlineStr"/>
       <c r="F221" t="inlineStr">
         <is>
-          <t>Idrotts- och hälsovetenskap</t>
+          <t>Socialt arbete</t>
         </is>
       </c>
       <c r="G221" t="inlineStr">
         <is>
-          <t>Grundläggande idrottsfysiologi</t>
+          <t>Samsjuklighet - skadligt bruk eller beroende och samtidig psykisk ohälsa</t>
         </is>
       </c>
       <c r="H221" t="inlineStr">
@@ -10217,14 +10217,14 @@
       </c>
       <c r="I221" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3CS</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA3AS</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" s="2" t="inlineStr">
         <is>
-          <t>GIH3D4</t>
+          <t>GIH3CS</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
@@ -10250,7 +10250,7 @@
       </c>
       <c r="G222" t="inlineStr">
         <is>
-          <t>Träningslära för tävlingsinriktad idrott</t>
+          <t>Grundläggande idrottsfysiologi</t>
         </is>
       </c>
       <c r="H222" t="inlineStr">
@@ -10260,14 +10260,14 @@
       </c>
       <c r="I222" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3D4</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3CS</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" s="2" t="inlineStr">
         <is>
-          <t>GIH3D5</t>
+          <t>GIH3D4</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
@@ -10293,7 +10293,7 @@
       </c>
       <c r="G223" t="inlineStr">
         <is>
-          <t>Träningslära för hälsoinriktad fysisk aktivitet</t>
+          <t>Träningslära för tävlingsinriktad idrott</t>
         </is>
       </c>
       <c r="H223" t="inlineStr">
@@ -10303,14 +10303,14 @@
       </c>
       <c r="I223" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3D5</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3D4</t>
         </is>
       </c>
     </row>
     <row r="224">
       <c r="A224" s="2" t="inlineStr">
         <is>
-          <t>GIH3D6</t>
+          <t>GIH3D5</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
@@ -10336,7 +10336,7 @@
       </c>
       <c r="G224" t="inlineStr">
         <is>
-          <t>Näringslära med inriktning mot idrott och fysisk aktivitet</t>
+          <t>Träningslära för hälsoinriktad fysisk aktivitet</t>
         </is>
       </c>
       <c r="H224" t="inlineStr">
@@ -10346,19 +10346,19 @@
       </c>
       <c r="I224" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3D6</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3D5</t>
         </is>
       </c>
     </row>
     <row r="225">
       <c r="A225" s="2" t="inlineStr">
         <is>
-          <t>GSA3DN</t>
+          <t>GIH3D6</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>SAA</t>
+          <t>IDA</t>
         </is>
       </c>
       <c r="C225" t="inlineStr">
@@ -10368,18 +10368,18 @@
       </c>
       <c r="D225" t="inlineStr">
         <is>
-          <t>2024-12-10</t>
+          <t>2024-11-12</t>
         </is>
       </c>
       <c r="E225" t="inlineStr"/>
       <c r="F225" t="inlineStr">
         <is>
-          <t>Socialt arbete</t>
+          <t>Idrotts- och hälsovetenskap</t>
         </is>
       </c>
       <c r="G225" t="inlineStr">
         <is>
-          <t>Försörjning, rehabilitering och aktivering i socialt arbete</t>
+          <t>Näringslära med inriktning mot idrott och fysisk aktivitet</t>
         </is>
       </c>
       <c r="H225" t="inlineStr">
@@ -10389,14 +10389,14 @@
       </c>
       <c r="I225" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA3DN</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3D6</t>
         </is>
       </c>
     </row>
     <row r="226">
       <c r="A226" s="2" t="inlineStr">
         <is>
-          <t>GSA3DS</t>
+          <t>GSA3DN</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
@@ -10422,7 +10422,7 @@
       </c>
       <c r="G226" t="inlineStr">
         <is>
-          <t>Organisation, grupp och samverkan</t>
+          <t>Försörjning, rehabilitering och aktivering i socialt arbete</t>
         </is>
       </c>
       <c r="H226" t="inlineStr">
@@ -10432,19 +10432,19 @@
       </c>
       <c r="I226" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA3DS</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA3DN</t>
         </is>
       </c>
     </row>
     <row r="227">
       <c r="A227" s="2" t="inlineStr">
         <is>
-          <t>GVÅ35Q</t>
+          <t>GSA3DS</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>OMV</t>
+          <t>SAA</t>
         </is>
       </c>
       <c r="C227" t="inlineStr">
@@ -10454,22 +10454,18 @@
       </c>
       <c r="D227" t="inlineStr">
         <is>
-          <t>2023-08-30</t>
-        </is>
-      </c>
-      <c r="E227" t="inlineStr">
-        <is>
-          <t>2025-01-13</t>
-        </is>
-      </c>
+          <t>2024-12-10</t>
+        </is>
+      </c>
+      <c r="E227" t="inlineStr"/>
       <c r="F227" t="inlineStr">
         <is>
-          <t>Omvårdnad</t>
+          <t>Socialt arbete</t>
         </is>
       </c>
       <c r="G227" t="inlineStr">
         <is>
-          <t>Personcentrerad vård inom olika vårdsammanhang</t>
+          <t>Organisation, grupp och samverkan</t>
         </is>
       </c>
       <c r="H227" t="inlineStr">
@@ -10479,19 +10475,19 @@
       </c>
       <c r="I227" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GVÅ35Q</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA3DS</t>
         </is>
       </c>
     </row>
     <row r="228">
       <c r="A228" s="2" t="inlineStr">
         <is>
-          <t>GIH3F4</t>
+          <t>GVÅ35Q</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>IDA</t>
+          <t>OMV</t>
         </is>
       </c>
       <c r="C228" t="inlineStr">
@@ -10501,18 +10497,22 @@
       </c>
       <c r="D228" t="inlineStr">
         <is>
-          <t>2025-02-24</t>
-        </is>
-      </c>
-      <c r="E228" t="inlineStr"/>
+          <t>2023-08-30</t>
+        </is>
+      </c>
+      <c r="E228" t="inlineStr">
+        <is>
+          <t>2025-01-13</t>
+        </is>
+      </c>
       <c r="F228" t="inlineStr">
         <is>
-          <t>Idrotts- och hälsovetenskap</t>
+          <t>Omvårdnad</t>
         </is>
       </c>
       <c r="G228" t="inlineStr">
         <is>
-          <t>Idrottspsykologi med praktisk tillämpning</t>
+          <t>Personcentrerad vård inom olika vårdsammanhang</t>
         </is>
       </c>
       <c r="H228" t="inlineStr">
@@ -10522,14 +10522,14 @@
       </c>
       <c r="I228" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3F4</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GVÅ35Q</t>
         </is>
       </c>
     </row>
     <row r="229">
       <c r="A229" s="2" t="inlineStr">
         <is>
-          <t>GIH3F5</t>
+          <t>GIH3F4</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
@@ -10555,7 +10555,7 @@
       </c>
       <c r="G229" t="inlineStr">
         <is>
-          <t>Idrottens organisation i samhället</t>
+          <t>Idrottspsykologi med praktisk tillämpning</t>
         </is>
       </c>
       <c r="H229" t="inlineStr">
@@ -10565,14 +10565,14 @@
       </c>
       <c r="I229" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3F5</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3F4</t>
         </is>
       </c>
     </row>
     <row r="230">
       <c r="A230" s="2" t="inlineStr">
         <is>
-          <t>GIH3F8</t>
+          <t>GIH3F5</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
@@ -10598,7 +10598,7 @@
       </c>
       <c r="G230" t="inlineStr">
         <is>
-          <t>Idrottens funktionella anatomi och biomekanik</t>
+          <t>Idrottens organisation i samhället</t>
         </is>
       </c>
       <c r="H230" t="inlineStr">
@@ -10608,14 +10608,14 @@
       </c>
       <c r="I230" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3F8</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3F5</t>
         </is>
       </c>
     </row>
     <row r="231">
       <c r="A231" s="2" t="inlineStr">
         <is>
-          <t>GIH3G5</t>
+          <t>GIH3F8</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
@@ -10630,7 +10630,7 @@
       </c>
       <c r="D231" t="inlineStr">
         <is>
-          <t>2025-06-09</t>
+          <t>2025-02-24</t>
         </is>
       </c>
       <c r="E231" t="inlineStr"/>
@@ -10641,7 +10641,7 @@
       </c>
       <c r="G231" t="inlineStr">
         <is>
-          <t>Idrottsvetenskaplig metod</t>
+          <t>Idrottens funktionella anatomi och biomekanik</t>
         </is>
       </c>
       <c r="H231" t="inlineStr">
@@ -10651,14 +10651,14 @@
       </c>
       <c r="I231" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3G5</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3F8</t>
         </is>
       </c>
     </row>
     <row r="232">
       <c r="A232" s="2" t="inlineStr">
         <is>
-          <t>GIH3G6</t>
+          <t>GIH3G5</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
@@ -10684,7 +10684,7 @@
       </c>
       <c r="G232" t="inlineStr">
         <is>
-          <t>Idrottsvetenskaplig fördjupning</t>
+          <t>Idrottsvetenskaplig metod</t>
         </is>
       </c>
       <c r="H232" t="inlineStr">
@@ -10694,14 +10694,14 @@
       </c>
       <c r="I232" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3G6</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3G5</t>
         </is>
       </c>
     </row>
     <row r="233">
       <c r="A233" s="2" t="inlineStr">
         <is>
-          <t>GIH3G8</t>
+          <t>GIH3G6</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
@@ -10727,7 +10727,7 @@
       </c>
       <c r="G233" t="inlineStr">
         <is>
-          <t>Coachning och träningsprocesser i praktiken</t>
+          <t>Idrottsvetenskaplig fördjupning</t>
         </is>
       </c>
       <c r="H233" t="inlineStr">
@@ -10737,14 +10737,14 @@
       </c>
       <c r="I233" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3G8</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3G6</t>
         </is>
       </c>
     </row>
     <row r="234">
       <c r="A234" s="2" t="inlineStr">
         <is>
-          <t>GIH3G9</t>
+          <t>GIH3G8</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
@@ -10770,7 +10770,7 @@
       </c>
       <c r="G234" t="inlineStr">
         <is>
-          <t>Entreprenörskap inom idrott och hälsa</t>
+          <t>Coachning och träningsprocesser i praktiken</t>
         </is>
       </c>
       <c r="H234" t="inlineStr">
@@ -10780,14 +10780,14 @@
       </c>
       <c r="I234" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3G9</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3G8</t>
         </is>
       </c>
     </row>
     <row r="235">
       <c r="A235" s="2" t="inlineStr">
         <is>
-          <t>GIH3GA</t>
+          <t>GIH3G9</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
@@ -10813,7 +10813,7 @@
       </c>
       <c r="G235" t="inlineStr">
         <is>
-          <t>Examensarbete för kandidatexamen i idrotts- och hälsovetenskap</t>
+          <t>Entreprenörskap inom idrott och hälsa</t>
         </is>
       </c>
       <c r="H235" t="inlineStr">
@@ -10823,14 +10823,14 @@
       </c>
       <c r="I235" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3GA</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3G9</t>
         </is>
       </c>
     </row>
     <row r="236">
       <c r="A236" s="2" t="inlineStr">
         <is>
-          <t>GIH3GC</t>
+          <t>GIH3GA</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
@@ -10856,7 +10856,7 @@
       </c>
       <c r="G236" t="inlineStr">
         <is>
-          <t>Idrottsnutrition</t>
+          <t>Examensarbete för kandidatexamen i idrotts- och hälsovetenskap</t>
         </is>
       </c>
       <c r="H236" t="inlineStr">
@@ -10866,19 +10866,19 @@
       </c>
       <c r="I236" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3GC</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3GA</t>
         </is>
       </c>
     </row>
     <row r="237">
       <c r="A237" s="2" t="inlineStr">
         <is>
-          <t>GNV3GV</t>
+          <t>GIH3GC</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>NAV</t>
+          <t>IDA</t>
         </is>
       </c>
       <c r="C237" t="inlineStr">
@@ -10888,18 +10888,18 @@
       </c>
       <c r="D237" t="inlineStr">
         <is>
-          <t>2025-09-10</t>
+          <t>2025-06-09</t>
         </is>
       </c>
       <c r="E237" t="inlineStr"/>
       <c r="F237" t="inlineStr">
         <is>
-          <t>Naturvetenskap</t>
+          <t>Idrotts- och hälsovetenskap</t>
         </is>
       </c>
       <c r="G237" t="inlineStr">
         <is>
-          <t>Naturorienterande ämnen och teknik för lärare i årskurs 1-3. Ingår i lärarlyftet.</t>
+          <t>Idrottsnutrition</t>
         </is>
       </c>
       <c r="H237" t="inlineStr">
@@ -10909,19 +10909,19 @@
       </c>
       <c r="I237" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GNV3GV</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3GC</t>
         </is>
       </c>
     </row>
     <row r="238">
       <c r="A238" s="2" t="inlineStr">
         <is>
-          <t>AFT2C8</t>
+          <t>GNV3GV</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>FYS</t>
+          <t>NAV</t>
         </is>
       </c>
       <c r="C238" t="inlineStr">
@@ -10931,18 +10931,18 @@
       </c>
       <c r="D238" t="inlineStr">
         <is>
-          <t>2025-12-04</t>
+          <t>2025-09-10</t>
         </is>
       </c>
       <c r="E238" t="inlineStr"/>
       <c r="F238" t="inlineStr">
         <is>
-          <t>Fysioterapi</t>
+          <t>Naturvetenskap</t>
         </is>
       </c>
       <c r="G238" t="inlineStr">
         <is>
-          <t>Forskningsmetodik och projektplan inför examensarbete för magisterexamen i fysioterapi</t>
+          <t>Naturorienterande ämnen och teknik för lärare i årskurs 1-3. Ingår i lärarlyftet.</t>
         </is>
       </c>
       <c r="H238" t="inlineStr">
@@ -10952,19 +10952,19 @@
       </c>
       <c r="I238" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AFT2C8</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GNV3GV</t>
         </is>
       </c>
     </row>
     <row r="239">
       <c r="A239" s="2" t="inlineStr">
         <is>
-          <t>GIH3JL</t>
+          <t>AFT2C8</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>IDA</t>
+          <t>FYS</t>
         </is>
       </c>
       <c r="C239" t="inlineStr">
@@ -10974,33 +10974,76 @@
       </c>
       <c r="D239" t="inlineStr">
         <is>
-          <t>2026-03-03</t>
+          <t>2025-12-04</t>
         </is>
       </c>
       <c r="E239" t="inlineStr"/>
       <c r="F239" t="inlineStr">
         <is>
+          <t>Fysioterapi</t>
+        </is>
+      </c>
+      <c r="G239" t="inlineStr">
+        <is>
+          <t>Forskningsmetodik och projektplan inför examensarbete för magisterexamen i fysioterapi</t>
+        </is>
+      </c>
+      <c r="H239" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I239" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AFT2C8</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" s="2" t="inlineStr">
+        <is>
+          <t>GIH3JL</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>IDA</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>IHV</t>
+        </is>
+      </c>
+      <c r="D240" t="inlineStr">
+        <is>
+          <t>2026-03-03</t>
+        </is>
+      </c>
+      <c r="E240" t="inlineStr"/>
+      <c r="F240" t="inlineStr">
+        <is>
           <t>Idrotts- och hälsovetenskap</t>
         </is>
       </c>
-      <c r="G239" t="inlineStr">
+      <c r="G240" t="inlineStr">
         <is>
           <t>Tillämpad idrottsfysiologi</t>
         </is>
       </c>
-      <c r="H239" t="inlineStr">
-        <is>
-          <t>Ingen aktiv kursomgång</t>
-        </is>
-      </c>
-      <c r="I239" s="2" t="inlineStr">
+      <c r="H240" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I240" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3JL</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I239"/>
+  <autoFilter ref="A1:I240"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I2" r:id="rId2"/>
@@ -11478,6 +11521,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I238" r:id="rId474"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A239" r:id="rId475"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I239" r:id="rId476"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A240" r:id="rId477"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I240" r:id="rId478"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update course plans and analysis files across multiple departments
- Updated the last scrape date in Dalarna Dashboard to 2026-08-29.
- Modified the download link for Vilande kursplaner to reflect the updated row count (241).
- Added new course entries and updated existing ones in various course plan markdown files.
- Updated multiple Excel analysis files for IIT, IHV, IKS, and ISLL departments to reflect recent changes.
- Marked specific courses as "vilande" in their respective metadata.
</commit_message>
<xml_diff>
--- a/vault-dalarna-university/02 IHV/Analys/Vilande kursplaner.xlsx
+++ b/vault-dalarna-university/02 IHV/Analys/Vilande kursplaner.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Vilande kursplaner" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Vilande kursplaner'!$A$1:$I$240</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Vilande kursplaner'!$A$1:$I$242</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I240"/>
+  <dimension ref="A1:I242"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6165,7 +6165,7 @@
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
         <is>
-          <t>ASR25U</t>
+          <t>ASR25T</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -6195,7 +6195,7 @@
       </c>
       <c r="G129" t="inlineStr">
         <is>
-          <t>Ledarskap och organisation inom hälso- och sjukvårdssystem</t>
+          <t>Hälso- och sjukvårdssystemforskning i låg-, medel- och höginkomstkontext</t>
         </is>
       </c>
       <c r="H129" t="inlineStr">
@@ -6205,14 +6205,14 @@
       </c>
       <c r="I129" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR25U</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR25T</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
         <is>
-          <t>ASR25V</t>
+          <t>ASR25U</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -6242,7 +6242,7 @@
       </c>
       <c r="G130" t="inlineStr">
         <is>
-          <t>Examensarbete i sexuell, reproduktiv och perinatal hälsa</t>
+          <t>Ledarskap och organisation inom hälso- och sjukvårdssystem</t>
         </is>
       </c>
       <c r="H130" t="inlineStr">
@@ -6252,19 +6252,19 @@
       </c>
       <c r="I130" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR25V</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR25U</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
         <is>
-          <t>GVÅ2HM</t>
+          <t>ASR25V</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>OMV</t>
+          <t>SRP</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
@@ -6274,22 +6274,22 @@
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>2020-08-27</t>
+          <t>2020-06-17</t>
         </is>
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>2020-09-10</t>
+          <t>2020-06-25</t>
         </is>
       </c>
       <c r="F131" t="inlineStr">
         <is>
-          <t>Omvårdnad</t>
+          <t>Sexuell, reproduktiv och perinatal hälsa</t>
         </is>
       </c>
       <c r="G131" t="inlineStr">
         <is>
-          <t>Personcentrerad vård inom psykiatrisk vård</t>
+          <t>Examensarbete i sexuell, reproduktiv och perinatal hälsa</t>
         </is>
       </c>
       <c r="H131" t="inlineStr">
@@ -6299,19 +6299,19 @@
       </c>
       <c r="I131" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GVÅ2HM</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR25V</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
         <is>
-          <t>AMC265</t>
+          <t>GVÅ2HM</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>MCA</t>
+          <t>OMV</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
@@ -6321,22 +6321,22 @@
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>2020-09-24</t>
+          <t>2020-08-27</t>
         </is>
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>2020-10-01</t>
+          <t>2020-09-10</t>
         </is>
       </c>
       <c r="F132" t="inlineStr">
         <is>
-          <t>Medicinsk vetenskap</t>
+          <t>Omvårdnad</t>
         </is>
       </c>
       <c r="G132" t="inlineStr">
         <is>
-          <t>Farmakologisk behandling vid diabetes</t>
+          <t>Personcentrerad vård inom psykiatrisk vård</t>
         </is>
       </c>
       <c r="H132" t="inlineStr">
@@ -6346,19 +6346,19 @@
       </c>
       <c r="I132" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMC265</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GVÅ2HM</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
         <is>
-          <t>GNV2KY</t>
+          <t>AMC265</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>NAV</t>
+          <t>MCA</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
@@ -6368,18 +6368,22 @@
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>2020-11-26</t>
-        </is>
-      </c>
-      <c r="E133" t="inlineStr"/>
+          <t>2020-09-24</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>2020-10-01</t>
+        </is>
+      </c>
       <c r="F133" t="inlineStr">
         <is>
-          <t>Naturvetenskap</t>
+          <t>Medicinsk vetenskap</t>
         </is>
       </c>
       <c r="G133" t="inlineStr">
         <is>
-          <t>Naturvetenskap och teknik i förskolan - med didaktisk inriktning</t>
+          <t>Farmakologisk behandling vid diabetes</t>
         </is>
       </c>
       <c r="H133" t="inlineStr">
@@ -6389,19 +6393,19 @@
       </c>
       <c r="I133" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GNV2KY</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMC265</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
         <is>
-          <t>GSR2KZ</t>
+          <t>GNV2KY</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>SRP</t>
+          <t>NAV</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
@@ -6414,19 +6418,15 @@
           <t>2020-11-26</t>
         </is>
       </c>
-      <c r="E134" t="inlineStr">
-        <is>
-          <t>2020-12-10</t>
-        </is>
-      </c>
+      <c r="E134" t="inlineStr"/>
       <c r="F134" t="inlineStr">
         <is>
-          <t>Sexuell, reproduktiv och perinatal hälsa</t>
+          <t>Naturvetenskap</t>
         </is>
       </c>
       <c r="G134" t="inlineStr">
         <is>
-          <t>Människa, hälsa, hållbarhet i ett mångkulturellt samhälle</t>
+          <t>Naturvetenskap och teknik i förskolan - med didaktisk inriktning</t>
         </is>
       </c>
       <c r="H134" t="inlineStr">
@@ -6436,19 +6436,19 @@
       </c>
       <c r="I134" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSR2KZ</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GNV2KY</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
         <is>
-          <t>GIH2LT</t>
+          <t>GSR2KZ</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>IDA</t>
+          <t>SRP</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
@@ -6458,18 +6458,22 @@
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>2021-02-04</t>
-        </is>
-      </c>
-      <c r="E135" t="inlineStr"/>
+          <t>2020-11-26</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>2020-12-10</t>
+        </is>
+      </c>
       <c r="F135" t="inlineStr">
         <is>
-          <t>Idrotts- och hälsovetenskap</t>
+          <t>Sexuell, reproduktiv och perinatal hälsa</t>
         </is>
       </c>
       <c r="G135" t="inlineStr">
         <is>
-          <t>Idrottspedagogik (judo)</t>
+          <t>Människa, hälsa, hållbarhet i ett mångkulturellt samhälle</t>
         </is>
       </c>
       <c r="H135" t="inlineStr">
@@ -6479,14 +6483,14 @@
       </c>
       <c r="I135" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2LT</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSR2KZ</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
         <is>
-          <t>GIH2LU</t>
+          <t>GIH2LT</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -6512,7 +6516,7 @@
       </c>
       <c r="G136" t="inlineStr">
         <is>
-          <t>Idrottspedagogik (styrkelyft)</t>
+          <t>Idrottspedagogik (judo)</t>
         </is>
       </c>
       <c r="H136" t="inlineStr">
@@ -6522,14 +6526,14 @@
       </c>
       <c r="I136" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2LU</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2LT</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
         <is>
-          <t>GIH2LW</t>
+          <t>GIH2LU</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -6555,7 +6559,7 @@
       </c>
       <c r="G137" t="inlineStr">
         <is>
-          <t>Tränings- och tävlingslära (styrkelyft)</t>
+          <t>Idrottspedagogik (styrkelyft)</t>
         </is>
       </c>
       <c r="H137" t="inlineStr">
@@ -6565,14 +6569,14 @@
       </c>
       <c r="I137" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2LW</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2LU</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
         <is>
-          <t>GIH2LX</t>
+          <t>GIH2LW</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
@@ -6598,7 +6602,7 @@
       </c>
       <c r="G138" t="inlineStr">
         <is>
-          <t>Motorisk kontroll och lärande (judo)</t>
+          <t>Tränings- och tävlingslära (styrkelyft)</t>
         </is>
       </c>
       <c r="H138" t="inlineStr">
@@ -6608,14 +6612,14 @@
       </c>
       <c r="I138" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2LX</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2LW</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
         <is>
-          <t>GIH2M4</t>
+          <t>GIH2LX</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
@@ -6630,7 +6634,7 @@
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>2021-02-10</t>
+          <t>2021-02-04</t>
         </is>
       </c>
       <c r="E139" t="inlineStr"/>
@@ -6641,7 +6645,7 @@
       </c>
       <c r="G139" t="inlineStr">
         <is>
-          <t>Motorisk kontroll och lärande (Klättring)</t>
+          <t>Motorisk kontroll och lärande (judo)</t>
         </is>
       </c>
       <c r="H139" t="inlineStr">
@@ -6651,14 +6655,14 @@
       </c>
       <c r="I139" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2M4</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2LX</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
         <is>
-          <t>GIH2M5</t>
+          <t>GIH2M4</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
@@ -6684,7 +6688,7 @@
       </c>
       <c r="G140" t="inlineStr">
         <is>
-          <t>Tränings- och tävlingslära (Klättring)</t>
+          <t>Motorisk kontroll och lärande (Klättring)</t>
         </is>
       </c>
       <c r="H140" t="inlineStr">
@@ -6694,14 +6698,14 @@
       </c>
       <c r="I140" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2M5</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2M4</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
         <is>
-          <t>GIH2M6</t>
+          <t>GIH2M5</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
@@ -6727,7 +6731,7 @@
       </c>
       <c r="G141" t="inlineStr">
         <is>
-          <t>Idrottspedagogik (klättring)</t>
+          <t>Tränings- och tävlingslära (Klättring)</t>
         </is>
       </c>
       <c r="H141" t="inlineStr">
@@ -6737,14 +6741,14 @@
       </c>
       <c r="I141" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2M6</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2M5</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
         <is>
-          <t>GIH2LV</t>
+          <t>GIH2M6</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
@@ -6759,14 +6763,10 @@
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>2021-02-04</t>
-        </is>
-      </c>
-      <c r="E142" t="inlineStr">
-        <is>
-          <t>2021-02-15</t>
-        </is>
-      </c>
+          <t>2021-02-10</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr"/>
       <c r="F142" t="inlineStr">
         <is>
           <t>Idrotts- och hälsovetenskap</t>
@@ -6774,7 +6774,7 @@
       </c>
       <c r="G142" t="inlineStr">
         <is>
-          <t>Tränings- och tävlingslära (judo)</t>
+          <t>Idrottspedagogik (klättring)</t>
         </is>
       </c>
       <c r="H142" t="inlineStr">
@@ -6784,14 +6784,14 @@
       </c>
       <c r="I142" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2LV</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2M6</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
         <is>
-          <t>GIH2LY</t>
+          <t>GIH2LV</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -6821,7 +6821,7 @@
       </c>
       <c r="G143" t="inlineStr">
         <is>
-          <t>Motorisk kontroll och lärande (styrkelyft)</t>
+          <t>Tränings- och tävlingslära (judo)</t>
         </is>
       </c>
       <c r="H143" t="inlineStr">
@@ -6831,19 +6831,19 @@
       </c>
       <c r="I143" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2LY</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2LV</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
         <is>
-          <t>GSR2A5</t>
+          <t>GIH2LY</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>SRP</t>
+          <t>IDA</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
@@ -6853,22 +6853,22 @@
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>2019-06-19</t>
+          <t>2021-02-04</t>
         </is>
       </c>
       <c r="E144" t="inlineStr">
         <is>
-          <t>2021-02-19</t>
+          <t>2021-02-15</t>
         </is>
       </c>
       <c r="F144" t="inlineStr">
         <is>
-          <t>Sexuell, reproduktiv och perinatal hälsa</t>
+          <t>Idrotts- och hälsovetenskap</t>
         </is>
       </c>
       <c r="G144" t="inlineStr">
         <is>
-          <t>Ungdomar och unga vuxnas reproduktiva hälsa och rättigheter I</t>
+          <t>Motorisk kontroll och lärande (styrkelyft)</t>
         </is>
       </c>
       <c r="H144" t="inlineStr">
@@ -6878,19 +6878,19 @@
       </c>
       <c r="I144" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSR2A5</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2LY</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
         <is>
-          <t>AVV26K</t>
+          <t>GSR2A5</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>VÅE</t>
+          <t>SRP</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
@@ -6900,22 +6900,22 @@
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>2021-02-24</t>
+          <t>2019-06-19</t>
         </is>
       </c>
       <c r="E145" t="inlineStr">
         <is>
-          <t>2021-03-02</t>
+          <t>2021-02-19</t>
         </is>
       </c>
       <c r="F145" t="inlineStr">
         <is>
-          <t>Vårdvetenskap</t>
+          <t>Sexuell, reproduktiv och perinatal hälsa</t>
         </is>
       </c>
       <c r="G145" t="inlineStr">
         <is>
-          <t>Säker hälso- och sjukvård samt vård och omsorg - komplexa system och förbättringskunskap</t>
+          <t>Ungdomar och unga vuxnas reproduktiva hälsa och rättigheter I</t>
         </is>
       </c>
       <c r="H145" t="inlineStr">
@@ -6925,14 +6925,14 @@
       </c>
       <c r="I145" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AVV26K</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSR2A5</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
         <is>
-          <t>AVV26M</t>
+          <t>AVV26K</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
@@ -6962,7 +6962,7 @@
       </c>
       <c r="G146" t="inlineStr">
         <is>
-          <t>Implementering av nya arbetssätt i hälso- och sjukvården och socialtjänstens områden</t>
+          <t>Säker hälso- och sjukvård samt vård och omsorg - komplexa system och förbättringskunskap</t>
         </is>
       </c>
       <c r="H146" t="inlineStr">
@@ -6972,19 +6972,19 @@
       </c>
       <c r="I146" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AVV26M</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AVV26K</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
         <is>
-          <t>ASR26N</t>
+          <t>AVV26M</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>SRP</t>
+          <t>VÅE</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
@@ -6994,22 +6994,22 @@
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>2021-03-01</t>
+          <t>2021-02-24</t>
         </is>
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>2021-03-03</t>
+          <t>2021-03-02</t>
         </is>
       </c>
       <c r="F147" t="inlineStr">
         <is>
-          <t>Sexuell, reproduktiv och perinatal hälsa</t>
+          <t>Vårdvetenskap</t>
         </is>
       </c>
       <c r="G147" t="inlineStr">
         <is>
-          <t>Konstruktiv länkning av utbildnings- och kursplaner, läraktiviteter och examinationsformer för lärare i högre utbildning</t>
+          <t>Implementering av nya arbetssätt i hälso- och sjukvården och socialtjänstens områden</t>
         </is>
       </c>
       <c r="H147" t="inlineStr">
@@ -7019,14 +7019,14 @@
       </c>
       <c r="I147" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR26N</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AVV26M</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
         <is>
-          <t>ASR26S</t>
+          <t>ASR26N</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
@@ -7041,10 +7041,14 @@
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>2021-03-08</t>
-        </is>
-      </c>
-      <c r="E148" t="inlineStr"/>
+          <t>2021-03-01</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>2021-03-03</t>
+        </is>
+      </c>
       <c r="F148" t="inlineStr">
         <is>
           <t>Sexuell, reproduktiv och perinatal hälsa</t>
@@ -7052,7 +7056,7 @@
       </c>
       <c r="G148" t="inlineStr">
         <is>
-          <t>Graviditet, förlossning och postpartumvård II</t>
+          <t>Konstruktiv länkning av utbildnings- och kursplaner, läraktiviteter och examinationsformer för lärare i högre utbildning</t>
         </is>
       </c>
       <c r="H148" t="inlineStr">
@@ -7062,19 +7066,19 @@
       </c>
       <c r="I148" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR26S</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR26N</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
         <is>
-          <t>GSA2NC</t>
+          <t>ASR26S</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>SAA</t>
+          <t>SRP</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
@@ -7084,18 +7088,18 @@
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>2021-03-09</t>
+          <t>2021-03-08</t>
         </is>
       </c>
       <c r="E149" t="inlineStr"/>
       <c r="F149" t="inlineStr">
         <is>
-          <t>Socialt arbete</t>
+          <t>Sexuell, reproduktiv och perinatal hälsa</t>
         </is>
       </c>
       <c r="G149" t="inlineStr">
         <is>
-          <t>Organisation, grupp och samverkan</t>
+          <t>Graviditet, förlossning och postpartumvård II</t>
         </is>
       </c>
       <c r="H149" t="inlineStr">
@@ -7105,19 +7109,19 @@
       </c>
       <c r="I149" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA2NC</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR26S</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
         <is>
-          <t>GIH2NR</t>
+          <t>GSA2NC</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>IDA</t>
+          <t>SAA</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
@@ -7127,18 +7131,18 @@
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>2021-03-12</t>
+          <t>2021-03-09</t>
         </is>
       </c>
       <c r="E150" t="inlineStr"/>
       <c r="F150" t="inlineStr">
         <is>
-          <t>Idrotts- och hälsovetenskap</t>
+          <t>Socialt arbete</t>
         </is>
       </c>
       <c r="G150" t="inlineStr">
         <is>
-          <t>Grundläggande funktionell anatomi, biomekanik och rörelseanalys</t>
+          <t>Organisation, grupp och samverkan</t>
         </is>
       </c>
       <c r="H150" t="inlineStr">
@@ -7148,14 +7152,14 @@
       </c>
       <c r="I150" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2NR</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA2NC</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
         <is>
-          <t>GIH2QK</t>
+          <t>GIH2NR</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
@@ -7170,7 +7174,7 @@
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>2021-06-07</t>
+          <t>2021-03-12</t>
         </is>
       </c>
       <c r="E151" t="inlineStr"/>
@@ -7181,7 +7185,7 @@
       </c>
       <c r="G151" t="inlineStr">
         <is>
-          <t>Tillämpad anatomi och idrottsfysiologi</t>
+          <t>Grundläggande funktionell anatomi, biomekanik och rörelseanalys</t>
         </is>
       </c>
       <c r="H151" t="inlineStr">
@@ -7191,14 +7195,14 @@
       </c>
       <c r="I151" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2QK</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2NR</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
         <is>
-          <t>GIH2QL</t>
+          <t>GIH2QK</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -7224,7 +7228,7 @@
       </c>
       <c r="G152" t="inlineStr">
         <is>
-          <t>Motorisk kontroll, lärande och utveckling med didaktisk inriktning</t>
+          <t>Tillämpad anatomi och idrottsfysiologi</t>
         </is>
       </c>
       <c r="H152" t="inlineStr">
@@ -7234,19 +7238,19 @@
       </c>
       <c r="I152" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2QL</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2QK</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
         <is>
-          <t>GMC2M2</t>
+          <t>GIH2QL</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>MCA</t>
+          <t>IDA</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
@@ -7256,22 +7260,18 @@
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>2021-02-09</t>
-        </is>
-      </c>
-      <c r="E153" t="inlineStr">
-        <is>
-          <t>2021-06-24</t>
-        </is>
-      </c>
+          <t>2021-06-07</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr"/>
       <c r="F153" t="inlineStr">
         <is>
-          <t>Medicinsk vetenskap</t>
+          <t>Idrotts- och hälsovetenskap</t>
         </is>
       </c>
       <c r="G153" t="inlineStr">
         <is>
-          <t>Anatomi och fysiologi II</t>
+          <t>Motorisk kontroll, lärande och utveckling med didaktisk inriktning</t>
         </is>
       </c>
       <c r="H153" t="inlineStr">
@@ -7281,19 +7281,19 @@
       </c>
       <c r="I153" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMC2M2</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2QL</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
         <is>
-          <t>GVÅ2R2</t>
+          <t>GMC2M2</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>OMV</t>
+          <t>MCA</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
@@ -7303,18 +7303,22 @@
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>2021-08-27</t>
-        </is>
-      </c>
-      <c r="E154" t="inlineStr"/>
+          <t>2021-02-09</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>2021-06-24</t>
+        </is>
+      </c>
       <c r="F154" t="inlineStr">
         <is>
-          <t>Omvårdnad</t>
+          <t>Medicinsk vetenskap</t>
         </is>
       </c>
       <c r="G154" t="inlineStr">
         <is>
-          <t>Personcentrerad vård för personer med demens</t>
+          <t>Anatomi och fysiologi II</t>
         </is>
       </c>
       <c r="H154" t="inlineStr">
@@ -7324,14 +7328,14 @@
       </c>
       <c r="I154" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GVÅ2R2</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMC2M2</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
         <is>
-          <t>GVÅ2RA</t>
+          <t>GVÅ2R2</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
@@ -7346,7 +7350,7 @@
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>2021-09-07</t>
+          <t>2021-08-27</t>
         </is>
       </c>
       <c r="E155" t="inlineStr"/>
@@ -7357,7 +7361,7 @@
       </c>
       <c r="G155" t="inlineStr">
         <is>
-          <t>Människans grundläggande omvårdnadsbehov</t>
+          <t>Personcentrerad vård för personer med demens</t>
         </is>
       </c>
       <c r="H155" t="inlineStr">
@@ -7367,14 +7371,14 @@
       </c>
       <c r="I155" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GVÅ2RA</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GVÅ2R2</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
         <is>
-          <t>GVÅ2RT</t>
+          <t>GVÅ2RA</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
@@ -7389,7 +7393,7 @@
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>2021-09-30</t>
+          <t>2021-09-07</t>
         </is>
       </c>
       <c r="E156" t="inlineStr"/>
@@ -7400,7 +7404,7 @@
       </c>
       <c r="G156" t="inlineStr">
         <is>
-          <t>Vård och omsorg för personer med demens</t>
+          <t>Människans grundläggande omvårdnadsbehov</t>
         </is>
       </c>
       <c r="H156" t="inlineStr">
@@ -7410,14 +7414,14 @@
       </c>
       <c r="I156" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GVÅ2RT</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GVÅ2RA</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
         <is>
-          <t>GVÅ2RU</t>
+          <t>GVÅ2RT</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
@@ -7443,7 +7447,7 @@
       </c>
       <c r="G157" t="inlineStr">
         <is>
-          <t>Aktivitet och ätande vid demenssjukdom</t>
+          <t>Vård och omsorg för personer med demens</t>
         </is>
       </c>
       <c r="H157" t="inlineStr">
@@ -7453,14 +7457,14 @@
       </c>
       <c r="I157" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GVÅ2RU</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GVÅ2RT</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
         <is>
-          <t>GVÅ2RV</t>
+          <t>GVÅ2RU</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
@@ -7486,7 +7490,7 @@
       </c>
       <c r="G158" t="inlineStr">
         <is>
-          <t>Demenssjukdomar, diagnostik och behandling ur ett omvårdnadsperspektiv</t>
+          <t>Aktivitet och ätande vid demenssjukdom</t>
         </is>
       </c>
       <c r="H158" t="inlineStr">
@@ -7496,19 +7500,19 @@
       </c>
       <c r="I158" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GVÅ2RV</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GVÅ2RU</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
         <is>
-          <t>ASA27E</t>
+          <t>GVÅ2RV</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>SAA</t>
+          <t>OMV</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
@@ -7518,18 +7522,18 @@
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>2021-11-09</t>
+          <t>2021-09-30</t>
         </is>
       </c>
       <c r="E159" t="inlineStr"/>
       <c r="F159" t="inlineStr">
         <is>
-          <t>Socialt arbete</t>
+          <t>Omvårdnad</t>
         </is>
       </c>
       <c r="G159" t="inlineStr">
         <is>
-          <t>Socialt arbete i skolan - skolan som en arena för stöd och utveckling</t>
+          <t>Demenssjukdomar, diagnostik och behandling ur ett omvårdnadsperspektiv</t>
         </is>
       </c>
       <c r="H159" t="inlineStr">
@@ -7539,19 +7543,19 @@
       </c>
       <c r="I159" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASA27E</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GVÅ2RV</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
         <is>
-          <t>AVÅ27J</t>
+          <t>ASA27E</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>OMV</t>
+          <t>SAA</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
@@ -7561,18 +7565,18 @@
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>2021-12-08</t>
+          <t>2021-11-09</t>
         </is>
       </c>
       <c r="E160" t="inlineStr"/>
       <c r="F160" t="inlineStr">
         <is>
-          <t>Omvårdnad</t>
+          <t>Socialt arbete</t>
         </is>
       </c>
       <c r="G160" t="inlineStr">
         <is>
-          <t>Personcentrerad vård för personer med demens (fristående kurs)</t>
+          <t>Socialt arbete i skolan - skolan som en arena för stöd och utveckling</t>
         </is>
       </c>
       <c r="H160" t="inlineStr">
@@ -7582,14 +7586,14 @@
       </c>
       <c r="I160" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AVÅ27J</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASA27E</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
         <is>
-          <t>AVÅ27K</t>
+          <t>AVÅ27J</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
@@ -7615,7 +7619,7 @@
       </c>
       <c r="G161" t="inlineStr">
         <is>
-          <t>Demenssjukdomar, diagnostik och behandling ur ett omvårdnadsperspektiv (fristående kurs)</t>
+          <t>Personcentrerad vård för personer med demens (fristående kurs)</t>
         </is>
       </c>
       <c r="H161" t="inlineStr">
@@ -7625,14 +7629,14 @@
       </c>
       <c r="I161" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AVÅ27K</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AVÅ27J</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
         <is>
-          <t>AVÅ27L</t>
+          <t>AVÅ27K</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
@@ -7658,7 +7662,7 @@
       </c>
       <c r="G162" t="inlineStr">
         <is>
-          <t>Vård och omsorg för personer med demens (fristående kurs)</t>
+          <t>Demenssjukdomar, diagnostik och behandling ur ett omvårdnadsperspektiv (fristående kurs)</t>
         </is>
       </c>
       <c r="H162" t="inlineStr">
@@ -7668,19 +7672,19 @@
       </c>
       <c r="I162" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AVÅ27L</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AVÅ27K</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
         <is>
-          <t>GIH2UR</t>
+          <t>AVÅ27L</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>IDA</t>
+          <t>OMV</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
@@ -7690,18 +7694,18 @@
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>2022-02-24</t>
+          <t>2021-12-08</t>
         </is>
       </c>
       <c r="E163" t="inlineStr"/>
       <c r="F163" t="inlineStr">
         <is>
-          <t>Idrotts- och hälsovetenskap</t>
+          <t>Omvårdnad</t>
         </is>
       </c>
       <c r="G163" t="inlineStr">
         <is>
-          <t>Grundläggande vetenskaplig metod</t>
+          <t>Vård och omsorg för personer med demens (fristående kurs)</t>
         </is>
       </c>
       <c r="H163" t="inlineStr">
@@ -7711,19 +7715,19 @@
       </c>
       <c r="I163" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2UR</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AVÅ27L</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
         <is>
-          <t>AVÅ27S</t>
+          <t>GIH2UR</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>OMV</t>
+          <t>IDA</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
@@ -7739,12 +7743,12 @@
       <c r="E164" t="inlineStr"/>
       <c r="F164" t="inlineStr">
         <is>
-          <t>Omvårdnad</t>
+          <t>Idrotts- och hälsovetenskap</t>
         </is>
       </c>
       <c r="G164" t="inlineStr">
         <is>
-          <t>Bedömning och rådgivning vid distanskontakter inom hälso- och sjukvården</t>
+          <t>Grundläggande vetenskaplig metod</t>
         </is>
       </c>
       <c r="H164" t="inlineStr">
@@ -7754,19 +7758,19 @@
       </c>
       <c r="I164" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AVÅ27S</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2UR</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
         <is>
-          <t>GIH2UY</t>
+          <t>AVÅ27S</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>IDA</t>
+          <t>OMV</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
@@ -7776,18 +7780,18 @@
       </c>
       <c r="D165" t="inlineStr">
         <is>
-          <t>2022-02-28</t>
+          <t>2022-02-24</t>
         </is>
       </c>
       <c r="E165" t="inlineStr"/>
       <c r="F165" t="inlineStr">
         <is>
-          <t>Idrotts- och hälsovetenskap</t>
+          <t>Omvårdnad</t>
         </is>
       </c>
       <c r="G165" t="inlineStr">
         <is>
-          <t>Näringslära med inriktning mot idrott och fysisk aktivitet</t>
+          <t>Bedömning och rådgivning vid distanskontakter inom hälso- och sjukvården</t>
         </is>
       </c>
       <c r="H165" t="inlineStr">
@@ -7797,14 +7801,14 @@
       </c>
       <c r="I165" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2UY</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AVÅ27S</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" s="2" t="inlineStr">
         <is>
-          <t>GIH2VJ</t>
+          <t>GIH2UY</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
@@ -7819,7 +7823,7 @@
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>2022-03-03</t>
+          <t>2022-02-28</t>
         </is>
       </c>
       <c r="E166" t="inlineStr"/>
@@ -7830,7 +7834,7 @@
       </c>
       <c r="G166" t="inlineStr">
         <is>
-          <t>Idrottsmedicin</t>
+          <t>Näringslära med inriktning mot idrott och fysisk aktivitet</t>
         </is>
       </c>
       <c r="H166" t="inlineStr">
@@ -7840,14 +7844,14 @@
       </c>
       <c r="I166" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2VJ</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2UY</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" s="2" t="inlineStr">
         <is>
-          <t>GIH2VK</t>
+          <t>GIH2VJ</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
@@ -7873,7 +7877,7 @@
       </c>
       <c r="G167" t="inlineStr">
         <is>
-          <t>Grundläggande upplevelseproduktion</t>
+          <t>Idrottsmedicin</t>
         </is>
       </c>
       <c r="H167" t="inlineStr">
@@ -7883,19 +7887,19 @@
       </c>
       <c r="I167" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2VK</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2VJ</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" s="2" t="inlineStr">
         <is>
-          <t>GVÅ2VZ</t>
+          <t>GIH2VK</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>OMV</t>
+          <t>IDA</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
@@ -7905,18 +7909,18 @@
       </c>
       <c r="D168" t="inlineStr">
         <is>
-          <t>2022-04-13</t>
+          <t>2022-03-03</t>
         </is>
       </c>
       <c r="E168" t="inlineStr"/>
       <c r="F168" t="inlineStr">
         <is>
-          <t>Omvårdnad</t>
+          <t>Idrotts- och hälsovetenskap</t>
         </is>
       </c>
       <c r="G168" t="inlineStr">
         <is>
-          <t>Palliativ och evidensbaserad omvårdnad för personer med demens</t>
+          <t>Grundläggande upplevelseproduktion</t>
         </is>
       </c>
       <c r="H168" t="inlineStr">
@@ -7926,19 +7930,19 @@
       </c>
       <c r="I168" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GVÅ2VZ</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2VK</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" s="2" t="inlineStr">
         <is>
-          <t>GIH2WT</t>
+          <t>GVÅ2VZ</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>IDA</t>
+          <t>OMV</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
@@ -7948,18 +7952,18 @@
       </c>
       <c r="D169" t="inlineStr">
         <is>
-          <t>2022-06-16</t>
+          <t>2022-04-13</t>
         </is>
       </c>
       <c r="E169" t="inlineStr"/>
       <c r="F169" t="inlineStr">
         <is>
-          <t>Idrotts- och hälsovetenskap</t>
+          <t>Omvårdnad</t>
         </is>
       </c>
       <c r="G169" t="inlineStr">
         <is>
-          <t>Fotbollstränare - inriktning barn och ungdom (6-15 år)</t>
+          <t>Palliativ och evidensbaserad omvårdnad för personer med demens</t>
         </is>
       </c>
       <c r="H169" t="inlineStr">
@@ -7969,14 +7973,14 @@
       </c>
       <c r="I169" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2WT</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GVÅ2VZ</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" s="2" t="inlineStr">
         <is>
-          <t>GIH2WX</t>
+          <t>GIH2WT</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
@@ -8002,7 +8006,7 @@
       </c>
       <c r="G170" t="inlineStr">
         <is>
-          <t>Idrotten i samhället (VAL)</t>
+          <t>Fotbollstränare - inriktning barn och ungdom (6-15 år)</t>
         </is>
       </c>
       <c r="H170" t="inlineStr">
@@ -8012,14 +8016,14 @@
       </c>
       <c r="I170" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2WX</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2WT</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" s="2" t="inlineStr">
         <is>
-          <t>GIH2WY</t>
+          <t>GIH2WX</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
@@ -8045,7 +8049,7 @@
       </c>
       <c r="G171" t="inlineStr">
         <is>
-          <t>Friluftsliv i närmiljön: orientering, vandring, paddling (VAL)</t>
+          <t>Idrotten i samhället (VAL)</t>
         </is>
       </c>
       <c r="H171" t="inlineStr">
@@ -8055,19 +8059,19 @@
       </c>
       <c r="I171" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2WY</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2WX</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" s="2" t="inlineStr">
         <is>
-          <t>GVÅ2WS</t>
+          <t>GIH2WY</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>OMV</t>
+          <t>IDA</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
@@ -8083,12 +8087,12 @@
       <c r="E172" t="inlineStr"/>
       <c r="F172" t="inlineStr">
         <is>
-          <t>Omvårdnad</t>
+          <t>Idrotts- och hälsovetenskap</t>
         </is>
       </c>
       <c r="G172" t="inlineStr">
         <is>
-          <t>Global hälsa</t>
+          <t>Friluftsliv i närmiljön: orientering, vandring, paddling (VAL)</t>
         </is>
       </c>
       <c r="H172" t="inlineStr">
@@ -8098,19 +8102,19 @@
       </c>
       <c r="I172" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GVÅ2WS</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2WY</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" s="2" t="inlineStr">
         <is>
-          <t>ASR284</t>
+          <t>GVÅ2WS</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>SRP</t>
+          <t>OMV</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
@@ -8126,12 +8130,12 @@
       <c r="E173" t="inlineStr"/>
       <c r="F173" t="inlineStr">
         <is>
-          <t>Sexuell, reproduktiv och perinatal hälsa</t>
+          <t>Omvårdnad</t>
         </is>
       </c>
       <c r="G173" t="inlineStr">
         <is>
-          <t>Förlossningsvård I, verksamhetsförlagd utbildning</t>
+          <t>Global hälsa</t>
         </is>
       </c>
       <c r="H173" t="inlineStr">
@@ -8141,14 +8145,14 @@
       </c>
       <c r="I173" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR284</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GVÅ2WS</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" s="2" t="inlineStr">
         <is>
-          <t>ASR285</t>
+          <t>ASR284</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
@@ -8174,7 +8178,7 @@
       </c>
       <c r="G174" t="inlineStr">
         <is>
-          <t>Gynekologisk vård och postpartumvård, verksamhetsförlagd utbildning</t>
+          <t>Förlossningsvård I, verksamhetsförlagd utbildning</t>
         </is>
       </c>
       <c r="H174" t="inlineStr">
@@ -8184,14 +8188,14 @@
       </c>
       <c r="I174" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR285</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR284</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" s="2" t="inlineStr">
         <is>
-          <t>ASR286</t>
+          <t>ASR285</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
@@ -8217,7 +8221,7 @@
       </c>
       <c r="G175" t="inlineStr">
         <is>
-          <t>Examensarbete i sexuell, reproduktiv och perinatal hälsa</t>
+          <t>Gynekologisk vård och postpartumvård, verksamhetsförlagd utbildning</t>
         </is>
       </c>
       <c r="H175" t="inlineStr">
@@ -8227,19 +8231,19 @@
       </c>
       <c r="I175" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR286</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR285</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" s="2" t="inlineStr">
         <is>
-          <t>GIH2X3</t>
+          <t>ASR286</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>IDA</t>
+          <t>SRP</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
@@ -8252,19 +8256,15 @@
           <t>2022-06-16</t>
         </is>
       </c>
-      <c r="E176" t="inlineStr">
-        <is>
-          <t>2022-08-22</t>
-        </is>
-      </c>
+      <c r="E176" t="inlineStr"/>
       <c r="F176" t="inlineStr">
         <is>
-          <t>Idrotts- och hälsovetenskap</t>
+          <t>Sexuell, reproduktiv och perinatal hälsa</t>
         </is>
       </c>
       <c r="G176" t="inlineStr">
         <is>
-          <t>Träningslära för tävlingsinriktad idrott</t>
+          <t>Examensarbete i sexuell, reproduktiv och perinatal hälsa</t>
         </is>
       </c>
       <c r="H176" t="inlineStr">
@@ -8274,19 +8274,19 @@
       </c>
       <c r="I176" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2X3</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR286</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" s="2" t="inlineStr">
         <is>
-          <t>AMC288</t>
+          <t>GIH2X3</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>MCA</t>
+          <t>IDA</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
@@ -8296,18 +8296,22 @@
       </c>
       <c r="D177" t="inlineStr">
         <is>
-          <t>2022-09-08</t>
-        </is>
-      </c>
-      <c r="E177" t="inlineStr"/>
+          <t>2022-06-16</t>
+        </is>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>2022-08-22</t>
+        </is>
+      </c>
       <c r="F177" t="inlineStr">
         <is>
-          <t>Medicinsk vetenskap</t>
+          <t>Idrotts- och hälsovetenskap</t>
         </is>
       </c>
       <c r="G177" t="inlineStr">
         <is>
-          <t>Fysisk aktivitet och träning som prevention och behandling</t>
+          <t>Träningslära för tävlingsinriktad idrott</t>
         </is>
       </c>
       <c r="H177" t="inlineStr">
@@ -8317,19 +8321,19 @@
       </c>
       <c r="I177" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMC288</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2X3</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" s="2" t="inlineStr">
         <is>
-          <t>GSA2XN</t>
+          <t>AMC288</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>SAA</t>
+          <t>MCA</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
@@ -8345,12 +8349,12 @@
       <c r="E178" t="inlineStr"/>
       <c r="F178" t="inlineStr">
         <is>
-          <t>Socialt arbete</t>
+          <t>Medicinsk vetenskap</t>
         </is>
       </c>
       <c r="G178" t="inlineStr">
         <is>
-          <t>Missbruk och beroende</t>
+          <t>Fysisk aktivitet och träning som prevention och behandling</t>
         </is>
       </c>
       <c r="H178" t="inlineStr">
@@ -8360,19 +8364,19 @@
       </c>
       <c r="I178" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA2XN</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMC288</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" s="2" t="inlineStr">
         <is>
-          <t>GIH2XY</t>
+          <t>GSA2XN</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>IDA</t>
+          <t>SAA</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
@@ -8382,22 +8386,18 @@
       </c>
       <c r="D179" t="inlineStr">
         <is>
-          <t>2022-09-26</t>
-        </is>
-      </c>
-      <c r="E179" t="inlineStr">
-        <is>
-          <t>2022-09-30</t>
-        </is>
-      </c>
+          <t>2022-09-08</t>
+        </is>
+      </c>
+      <c r="E179" t="inlineStr"/>
       <c r="F179" t="inlineStr">
         <is>
-          <t>Idrotts- och hälsovetenskap</t>
+          <t>Socialt arbete</t>
         </is>
       </c>
       <c r="G179" t="inlineStr">
         <is>
-          <t>Idrottsvetenskaplig uppsats</t>
+          <t>Missbruk och beroende</t>
         </is>
       </c>
       <c r="H179" t="inlineStr">
@@ -8407,19 +8407,19 @@
       </c>
       <c r="I179" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2XY</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA2XN</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" s="2" t="inlineStr">
         <is>
-          <t>AVÅ28C</t>
+          <t>GIH2XY</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>OMV</t>
+          <t>IDA</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
@@ -8429,18 +8429,22 @@
       </c>
       <c r="D180" t="inlineStr">
         <is>
-          <t>2022-11-14</t>
-        </is>
-      </c>
-      <c r="E180" t="inlineStr"/>
+          <t>2022-09-26</t>
+        </is>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>2022-09-30</t>
+        </is>
+      </c>
       <c r="F180" t="inlineStr">
         <is>
-          <t>Omvårdnad</t>
+          <t>Idrotts- och hälsovetenskap</t>
         </is>
       </c>
       <c r="G180" t="inlineStr">
         <is>
-          <t>Telefonrådgivning vid distanskontakter inom hälso- och sjukvården</t>
+          <t>Idrottsvetenskaplig uppsats</t>
         </is>
       </c>
       <c r="H180" t="inlineStr">
@@ -8450,14 +8454,14 @@
       </c>
       <c r="I180" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AVÅ28C</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2XY</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" s="2" t="inlineStr">
         <is>
-          <t>AVÅ28H</t>
+          <t>AVÅ28C</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
@@ -8483,7 +8487,7 @@
       </c>
       <c r="G181" t="inlineStr">
         <is>
-          <t>Nutrition och ätande (fristående kurs)</t>
+          <t>Telefonrådgivning vid distanskontakter inom hälso- och sjukvården</t>
         </is>
       </c>
       <c r="H181" t="inlineStr">
@@ -8493,19 +8497,19 @@
       </c>
       <c r="I181" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AVÅ28H</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AVÅ28C</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" s="2" t="inlineStr">
         <is>
-          <t>GIH2ZA</t>
+          <t>AVÅ28H</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>IDA</t>
+          <t>OMV</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
@@ -8515,18 +8519,18 @@
       </c>
       <c r="D182" t="inlineStr">
         <is>
-          <t>2022-12-12</t>
+          <t>2022-11-14</t>
         </is>
       </c>
       <c r="E182" t="inlineStr"/>
       <c r="F182" t="inlineStr">
         <is>
-          <t>Idrotts- och hälsovetenskap</t>
+          <t>Omvårdnad</t>
         </is>
       </c>
       <c r="G182" t="inlineStr">
         <is>
-          <t>Vinterfriluftsliv genom skidor och skridskor (VAL)</t>
+          <t>Nutrition och ätande (fristående kurs)</t>
         </is>
       </c>
       <c r="H182" t="inlineStr">
@@ -8536,14 +8540,14 @@
       </c>
       <c r="I182" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2ZA</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AVÅ28H</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" s="2" t="inlineStr">
         <is>
-          <t>GIH2ZB</t>
+          <t>GIH2ZA</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
@@ -8569,7 +8573,7 @@
       </c>
       <c r="G183" t="inlineStr">
         <is>
-          <t>Hälsopedagogik (VAL)</t>
+          <t>Vinterfriluftsliv genom skidor och skridskor (VAL)</t>
         </is>
       </c>
       <c r="H183" t="inlineStr">
@@ -8579,14 +8583,14 @@
       </c>
       <c r="I183" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2ZB</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2ZA</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" s="2" t="inlineStr">
         <is>
-          <t>GIH2ZC</t>
+          <t>GIH2ZB</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
@@ -8612,7 +8616,7 @@
       </c>
       <c r="G184" t="inlineStr">
         <is>
-          <t>Humanbiologi 1 (VAL)</t>
+          <t>Hälsopedagogik (VAL)</t>
         </is>
       </c>
       <c r="H184" t="inlineStr">
@@ -8622,14 +8626,14 @@
       </c>
       <c r="I184" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2ZC</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2ZB</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" s="2" t="inlineStr">
         <is>
-          <t>GIH2ZD</t>
+          <t>GIH2ZC</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
@@ -8655,7 +8659,7 @@
       </c>
       <c r="G185" t="inlineStr">
         <is>
-          <t>Simning (VAL)</t>
+          <t>Humanbiologi 1 (VAL)</t>
         </is>
       </c>
       <c r="H185" t="inlineStr">
@@ -8665,14 +8669,14 @@
       </c>
       <c r="I185" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2ZD</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2ZC</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" s="2" t="inlineStr">
         <is>
-          <t>GIH2ZE</t>
+          <t>GIH2ZD</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
@@ -8698,7 +8702,7 @@
       </c>
       <c r="G186" t="inlineStr">
         <is>
-          <t>Bedömning och betygssättning i idrott och hälsa (VAL)</t>
+          <t>Simning (VAL)</t>
         </is>
       </c>
       <c r="H186" t="inlineStr">
@@ -8708,19 +8712,19 @@
       </c>
       <c r="I186" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2ZE</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2ZD</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" s="2" t="inlineStr">
         <is>
-          <t>GVÅ2ZG</t>
+          <t>GIH2ZE</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>OMV</t>
+          <t>IDA</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
@@ -8736,12 +8740,12 @@
       <c r="E187" t="inlineStr"/>
       <c r="F187" t="inlineStr">
         <is>
-          <t>Omvårdnad</t>
+          <t>Idrotts- och hälsovetenskap</t>
         </is>
       </c>
       <c r="G187" t="inlineStr">
         <is>
-          <t>Personcentrerad vård med fördjupning inom omvårdnad</t>
+          <t>Bedömning och betygssättning i idrott och hälsa (VAL)</t>
         </is>
       </c>
       <c r="H187" t="inlineStr">
@@ -8751,14 +8755,14 @@
       </c>
       <c r="I187" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GVÅ2ZG</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH2ZE</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" s="2" t="inlineStr">
         <is>
-          <t>GVÅ2ZY</t>
+          <t>GVÅ2ZG</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
@@ -8784,7 +8788,7 @@
       </c>
       <c r="G188" t="inlineStr">
         <is>
-          <t>Metoder för evidensbaserad vård II</t>
+          <t>Personcentrerad vård med fördjupning inom omvårdnad</t>
         </is>
       </c>
       <c r="H188" t="inlineStr">
@@ -8794,19 +8798,19 @@
       </c>
       <c r="I188" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GVÅ2ZY</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GVÅ2ZG</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" s="2" t="inlineStr">
         <is>
-          <t>GIH334</t>
+          <t>GVÅ2ZY</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>IDA</t>
+          <t>OMV</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
@@ -8816,18 +8820,18 @@
       </c>
       <c r="D189" t="inlineStr">
         <is>
-          <t>2023-02-07</t>
+          <t>2022-12-12</t>
         </is>
       </c>
       <c r="E189" t="inlineStr"/>
       <c r="F189" t="inlineStr">
         <is>
-          <t>Idrotts- och hälsovetenskap</t>
+          <t>Omvårdnad</t>
         </is>
       </c>
       <c r="G189" t="inlineStr">
         <is>
-          <t>Sportjournalistik</t>
+          <t>Metoder för evidensbaserad vård II</t>
         </is>
       </c>
       <c r="H189" t="inlineStr">
@@ -8837,19 +8841,19 @@
       </c>
       <c r="I189" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH334</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GVÅ2ZY</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" s="2" t="inlineStr">
         <is>
-          <t>GSA32Y</t>
+          <t>GSR2ZH</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>SAA</t>
+          <t>SRP</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
@@ -8859,18 +8863,18 @@
       </c>
       <c r="D190" t="inlineStr">
         <is>
-          <t>2023-02-07</t>
+          <t>2022-12-12</t>
         </is>
       </c>
       <c r="E190" t="inlineStr"/>
       <c r="F190" t="inlineStr">
         <is>
-          <t>Socialt arbete</t>
+          <t>Sexuell, reproduktiv och perinatal hälsa</t>
         </is>
       </c>
       <c r="G190" t="inlineStr">
         <is>
-          <t>Organisation, grupp och samverkan</t>
+          <t>Ungdomar och unga vuxnas sexuella och reproduktiva hälsa och rättigheter I</t>
         </is>
       </c>
       <c r="H190" t="inlineStr">
@@ -8880,14 +8884,14 @@
       </c>
       <c r="I190" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA32Y</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSR2ZH</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" s="2" t="inlineStr">
         <is>
-          <t>GIH33J</t>
+          <t>GIH334</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
@@ -8902,7 +8906,7 @@
       </c>
       <c r="D191" t="inlineStr">
         <is>
-          <t>2023-02-23</t>
+          <t>2023-02-07</t>
         </is>
       </c>
       <c r="E191" t="inlineStr"/>
@@ -8913,7 +8917,7 @@
       </c>
       <c r="G191" t="inlineStr">
         <is>
-          <t>Grundläggande fysiologi och tillämpad idrottsfysiologi (Klättring)</t>
+          <t>Sportjournalistik</t>
         </is>
       </c>
       <c r="H191" t="inlineStr">
@@ -8923,19 +8927,19 @@
       </c>
       <c r="I191" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH33J</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH334</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" s="2" t="inlineStr">
         <is>
-          <t>GIH33K</t>
+          <t>GSA32Y</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>IDA</t>
+          <t>SAA</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
@@ -8945,18 +8949,18 @@
       </c>
       <c r="D192" t="inlineStr">
         <is>
-          <t>2023-02-23</t>
+          <t>2023-02-07</t>
         </is>
       </c>
       <c r="E192" t="inlineStr"/>
       <c r="F192" t="inlineStr">
         <is>
-          <t>Idrotts- och hälsovetenskap</t>
+          <t>Socialt arbete</t>
         </is>
       </c>
       <c r="G192" t="inlineStr">
         <is>
-          <t>Funktionell anatomi (Klättring)</t>
+          <t>Organisation, grupp och samverkan</t>
         </is>
       </c>
       <c r="H192" t="inlineStr">
@@ -8966,14 +8970,14 @@
       </c>
       <c r="I192" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH33K</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA32Y</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" s="2" t="inlineStr">
         <is>
-          <t>GIH33P</t>
+          <t>GIH33J</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
@@ -8999,7 +9003,7 @@
       </c>
       <c r="G193" t="inlineStr">
         <is>
-          <t>Biomekanik (Klättring)</t>
+          <t>Grundläggande fysiologi och tillämpad idrottsfysiologi (Klättring)</t>
         </is>
       </c>
       <c r="H193" t="inlineStr">
@@ -9009,14 +9013,14 @@
       </c>
       <c r="I193" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH33P</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH33J</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" s="2" t="inlineStr">
         <is>
-          <t>GIH34D</t>
+          <t>GIH33K</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
@@ -9031,7 +9035,7 @@
       </c>
       <c r="D194" t="inlineStr">
         <is>
-          <t>2023-04-05</t>
+          <t>2023-02-23</t>
         </is>
       </c>
       <c r="E194" t="inlineStr"/>
@@ -9042,7 +9046,7 @@
       </c>
       <c r="G194" t="inlineStr">
         <is>
-          <t>Kvalitativ och kvantitativ vetenskaplig metod</t>
+          <t>Funktionell anatomi (Klättring)</t>
         </is>
       </c>
       <c r="H194" t="inlineStr">
@@ -9052,14 +9056,14 @@
       </c>
       <c r="I194" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH34D</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH33K</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" s="2" t="inlineStr">
         <is>
-          <t>GIH34S</t>
+          <t>GIH33P</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
@@ -9074,7 +9078,7 @@
       </c>
       <c r="D195" t="inlineStr">
         <is>
-          <t>2023-05-09</t>
+          <t>2023-02-23</t>
         </is>
       </c>
       <c r="E195" t="inlineStr"/>
@@ -9085,7 +9089,7 @@
       </c>
       <c r="G195" t="inlineStr">
         <is>
-          <t>Lek, dans samt mål- och nätspel (VAL)</t>
+          <t>Biomekanik (Klättring)</t>
         </is>
       </c>
       <c r="H195" t="inlineStr">
@@ -9095,14 +9099,14 @@
       </c>
       <c r="I195" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH34S</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH33P</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" s="2" t="inlineStr">
         <is>
-          <t>GIH34T</t>
+          <t>GIH34D</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
@@ -9117,7 +9121,7 @@
       </c>
       <c r="D196" t="inlineStr">
         <is>
-          <t>2023-05-09</t>
+          <t>2023-04-05</t>
         </is>
       </c>
       <c r="E196" t="inlineStr"/>
@@ -9128,7 +9132,7 @@
       </c>
       <c r="G196" t="inlineStr">
         <is>
-          <t>Humanbiologi 2 (VAL)</t>
+          <t>Kvalitativ och kvantitativ vetenskaplig metod</t>
         </is>
       </c>
       <c r="H196" t="inlineStr">
@@ -9138,14 +9142,14 @@
       </c>
       <c r="I196" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH34T</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH34D</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" s="2" t="inlineStr">
         <is>
-          <t>GIH34U</t>
+          <t>GIH34S</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
@@ -9171,7 +9175,7 @@
       </c>
       <c r="G197" t="inlineStr">
         <is>
-          <t>Dans, gymnastik och friidrott (VAL)</t>
+          <t>Lek, dans samt mål- och nätspel (VAL)</t>
         </is>
       </c>
       <c r="H197" t="inlineStr">
@@ -9181,14 +9185,14 @@
       </c>
       <c r="I197" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH34U</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH34S</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" s="2" t="inlineStr">
         <is>
-          <t>GIH34V</t>
+          <t>GIH34T</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
@@ -9214,7 +9218,7 @@
       </c>
       <c r="G198" t="inlineStr">
         <is>
-          <t>Arbetsmiljö, ergonomi och näringslära (VAL)</t>
+          <t>Humanbiologi 2 (VAL)</t>
         </is>
       </c>
       <c r="H198" t="inlineStr">
@@ -9224,14 +9228,14 @@
       </c>
       <c r="I198" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH34V</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH34T</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" s="2" t="inlineStr">
         <is>
-          <t>GIH35B</t>
+          <t>GIH34U</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
@@ -9246,7 +9250,7 @@
       </c>
       <c r="D199" t="inlineStr">
         <is>
-          <t>2023-06-19</t>
+          <t>2023-05-09</t>
         </is>
       </c>
       <c r="E199" t="inlineStr"/>
@@ -9257,7 +9261,7 @@
       </c>
       <c r="G199" t="inlineStr">
         <is>
-          <t>Examensarbete för kandidatexamen i idrotts- och hälsovetenskap</t>
+          <t>Dans, gymnastik och friidrott (VAL)</t>
         </is>
       </c>
       <c r="H199" t="inlineStr">
@@ -9267,14 +9271,14 @@
       </c>
       <c r="I199" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH35B</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH34U</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" s="2" t="inlineStr">
         <is>
-          <t>GIH35P</t>
+          <t>GIH34V</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
@@ -9289,7 +9293,7 @@
       </c>
       <c r="D200" t="inlineStr">
         <is>
-          <t>2023-08-30</t>
+          <t>2023-05-09</t>
         </is>
       </c>
       <c r="E200" t="inlineStr"/>
@@ -9300,7 +9304,7 @@
       </c>
       <c r="G200" t="inlineStr">
         <is>
-          <t>Träningslära: styrkelyft för öppen klass och veteraner</t>
+          <t>Arbetsmiljö, ergonomi och näringslära (VAL)</t>
         </is>
       </c>
       <c r="H200" t="inlineStr">
@@ -9310,14 +9314,14 @@
       </c>
       <c r="I200" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH35P</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH34V</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" s="2" t="inlineStr">
         <is>
-          <t>GIH35V</t>
+          <t>GIH35B</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
@@ -9332,7 +9336,7 @@
       </c>
       <c r="D201" t="inlineStr">
         <is>
-          <t>2023-08-30</t>
+          <t>2023-06-19</t>
         </is>
       </c>
       <c r="E201" t="inlineStr"/>
@@ -9343,7 +9347,7 @@
       </c>
       <c r="G201" t="inlineStr">
         <is>
-          <t>Idrottens träningslära</t>
+          <t>Examensarbete för kandidatexamen i idrotts- och hälsovetenskap</t>
         </is>
       </c>
       <c r="H201" t="inlineStr">
@@ -9353,14 +9357,14 @@
       </c>
       <c r="I201" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH35V</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH35B</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" s="2" t="inlineStr">
         <is>
-          <t>GIH35Z</t>
+          <t>GIH35P</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
@@ -9386,7 +9390,7 @@
       </c>
       <c r="G202" t="inlineStr">
         <is>
-          <t>Medier och kommunikation inom hälsa och idrott</t>
+          <t>Träningslära: styrkelyft för öppen klass och veteraner</t>
         </is>
       </c>
       <c r="H202" t="inlineStr">
@@ -9396,19 +9400,19 @@
       </c>
       <c r="I202" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH35Z</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH35P</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" s="2" t="inlineStr">
         <is>
-          <t>AMC29F</t>
+          <t>GIH35V</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>MCA</t>
+          <t>IDA</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
@@ -9424,12 +9428,12 @@
       <c r="E203" t="inlineStr"/>
       <c r="F203" t="inlineStr">
         <is>
-          <t>Medicinsk vetenskap</t>
+          <t>Idrotts- och hälsovetenskap</t>
         </is>
       </c>
       <c r="G203" t="inlineStr">
         <is>
-          <t>Examensarbete för magisterexamen i fysioterapi</t>
+          <t>Idrottens träningslära</t>
         </is>
       </c>
       <c r="H203" t="inlineStr">
@@ -9439,19 +9443,19 @@
       </c>
       <c r="I203" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMC29F</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH35V</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" s="2" t="inlineStr">
         <is>
-          <t>ASR29U</t>
+          <t>GIH35Z</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>SRP</t>
+          <t>IDA</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
@@ -9461,18 +9465,18 @@
       </c>
       <c r="D204" t="inlineStr">
         <is>
-          <t>2023-10-03</t>
+          <t>2023-08-30</t>
         </is>
       </c>
       <c r="E204" t="inlineStr"/>
       <c r="F204" t="inlineStr">
         <is>
-          <t>Sexuell, reproduktiv och perinatal hälsa</t>
+          <t>Idrotts- och hälsovetenskap</t>
         </is>
       </c>
       <c r="G204" t="inlineStr">
         <is>
-          <t>Graviditet, förlossning och postpartumvård II</t>
+          <t>Medier och kommunikation inom hälsa och idrott</t>
         </is>
       </c>
       <c r="H204" t="inlineStr">
@@ -9482,19 +9486,19 @@
       </c>
       <c r="I204" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29U</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH35Z</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" s="2" t="inlineStr">
         <is>
-          <t>GIH37B</t>
+          <t>AMC29F</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>IDA</t>
+          <t>MCA</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
@@ -9504,18 +9508,18 @@
       </c>
       <c r="D205" t="inlineStr">
         <is>
-          <t>2023-11-07</t>
+          <t>2023-08-30</t>
         </is>
       </c>
       <c r="E205" t="inlineStr"/>
       <c r="F205" t="inlineStr">
         <is>
-          <t>Idrotts- och hälsovetenskap</t>
+          <t>Medicinsk vetenskap</t>
         </is>
       </c>
       <c r="G205" t="inlineStr">
         <is>
-          <t>Mål- och nätspel (VAL)</t>
+          <t>Examensarbete för magisterexamen i fysioterapi</t>
         </is>
       </c>
       <c r="H205" t="inlineStr">
@@ -9525,19 +9529,19 @@
       </c>
       <c r="I205" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH37B</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMC29F</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" s="2" t="inlineStr">
         <is>
-          <t>GIH37C</t>
+          <t>ASR29U</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>IDA</t>
+          <t>SRP</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
@@ -9547,18 +9551,18 @@
       </c>
       <c r="D206" t="inlineStr">
         <is>
-          <t>2023-11-07</t>
+          <t>2023-10-03</t>
         </is>
       </c>
       <c r="E206" t="inlineStr"/>
       <c r="F206" t="inlineStr">
         <is>
-          <t>Idrotts- och hälsovetenskap</t>
+          <t>Sexuell, reproduktiv och perinatal hälsa</t>
         </is>
       </c>
       <c r="G206" t="inlineStr">
         <is>
-          <t>Rörelse, rytm och dans (VAL)</t>
+          <t>Graviditet, förlossning och postpartumvård II</t>
         </is>
       </c>
       <c r="H206" t="inlineStr">
@@ -9568,19 +9572,19 @@
       </c>
       <c r="I206" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH37C</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASR29U</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" s="2" t="inlineStr">
         <is>
-          <t>GVÅ37H</t>
+          <t>GIH37B</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>OMV</t>
+          <t>IDA</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
@@ -9596,12 +9600,12 @@
       <c r="E207" t="inlineStr"/>
       <c r="F207" t="inlineStr">
         <is>
-          <t>Omvårdnad</t>
+          <t>Idrotts- och hälsovetenskap</t>
         </is>
       </c>
       <c r="G207" t="inlineStr">
         <is>
-          <t>Personcentrerad vård inom psykiatrisk vård</t>
+          <t>Mål- och nätspel (VAL)</t>
         </is>
       </c>
       <c r="H207" t="inlineStr">
@@ -9611,19 +9615,19 @@
       </c>
       <c r="I207" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GVÅ37H</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH37B</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" s="2" t="inlineStr">
         <is>
-          <t>GVÅ382</t>
+          <t>GIH37C</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>OMV</t>
+          <t>IDA</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
@@ -9639,12 +9643,12 @@
       <c r="E208" t="inlineStr"/>
       <c r="F208" t="inlineStr">
         <is>
-          <t>Omvårdnad</t>
+          <t>Idrotts- och hälsovetenskap</t>
         </is>
       </c>
       <c r="G208" t="inlineStr">
         <is>
-          <t>Personcentrerad vård inom olika vårdsammanhang</t>
+          <t>Rörelse, rytm och dans (VAL)</t>
         </is>
       </c>
       <c r="H208" t="inlineStr">
@@ -9654,19 +9658,19 @@
       </c>
       <c r="I208" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GVÅ382</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH37C</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" s="2" t="inlineStr">
         <is>
-          <t>GSA2DW</t>
+          <t>GVÅ37H</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>SAA</t>
+          <t>OMV</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
@@ -9676,22 +9680,18 @@
       </c>
       <c r="D209" t="inlineStr">
         <is>
-          <t>2020-02-20</t>
-        </is>
-      </c>
-      <c r="E209" t="inlineStr">
-        <is>
-          <t>2023-11-30</t>
-        </is>
-      </c>
+          <t>2023-11-07</t>
+        </is>
+      </c>
+      <c r="E209" t="inlineStr"/>
       <c r="F209" t="inlineStr">
         <is>
-          <t>Socialt arbete</t>
+          <t>Omvårdnad</t>
         </is>
       </c>
       <c r="G209" t="inlineStr">
         <is>
-          <t>Försörjning, rehabilitering och aktivering i socialt arbete</t>
+          <t>Personcentrerad vård inom psykiatrisk vård</t>
         </is>
       </c>
       <c r="H209" t="inlineStr">
@@ -9701,19 +9701,19 @@
       </c>
       <c r="I209" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA2DW</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GVÅ37H</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" s="2" t="inlineStr">
         <is>
-          <t>GIH37N</t>
+          <t>GVÅ382</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>IDA</t>
+          <t>OMV</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
@@ -9723,18 +9723,18 @@
       </c>
       <c r="D210" t="inlineStr">
         <is>
-          <t>2023-12-05</t>
+          <t>2023-11-07</t>
         </is>
       </c>
       <c r="E210" t="inlineStr"/>
       <c r="F210" t="inlineStr">
         <is>
-          <t>Idrotts- och hälsovetenskap</t>
+          <t>Omvårdnad</t>
         </is>
       </c>
       <c r="G210" t="inlineStr">
         <is>
-          <t>Friluftsliv och bedömning i ämnet idrott och hälsa</t>
+          <t>Personcentrerad vård inom olika vårdsammanhang</t>
         </is>
       </c>
       <c r="H210" t="inlineStr">
@@ -9744,19 +9744,19 @@
       </c>
       <c r="I210" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH37N</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GVÅ382</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" s="2" t="inlineStr">
         <is>
-          <t>GIH37P</t>
+          <t>GSA2DW</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>IDA</t>
+          <t>SAA</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
@@ -9766,18 +9766,22 @@
       </c>
       <c r="D211" t="inlineStr">
         <is>
-          <t>2023-12-05</t>
-        </is>
-      </c>
-      <c r="E211" t="inlineStr"/>
+          <t>2020-02-20</t>
+        </is>
+      </c>
+      <c r="E211" t="inlineStr">
+        <is>
+          <t>2023-11-30</t>
+        </is>
+      </c>
       <c r="F211" t="inlineStr">
         <is>
-          <t>Idrotts- och hälsovetenskap</t>
+          <t>Socialt arbete</t>
         </is>
       </c>
       <c r="G211" t="inlineStr">
         <is>
-          <t>Idrott och hälsa I med didaktisk inriktning åk 4-6</t>
+          <t>Försörjning, rehabilitering och aktivering i socialt arbete</t>
         </is>
       </c>
       <c r="H211" t="inlineStr">
@@ -9787,14 +9791,14 @@
       </c>
       <c r="I211" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH37P</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA2DW</t>
         </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" s="2" t="inlineStr">
         <is>
-          <t>GIH37Q</t>
+          <t>GIH37N</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
@@ -9820,7 +9824,7 @@
       </c>
       <c r="G212" t="inlineStr">
         <is>
-          <t>Idrott och hälsa I med didaktisk inriktning</t>
+          <t>Friluftsliv och bedömning i ämnet idrott och hälsa</t>
         </is>
       </c>
       <c r="H212" t="inlineStr">
@@ -9830,19 +9834,19 @@
       </c>
       <c r="I212" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH37Q</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH37N</t>
         </is>
       </c>
     </row>
     <row r="213">
       <c r="A213" s="2" t="inlineStr">
         <is>
-          <t>AMC29Y</t>
+          <t>GIH37P</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>MCA</t>
+          <t>IDA</t>
         </is>
       </c>
       <c r="C213" t="inlineStr">
@@ -9858,12 +9862,12 @@
       <c r="E213" t="inlineStr"/>
       <c r="F213" t="inlineStr">
         <is>
-          <t>Medicinsk vetenskap</t>
+          <t>Idrotts- och hälsovetenskap</t>
         </is>
       </c>
       <c r="G213" t="inlineStr">
         <is>
-          <t>Förskrivningsrätt för vissa läkemedel och förbrukningsartiklar</t>
+          <t>Idrott och hälsa I med didaktisk inriktning åk 4-6</t>
         </is>
       </c>
       <c r="H213" t="inlineStr">
@@ -9873,19 +9877,19 @@
       </c>
       <c r="I213" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMC29Y</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH37P</t>
         </is>
       </c>
     </row>
     <row r="214">
       <c r="A214" s="2" t="inlineStr">
         <is>
-          <t>AMC2A7</t>
+          <t>GIH37Q</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>MCA</t>
+          <t>IDA</t>
         </is>
       </c>
       <c r="C214" t="inlineStr">
@@ -9901,12 +9905,12 @@
       <c r="E214" t="inlineStr"/>
       <c r="F214" t="inlineStr">
         <is>
-          <t>Medicinsk vetenskap</t>
+          <t>Idrotts- och hälsovetenskap</t>
         </is>
       </c>
       <c r="G214" t="inlineStr">
         <is>
-          <t>Kardiologi: Arytmi</t>
+          <t>Idrott och hälsa I med didaktisk inriktning</t>
         </is>
       </c>
       <c r="H214" t="inlineStr">
@@ -9916,19 +9920,19 @@
       </c>
       <c r="I214" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMC2A7</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH37Q</t>
         </is>
       </c>
     </row>
     <row r="215">
       <c r="A215" s="2" t="inlineStr">
         <is>
-          <t>GVÅ384</t>
+          <t>AMC29Y</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>OMV</t>
+          <t>MCA</t>
         </is>
       </c>
       <c r="C215" t="inlineStr">
@@ -9944,12 +9948,12 @@
       <c r="E215" t="inlineStr"/>
       <c r="F215" t="inlineStr">
         <is>
-          <t>Omvårdnad</t>
+          <t>Medicinsk vetenskap</t>
         </is>
       </c>
       <c r="G215" t="inlineStr">
         <is>
-          <t>Personcentrerad vård inom somatisk vård</t>
+          <t>Förskrivningsrätt för vissa läkemedel och förbrukningsartiklar</t>
         </is>
       </c>
       <c r="H215" t="inlineStr">
@@ -9959,19 +9963,19 @@
       </c>
       <c r="I215" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GVÅ384</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMC29Y</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" s="2" t="inlineStr">
         <is>
-          <t>GSR38B</t>
+          <t>AMC2A7</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>SRP</t>
+          <t>MCA</t>
         </is>
       </c>
       <c r="C216" t="inlineStr">
@@ -9987,12 +9991,12 @@
       <c r="E216" t="inlineStr"/>
       <c r="F216" t="inlineStr">
         <is>
-          <t>Sexuell, reproduktiv och perinatal hälsa</t>
+          <t>Medicinsk vetenskap</t>
         </is>
       </c>
       <c r="G216" t="inlineStr">
         <is>
-          <t>Sexuell och reproduktiv hälsa samt rättigheter för ungdomar och unga vuxna i Ukraina</t>
+          <t>Kardiologi: Arytmi</t>
         </is>
       </c>
       <c r="H216" t="inlineStr">
@@ -10002,19 +10006,19 @@
       </c>
       <c r="I216" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSR38B</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMC2A7</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" s="2" t="inlineStr">
         <is>
-          <t>GNV396</t>
+          <t>GVÅ384</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>NAV</t>
+          <t>OMV</t>
         </is>
       </c>
       <c r="C217" t="inlineStr">
@@ -10024,18 +10028,18 @@
       </c>
       <c r="D217" t="inlineStr">
         <is>
-          <t>2023-12-20</t>
+          <t>2023-12-05</t>
         </is>
       </c>
       <c r="E217" t="inlineStr"/>
       <c r="F217" t="inlineStr">
         <is>
-          <t>Naturvetenskap</t>
+          <t>Omvårdnad</t>
         </is>
       </c>
       <c r="G217" t="inlineStr">
         <is>
-          <t>Teknik för grundlärare i förskoleklass och årskurs 1-6</t>
+          <t>Personcentrerad vård inom somatisk vård</t>
         </is>
       </c>
       <c r="H217" t="inlineStr">
@@ -10045,19 +10049,19 @@
       </c>
       <c r="I217" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GNV396</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GVÅ384</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" s="2" t="inlineStr">
         <is>
-          <t>GIH3AM</t>
+          <t>GSR38B</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>IDA</t>
+          <t>SRP</t>
         </is>
       </c>
       <c r="C218" t="inlineStr">
@@ -10067,18 +10071,18 @@
       </c>
       <c r="D218" t="inlineStr">
         <is>
-          <t>2024-02-27</t>
+          <t>2023-12-05</t>
         </is>
       </c>
       <c r="E218" t="inlineStr"/>
       <c r="F218" t="inlineStr">
         <is>
-          <t>Idrotts- och hälsovetenskap</t>
+          <t>Sexuell, reproduktiv och perinatal hälsa</t>
         </is>
       </c>
       <c r="G218" t="inlineStr">
         <is>
-          <t>Klättringens tränarskap</t>
+          <t>Sexuell och reproduktiv hälsa samt rättigheter för ungdomar och unga vuxna i Ukraina</t>
         </is>
       </c>
       <c r="H218" t="inlineStr">
@@ -10088,19 +10092,19 @@
       </c>
       <c r="I218" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3AM</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSR38B</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" s="2" t="inlineStr">
         <is>
-          <t>GIH3AQ</t>
+          <t>GNV396</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>IDA</t>
+          <t>NAV</t>
         </is>
       </c>
       <c r="C219" t="inlineStr">
@@ -10110,18 +10114,18 @@
       </c>
       <c r="D219" t="inlineStr">
         <is>
-          <t>2024-02-27</t>
+          <t>2023-12-20</t>
         </is>
       </c>
       <c r="E219" t="inlineStr"/>
       <c r="F219" t="inlineStr">
         <is>
-          <t>Idrotts- och hälsovetenskap</t>
+          <t>Naturvetenskap</t>
         </is>
       </c>
       <c r="G219" t="inlineStr">
         <is>
-          <t>Styrketräningens teori och praktiska tillämpning</t>
+          <t>Teknik för grundlärare i förskoleklass och årskurs 1-6</t>
         </is>
       </c>
       <c r="H219" t="inlineStr">
@@ -10131,19 +10135,19 @@
       </c>
       <c r="I219" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3AQ</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GNV396</t>
         </is>
       </c>
     </row>
     <row r="220">
       <c r="A220" s="2" t="inlineStr">
         <is>
-          <t>AMC2AE</t>
+          <t>GIH3AM</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>MCA</t>
+          <t>IDA</t>
         </is>
       </c>
       <c r="C220" t="inlineStr">
@@ -10159,12 +10163,12 @@
       <c r="E220" t="inlineStr"/>
       <c r="F220" t="inlineStr">
         <is>
-          <t>Medicinsk vetenskap</t>
+          <t>Idrotts- och hälsovetenskap</t>
         </is>
       </c>
       <c r="G220" t="inlineStr">
         <is>
-          <t>Fysioterapi med fokus på smärta och hållbar utveckling</t>
+          <t>Klättringens tränarskap</t>
         </is>
       </c>
       <c r="H220" t="inlineStr">
@@ -10174,19 +10178,19 @@
       </c>
       <c r="I220" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMC2AE</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3AM</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" s="2" t="inlineStr">
         <is>
-          <t>GSA3AS</t>
+          <t>GIH3AQ</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>SAA</t>
+          <t>IDA</t>
         </is>
       </c>
       <c r="C221" t="inlineStr">
@@ -10196,18 +10200,18 @@
       </c>
       <c r="D221" t="inlineStr">
         <is>
-          <t>2024-03-04</t>
+          <t>2024-02-27</t>
         </is>
       </c>
       <c r="E221" t="inlineStr"/>
       <c r="F221" t="inlineStr">
         <is>
-          <t>Socialt arbete</t>
+          <t>Idrotts- och hälsovetenskap</t>
         </is>
       </c>
       <c r="G221" t="inlineStr">
         <is>
-          <t>Samsjuklighet - skadligt bruk eller beroende och samtidig psykisk ohälsa</t>
+          <t>Styrketräningens teori och praktiska tillämpning</t>
         </is>
       </c>
       <c r="H221" t="inlineStr">
@@ -10217,19 +10221,19 @@
       </c>
       <c r="I221" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA3AS</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3AQ</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" s="2" t="inlineStr">
         <is>
-          <t>GIH3CS</t>
+          <t>AMC2AE</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>IDA</t>
+          <t>MCA</t>
         </is>
       </c>
       <c r="C222" t="inlineStr">
@@ -10239,18 +10243,18 @@
       </c>
       <c r="D222" t="inlineStr">
         <is>
-          <t>2024-11-12</t>
+          <t>2024-02-27</t>
         </is>
       </c>
       <c r="E222" t="inlineStr"/>
       <c r="F222" t="inlineStr">
         <is>
-          <t>Idrotts- och hälsovetenskap</t>
+          <t>Medicinsk vetenskap</t>
         </is>
       </c>
       <c r="G222" t="inlineStr">
         <is>
-          <t>Grundläggande idrottsfysiologi</t>
+          <t>Fysioterapi med fokus på smärta och hållbar utveckling</t>
         </is>
       </c>
       <c r="H222" t="inlineStr">
@@ -10260,19 +10264,19 @@
       </c>
       <c r="I222" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3CS</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMC2AE</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" s="2" t="inlineStr">
         <is>
-          <t>GIH3D4</t>
+          <t>GSA3AS</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>IDA</t>
+          <t>SAA</t>
         </is>
       </c>
       <c r="C223" t="inlineStr">
@@ -10282,18 +10286,18 @@
       </c>
       <c r="D223" t="inlineStr">
         <is>
-          <t>2024-11-12</t>
+          <t>2024-03-04</t>
         </is>
       </c>
       <c r="E223" t="inlineStr"/>
       <c r="F223" t="inlineStr">
         <is>
-          <t>Idrotts- och hälsovetenskap</t>
+          <t>Socialt arbete</t>
         </is>
       </c>
       <c r="G223" t="inlineStr">
         <is>
-          <t>Träningslära för tävlingsinriktad idrott</t>
+          <t>Samsjuklighet - skadligt bruk eller beroende och samtidig psykisk ohälsa</t>
         </is>
       </c>
       <c r="H223" t="inlineStr">
@@ -10303,14 +10307,14 @@
       </c>
       <c r="I223" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3D4</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA3AS</t>
         </is>
       </c>
     </row>
     <row r="224">
       <c r="A224" s="2" t="inlineStr">
         <is>
-          <t>GIH3D5</t>
+          <t>GIH3CS</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
@@ -10336,7 +10340,7 @@
       </c>
       <c r="G224" t="inlineStr">
         <is>
-          <t>Träningslära för hälsoinriktad fysisk aktivitet</t>
+          <t>Grundläggande idrottsfysiologi</t>
         </is>
       </c>
       <c r="H224" t="inlineStr">
@@ -10346,14 +10350,14 @@
       </c>
       <c r="I224" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3D5</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3CS</t>
         </is>
       </c>
     </row>
     <row r="225">
       <c r="A225" s="2" t="inlineStr">
         <is>
-          <t>GIH3D6</t>
+          <t>GIH3D4</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
@@ -10379,7 +10383,7 @@
       </c>
       <c r="G225" t="inlineStr">
         <is>
-          <t>Näringslära med inriktning mot idrott och fysisk aktivitet</t>
+          <t>Träningslära för tävlingsinriktad idrott</t>
         </is>
       </c>
       <c r="H225" t="inlineStr">
@@ -10389,19 +10393,19 @@
       </c>
       <c r="I225" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3D6</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3D4</t>
         </is>
       </c>
     </row>
     <row r="226">
       <c r="A226" s="2" t="inlineStr">
         <is>
-          <t>GSA3DN</t>
+          <t>GIH3D5</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>SAA</t>
+          <t>IDA</t>
         </is>
       </c>
       <c r="C226" t="inlineStr">
@@ -10411,18 +10415,18 @@
       </c>
       <c r="D226" t="inlineStr">
         <is>
-          <t>2024-12-10</t>
+          <t>2024-11-12</t>
         </is>
       </c>
       <c r="E226" t="inlineStr"/>
       <c r="F226" t="inlineStr">
         <is>
-          <t>Socialt arbete</t>
+          <t>Idrotts- och hälsovetenskap</t>
         </is>
       </c>
       <c r="G226" t="inlineStr">
         <is>
-          <t>Försörjning, rehabilitering och aktivering i socialt arbete</t>
+          <t>Träningslära för hälsoinriktad fysisk aktivitet</t>
         </is>
       </c>
       <c r="H226" t="inlineStr">
@@ -10432,19 +10436,19 @@
       </c>
       <c r="I226" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA3DN</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3D5</t>
         </is>
       </c>
     </row>
     <row r="227">
       <c r="A227" s="2" t="inlineStr">
         <is>
-          <t>GSA3DS</t>
+          <t>GIH3D6</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>SAA</t>
+          <t>IDA</t>
         </is>
       </c>
       <c r="C227" t="inlineStr">
@@ -10454,18 +10458,18 @@
       </c>
       <c r="D227" t="inlineStr">
         <is>
-          <t>2024-12-10</t>
+          <t>2024-11-12</t>
         </is>
       </c>
       <c r="E227" t="inlineStr"/>
       <c r="F227" t="inlineStr">
         <is>
-          <t>Socialt arbete</t>
+          <t>Idrotts- och hälsovetenskap</t>
         </is>
       </c>
       <c r="G227" t="inlineStr">
         <is>
-          <t>Organisation, grupp och samverkan</t>
+          <t>Näringslära med inriktning mot idrott och fysisk aktivitet</t>
         </is>
       </c>
       <c r="H227" t="inlineStr">
@@ -10475,19 +10479,19 @@
       </c>
       <c r="I227" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA3DS</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3D6</t>
         </is>
       </c>
     </row>
     <row r="228">
       <c r="A228" s="2" t="inlineStr">
         <is>
-          <t>GVÅ35Q</t>
+          <t>GSA3DN</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>OMV</t>
+          <t>SAA</t>
         </is>
       </c>
       <c r="C228" t="inlineStr">
@@ -10497,22 +10501,18 @@
       </c>
       <c r="D228" t="inlineStr">
         <is>
-          <t>2023-08-30</t>
-        </is>
-      </c>
-      <c r="E228" t="inlineStr">
-        <is>
-          <t>2025-01-13</t>
-        </is>
-      </c>
+          <t>2024-12-10</t>
+        </is>
+      </c>
+      <c r="E228" t="inlineStr"/>
       <c r="F228" t="inlineStr">
         <is>
-          <t>Omvårdnad</t>
+          <t>Socialt arbete</t>
         </is>
       </c>
       <c r="G228" t="inlineStr">
         <is>
-          <t>Personcentrerad vård inom olika vårdsammanhang</t>
+          <t>Försörjning, rehabilitering och aktivering i socialt arbete</t>
         </is>
       </c>
       <c r="H228" t="inlineStr">
@@ -10522,19 +10522,19 @@
       </c>
       <c r="I228" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GVÅ35Q</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA3DN</t>
         </is>
       </c>
     </row>
     <row r="229">
       <c r="A229" s="2" t="inlineStr">
         <is>
-          <t>GIH3F4</t>
+          <t>GSA3DS</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>IDA</t>
+          <t>SAA</t>
         </is>
       </c>
       <c r="C229" t="inlineStr">
@@ -10544,18 +10544,18 @@
       </c>
       <c r="D229" t="inlineStr">
         <is>
-          <t>2025-02-24</t>
+          <t>2024-12-10</t>
         </is>
       </c>
       <c r="E229" t="inlineStr"/>
       <c r="F229" t="inlineStr">
         <is>
-          <t>Idrotts- och hälsovetenskap</t>
+          <t>Socialt arbete</t>
         </is>
       </c>
       <c r="G229" t="inlineStr">
         <is>
-          <t>Idrottspsykologi med praktisk tillämpning</t>
+          <t>Organisation, grupp och samverkan</t>
         </is>
       </c>
       <c r="H229" t="inlineStr">
@@ -10565,19 +10565,19 @@
       </c>
       <c r="I229" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3F4</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSA3DS</t>
         </is>
       </c>
     </row>
     <row r="230">
       <c r="A230" s="2" t="inlineStr">
         <is>
-          <t>GIH3F5</t>
+          <t>GVÅ35Q</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>IDA</t>
+          <t>OMV</t>
         </is>
       </c>
       <c r="C230" t="inlineStr">
@@ -10587,18 +10587,22 @@
       </c>
       <c r="D230" t="inlineStr">
         <is>
-          <t>2025-02-24</t>
-        </is>
-      </c>
-      <c r="E230" t="inlineStr"/>
+          <t>2023-08-30</t>
+        </is>
+      </c>
+      <c r="E230" t="inlineStr">
+        <is>
+          <t>2025-01-13</t>
+        </is>
+      </c>
       <c r="F230" t="inlineStr">
         <is>
-          <t>Idrotts- och hälsovetenskap</t>
+          <t>Omvårdnad</t>
         </is>
       </c>
       <c r="G230" t="inlineStr">
         <is>
-          <t>Idrottens organisation i samhället</t>
+          <t>Personcentrerad vård inom olika vårdsammanhang</t>
         </is>
       </c>
       <c r="H230" t="inlineStr">
@@ -10608,14 +10612,14 @@
       </c>
       <c r="I230" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3F5</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GVÅ35Q</t>
         </is>
       </c>
     </row>
     <row r="231">
       <c r="A231" s="2" t="inlineStr">
         <is>
-          <t>GIH3F8</t>
+          <t>GIH3F4</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
@@ -10641,7 +10645,7 @@
       </c>
       <c r="G231" t="inlineStr">
         <is>
-          <t>Idrottens funktionella anatomi och biomekanik</t>
+          <t>Idrottspsykologi med praktisk tillämpning</t>
         </is>
       </c>
       <c r="H231" t="inlineStr">
@@ -10651,14 +10655,14 @@
       </c>
       <c r="I231" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3F8</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3F4</t>
         </is>
       </c>
     </row>
     <row r="232">
       <c r="A232" s="2" t="inlineStr">
         <is>
-          <t>GIH3G5</t>
+          <t>GIH3F5</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
@@ -10673,7 +10677,7 @@
       </c>
       <c r="D232" t="inlineStr">
         <is>
-          <t>2025-06-09</t>
+          <t>2025-02-24</t>
         </is>
       </c>
       <c r="E232" t="inlineStr"/>
@@ -10684,7 +10688,7 @@
       </c>
       <c r="G232" t="inlineStr">
         <is>
-          <t>Idrottsvetenskaplig metod</t>
+          <t>Idrottens organisation i samhället</t>
         </is>
       </c>
       <c r="H232" t="inlineStr">
@@ -10694,14 +10698,14 @@
       </c>
       <c r="I232" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3G5</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3F5</t>
         </is>
       </c>
     </row>
     <row r="233">
       <c r="A233" s="2" t="inlineStr">
         <is>
-          <t>GIH3G6</t>
+          <t>GIH3F8</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
@@ -10716,7 +10720,7 @@
       </c>
       <c r="D233" t="inlineStr">
         <is>
-          <t>2025-06-09</t>
+          <t>2025-02-24</t>
         </is>
       </c>
       <c r="E233" t="inlineStr"/>
@@ -10727,7 +10731,7 @@
       </c>
       <c r="G233" t="inlineStr">
         <is>
-          <t>Idrottsvetenskaplig fördjupning</t>
+          <t>Idrottens funktionella anatomi och biomekanik</t>
         </is>
       </c>
       <c r="H233" t="inlineStr">
@@ -10737,14 +10741,14 @@
       </c>
       <c r="I233" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3G6</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3F8</t>
         </is>
       </c>
     </row>
     <row r="234">
       <c r="A234" s="2" t="inlineStr">
         <is>
-          <t>GIH3G8</t>
+          <t>GIH3G5</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
@@ -10770,7 +10774,7 @@
       </c>
       <c r="G234" t="inlineStr">
         <is>
-          <t>Coachning och träningsprocesser i praktiken</t>
+          <t>Idrottsvetenskaplig metod</t>
         </is>
       </c>
       <c r="H234" t="inlineStr">
@@ -10780,14 +10784,14 @@
       </c>
       <c r="I234" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3G8</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3G5</t>
         </is>
       </c>
     </row>
     <row r="235">
       <c r="A235" s="2" t="inlineStr">
         <is>
-          <t>GIH3G9</t>
+          <t>GIH3G6</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
@@ -10813,7 +10817,7 @@
       </c>
       <c r="G235" t="inlineStr">
         <is>
-          <t>Entreprenörskap inom idrott och hälsa</t>
+          <t>Idrottsvetenskaplig fördjupning</t>
         </is>
       </c>
       <c r="H235" t="inlineStr">
@@ -10823,14 +10827,14 @@
       </c>
       <c r="I235" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3G9</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3G6</t>
         </is>
       </c>
     </row>
     <row r="236">
       <c r="A236" s="2" t="inlineStr">
         <is>
-          <t>GIH3GA</t>
+          <t>GIH3G8</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
@@ -10856,7 +10860,7 @@
       </c>
       <c r="G236" t="inlineStr">
         <is>
-          <t>Examensarbete för kandidatexamen i idrotts- och hälsovetenskap</t>
+          <t>Coachning och träningsprocesser i praktiken</t>
         </is>
       </c>
       <c r="H236" t="inlineStr">
@@ -10866,14 +10870,14 @@
       </c>
       <c r="I236" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3GA</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3G8</t>
         </is>
       </c>
     </row>
     <row r="237">
       <c r="A237" s="2" t="inlineStr">
         <is>
-          <t>GIH3GC</t>
+          <t>GIH3G9</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
@@ -10899,7 +10903,7 @@
       </c>
       <c r="G237" t="inlineStr">
         <is>
-          <t>Idrottsnutrition</t>
+          <t>Entreprenörskap inom idrott och hälsa</t>
         </is>
       </c>
       <c r="H237" t="inlineStr">
@@ -10909,19 +10913,19 @@
       </c>
       <c r="I237" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3GC</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3G9</t>
         </is>
       </c>
     </row>
     <row r="238">
       <c r="A238" s="2" t="inlineStr">
         <is>
-          <t>GNV3GV</t>
+          <t>GIH3GA</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>NAV</t>
+          <t>IDA</t>
         </is>
       </c>
       <c r="C238" t="inlineStr">
@@ -10931,18 +10935,18 @@
       </c>
       <c r="D238" t="inlineStr">
         <is>
-          <t>2025-09-10</t>
+          <t>2025-06-09</t>
         </is>
       </c>
       <c r="E238" t="inlineStr"/>
       <c r="F238" t="inlineStr">
         <is>
-          <t>Naturvetenskap</t>
+          <t>Idrotts- och hälsovetenskap</t>
         </is>
       </c>
       <c r="G238" t="inlineStr">
         <is>
-          <t>Naturorienterande ämnen och teknik för lärare i årskurs 1-3. Ingår i lärarlyftet.</t>
+          <t>Examensarbete för kandidatexamen i idrotts- och hälsovetenskap</t>
         </is>
       </c>
       <c r="H238" t="inlineStr">
@@ -10952,19 +10956,19 @@
       </c>
       <c r="I238" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GNV3GV</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3GA</t>
         </is>
       </c>
     </row>
     <row r="239">
       <c r="A239" s="2" t="inlineStr">
         <is>
-          <t>AFT2C8</t>
+          <t>GIH3GC</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>FYS</t>
+          <t>IDA</t>
         </is>
       </c>
       <c r="C239" t="inlineStr">
@@ -10974,18 +10978,18 @@
       </c>
       <c r="D239" t="inlineStr">
         <is>
-          <t>2025-12-04</t>
+          <t>2025-06-09</t>
         </is>
       </c>
       <c r="E239" t="inlineStr"/>
       <c r="F239" t="inlineStr">
         <is>
-          <t>Fysioterapi</t>
+          <t>Idrotts- och hälsovetenskap</t>
         </is>
       </c>
       <c r="G239" t="inlineStr">
         <is>
-          <t>Forskningsmetodik och projektplan inför examensarbete för magisterexamen i fysioterapi</t>
+          <t>Idrottsnutrition</t>
         </is>
       </c>
       <c r="H239" t="inlineStr">
@@ -10995,19 +10999,19 @@
       </c>
       <c r="I239" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AFT2C8</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3GC</t>
         </is>
       </c>
     </row>
     <row r="240">
       <c r="A240" s="2" t="inlineStr">
         <is>
-          <t>GIH3JL</t>
+          <t>GNV3GV</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>IDA</t>
+          <t>NAV</t>
         </is>
       </c>
       <c r="C240" t="inlineStr">
@@ -11017,33 +11021,119 @@
       </c>
       <c r="D240" t="inlineStr">
         <is>
-          <t>2026-03-03</t>
+          <t>2025-09-10</t>
         </is>
       </c>
       <c r="E240" t="inlineStr"/>
       <c r="F240" t="inlineStr">
         <is>
+          <t>Naturvetenskap</t>
+        </is>
+      </c>
+      <c r="G240" t="inlineStr">
+        <is>
+          <t>Naturorienterande ämnen och teknik för lärare i årskurs 1-3. Ingår i lärarlyftet.</t>
+        </is>
+      </c>
+      <c r="H240" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I240" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GNV3GV</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" s="2" t="inlineStr">
+        <is>
+          <t>AFT2C8</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>FYS</t>
+        </is>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>IHV</t>
+        </is>
+      </c>
+      <c r="D241" t="inlineStr">
+        <is>
+          <t>2025-12-04</t>
+        </is>
+      </c>
+      <c r="E241" t="inlineStr"/>
+      <c r="F241" t="inlineStr">
+        <is>
+          <t>Fysioterapi</t>
+        </is>
+      </c>
+      <c r="G241" t="inlineStr">
+        <is>
+          <t>Forskningsmetodik och projektplan inför examensarbete för magisterexamen i fysioterapi</t>
+        </is>
+      </c>
+      <c r="H241" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I241" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AFT2C8</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" s="2" t="inlineStr">
+        <is>
+          <t>GIH3JL</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>IDA</t>
+        </is>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>IHV</t>
+        </is>
+      </c>
+      <c r="D242" t="inlineStr">
+        <is>
+          <t>2026-03-03</t>
+        </is>
+      </c>
+      <c r="E242" t="inlineStr"/>
+      <c r="F242" t="inlineStr">
+        <is>
           <t>Idrotts- och hälsovetenskap</t>
         </is>
       </c>
-      <c r="G240" t="inlineStr">
+      <c r="G242" t="inlineStr">
         <is>
           <t>Tillämpad idrottsfysiologi</t>
         </is>
       </c>
-      <c r="H240" t="inlineStr">
-        <is>
-          <t>Ingen aktiv kursomgång</t>
-        </is>
-      </c>
-      <c r="I240" s="2" t="inlineStr">
+      <c r="H242" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I242" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIH3JL</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I240"/>
+  <autoFilter ref="A1:I242"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I2" r:id="rId2"/>
@@ -11523,6 +11613,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I239" r:id="rId476"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A240" r:id="rId477"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I240" r:id="rId478"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A241" r:id="rId479"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I241" r:id="rId480"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A242" r:id="rId481"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I242" r:id="rId482"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>